<commit_message>
Make manual/ first-class source data; retire sheet-import machinery
The one-time importers (import_sheet_export.py, bootstrap_manual_from_
sheet.py) and the sheet-export inputs now live only in git history.
manual/ CSVs are the source of truth for human-collected facts, each
row credited (collaborator-sheet | manual-repo-edit); manual/README.md
documents the contract. The 4 in-transition LA AINs' fallback values
moved into manual/parcel_values_manual.csv, removing build_dataset's
dependency on the sheet export. Extraction and basic-list scripts no
longer compare against the sheet (superseded by merge-time QA).

Also: QA findings become a fourth tab in review.xlsx so the
collaborator can review discrepancies in the sheet; README/CLAUDE.md
rewritten for the current pipeline.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grants" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parcels" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA findings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -60325,6 +60326,3442 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C201"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>project_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>duplicate-sheet-rows</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>76/182</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>multiple sheet projects map to one authorization (1451 w mlk blvd)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>301</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2025 New Jersey Apartments (CMFA, 2023-07-14) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>302</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Bernardine Apartments (CMFA, 2023-07-14) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>303</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>10705 Avalon Blvd Apartments (CMFA, 2024-02-02) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>304</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>820 MacArthur Apartments (CMFA, 2024-02-02) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>305</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>4252 Crenshaw Apartments (CMFA, 2024-04-26) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>306</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Montessa Apartments (CMFA, 2024-04-26) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>307</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2330 3rd Street Apartments (CMFA, 2024-08-09) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>308</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Hillsdale Gardens Apartments (CMFA, 2024-08-30) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>309</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>6171 Mission Gorge Apartments (CMFA, 2024-09-20) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Horizon Apartments (CMFA, 2024-09-20) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>313</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Bella Vista Apartments (CMFA, 2025-01-10) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>316</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Electric Lofts Apartments (CMFA, 2025-01-31) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>323</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Meridian Apartments (CMFA, 2025-02-21) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>330</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>569 W 6th Apartments (CMFA, 2025-04-25) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>331</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>685 W 4th Apartments (CMFA, 2025-04-25) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>334</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Bella Vista at Hilltop Apartments (CMFA, 2025-05-30) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>335</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Chadwick Apartments (CMFA, 2025-05-30) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>337</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Bella Vista at Hilltop Apartments (CMFA, 2025-06-06) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>338</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Chadwick Apartments (CMFA, 2025-06-06) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>341</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Meridian Apartments (CMFA, 2025-07-18) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>345</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Meridian Apartments (CMFA, 2025-08-08) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>346</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Citrine Apartments (CMFA, 2025-08-29) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>348</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>4228 Western Apartments (CMFA, 2025-10-24) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>349</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>4228 Western Ave Apartments (CMFA, 2025-11-07) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>351</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>12th Street Apartments (CMFA, 2026-01-09) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>358</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Del Norte Apartments (CMFA, 2026-04-17) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>359</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Terrace View Apartments (CMFA, 2026-06-12) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>360</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>The Heltsley Apartments FKA SoFi Redwood Park Apartments (CMFA, 2026-06-12) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>363</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Terrace View Apartments (CMFA, 2026-06-26) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>364</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>The Heltsley Apartments FKA SoFi Redwood Park Apartments (CMFA, 2026-06-26) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>new-grant</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>369</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Verdana Apartments (CSCDA, 2026-08-20) not in collaborator sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>investor_1: generated 'Oak Road' -&gt; manual 'Eleos Ventures, LLC'</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>entity: generated '2019 Ozone Affordable Housing – 820 MacArthur, LP' -&gt; manual '2019 Ozone Affordable Housing'</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>entity: generated 'OODB2, LP, a Washington Limited Partnership' -&gt; manual 'OODB2, LP'</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>entity: generated 'Affordable Housing Alliance II, Inc., d/b/a Integrity Housing, a Colorado nonprofit corporation' -&gt; manual 'Affordable Housing Alliance II, Inc. dba Integrity Housing'</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>investor_1: generated 'AOF / Pacific Affordable Housing Corp.' -&gt; manual 'AOF'</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>nonprofit_partner: generated 'AOF / Pacific Affordable Housing Corp.' -&gt; manual 'Pacific Affordable Housing Corp'</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>city: generated 'Los Angeles' -&gt; manual 'El Sobrante'</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>county: generated 'Los Angeles' -&gt; manual 'Contra Costa'</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>total_units: generated '24' -&gt; manual '52'</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>total_units: generated '22' -&gt; manual '72'</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>total_units: generated '24' -&gt; manual '48'</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>total_units: generated '65' -&gt; manual '165'</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>property_name: generated '2330 3rd Street Apartments' -&gt; manual '2330 E. 3rd Street Apartments'</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>investor_1: generated 'Ethos Real Estate' -&gt; manual 'Vistria Group'</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>nonprofit_partner: generated 'Step Forward Communities' -&gt; manual 'Step Forward Comminities'</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>total_units: generated '144' -&gt; manual '145'</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>total_units: generated '42' -&gt; manual '356'</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>investor_1: generated 'BRIDGE Housing Corporation' -&gt; manual 'Bridge Housing'</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>nonprofit_partner: generated 'BRIDGE Housing Corporation' -&gt; manual 'Bridge Housing'</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>entity: generated 'PREG 5150 ECR Los Altos, LP, a California limited partnership' -&gt; manual 'Prometheus Real Estate Group'</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>total_units: generated '29' -&gt; manual '196'</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>entity: generated '3 SIOF 1451 W MLK BLVD, LP' -&gt; manual '1451 W. MLK Boulevard Apartments'</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>investor_1: generated 'Vintage Housing Holdings, LLC / Kennedy Wilson' -&gt; manual 'Kennedy Wilson'</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>nonprofit_partner: generated 'Pacific Housing, Inc.' -&gt; manual 'Hearthstone Housing Foundation'</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>total_units: generated '8' -&gt; manual '1008'</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>total_units: generated '32' -&gt; manual '31'</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>city_cut: generated '4650.0' -&gt; manual '4500'</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>entity: generated '2 SIOF 10811 S Compton Ave, LP' -&gt; manual '10811 S. Compton Ave Apartments'</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>entity: generated 'SIOF 5 Properties, LP, a California limited partnership' -&gt; manual 'SIOF 5 Properties, LP, California limited partnership'</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>entity: generated '2 SIOF 685 W Fourth St, LP, a Delaware limited partnership' -&gt; manual '2 SIOF 685 W Fourth St, LP, Delaware limited partnership'</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>investor_1: generated 'Vintage Housing Holdings, LLC / Kennedy Wilson' -&gt; manual 'Vintage Housing Holdings'</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>158</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>total_units: generated '30' -&gt; manual '29'</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>investor_1: generated 'Belveron Partners' -&gt; manual 'Sack Capital Partners'</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>nonprofit_partner: generated 'Las Palmas Housing &amp; Development Corporation' -&gt; manual 'Las Palmas Housing &amp; Development Corp.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>investor_1: generated 'BRIDGE Housing Corporation' -&gt; manual 'BRIDGE Housing Corp.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>total_units: generated '24' -&gt; manual '42'</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>city: generated 'Sacramento' -&gt; manual 'Unincorporated'</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>property_name: generated 'Kinglsey Apartments' -&gt; manual 'Kingsley Apartments'</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>134</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>total_units: generated '69' -&gt; manual '68'</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>address: generated '5805 Charlotte Drive, San Jose, CA' -&gt; manual '5805 Charlotte Drive, San Jose, CA 95123'</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>total_units: generated '42' -&gt; manual '41'</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>143</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>property_name: generated 'Coliseum Connections Transit Village Apartments' -&gt; manual 'Coliseum Transit Village'</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>138</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>city: generated 'Santa Clara' -&gt; manual 'San Jose'</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>147</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>property_name: generated 'Coliseum Connections Transit Village Apartments' -&gt; manual 'Coliseum Connections'</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>property_name: generated 'The Langham Apartments' -&gt; manual 'Langham Apartments'</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>151</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>property_name: generated 'The Piccadilly Apartments' -&gt; manual 'Piccadilly Apartments'</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>152</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>total_units: generated '52' -&gt; manual '152'</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>155</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>156</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>171</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>city_cut: generated '15900.0' -&gt; manual '6300'</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>181</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>city: generated 'Long Beach' -&gt; manual 'Los Angeles'</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>181</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>total_units: generated '52' -&gt; manual '152'</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>entity: generated 'St. Anton Highlands LP' -&gt; manual 'St. Anton Highland, LP'</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>144</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>property_name: generated 'La Vista Apartments' -&gt; manual 'La Vista Apartment Homes'</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>total_units: generated '42' -&gt; manual '41'</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>196</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>address: generated '9750 Airport Blvd, Los Angeles, CA' -&gt; manual '9750 Airport Blvd, Westchester, CA 90045'</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>199</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>city_cut: generated '5550.0' -&gt; manual '5500'</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>207</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>address: generated '2625 Cullen Street, Los Angeles, CA' -&gt; manual '2625 Cullen St, Los Angeles, CA 90034'</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>208</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>address: generated '2481 South Sawtelle Blvd, Los Angeles, CA' -&gt; manual '2481 Sawtelle Blvd, Los Angeles, CA 90064'</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>property_name: generated 'Summerwood Apartment Homes' -&gt; manual 'Summerwood Apartments Homes Apartments'</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>entity: generated 'Standard Summerwood II LP' -&gt; manual 'Standard Properties'</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>investor_1: generated 'Standard Property Company, Inc.' -&gt; manual 'Standard Properties'</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>total_units: generated '50' -&gt; manual '49'</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>county: generated 'San Diego' -&gt; manual 'Los Angeles'</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>224</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>address: generated '1454 West Florence Avenue, Los Angeles, CA' -&gt; manual '1454 W Florence Ave, Los Angeles, CA 90047'</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>investor_1: generated 'Zenith Property Group LLC' -&gt; manual 'Red Stone Equity Partners'</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>term_years: generated '35' -&gt; manual '15'</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>term_years: generated '55' -&gt; manual '10'</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>address: generated '142 Fig Tree Lane, Martinez, CA' -&gt; manual '142 Fig Tree Lane, Martinez, CA 94553'</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>term_years: generated '15' -&gt; manual '10'</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>228</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>nonprofit_partner: generated 'The Foundation for Affordable Housing' -&gt; manual 'Foundation for Affordable Housing'</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>228</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>term_years: generated '10' -&gt; manual '15'</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>property_name: generated 'Hansen Village Apartments' -&gt; manual 'Hansen illage Apartments'</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>nonprofit_partner: generated 'The Foundation for Affordable Housing' -&gt; manual 'Foundation for Affordable Housing'</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>address: generated '11821 Foothill Blvd, Los Angeles, CA' -&gt; manual '11821 Foothill Blvd, Lake View Terrace, CA 91342'</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>232</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>address: generated '12091 Bayport Street, Garden Grove, CA' -&gt; manual '12091 Bayport St, Garden Grove, CA 92840'</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>222</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>address: generated '16077 Ashland Avenue, San Lorenzo' -&gt; manual '16077 Ashland Ave, San Lorenzo, CA 94580'</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>217</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>total_units: generated '35' -&gt; manual '34'</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>address: generated '511 N. Hoover Street, Los Angeles' -&gt; manual '511 N. Hoover Street, Los Angeles, California'</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>211</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>entity: generated 'Haven, LP' -&gt; manual 'Heven LP'</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>211</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>address: generated '6530 Independence Avenue, Los Angeles' -&gt; manual '6530 Independence Ave, Canoga Park, CA 91303'</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>address: generated '2075 West Jefferson Blvd., Los Angeles' -&gt; manual '2075 W Jefferson BlvdLos Angeles, CA 90018'</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>213</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>address: generated '5416 Jackson Street, North Highlands' -&gt; manual '5416 Jackson St, North Highlands, CA 95660'</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>214</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>address: generated '444 North Amelia Avenue, San Dimas' -&gt; manual '444 N Amelia Ave, San Dimas, CA 91773'</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>address: generated '220 47th Street, San Diego' -&gt; manual '220 47th St, San Diego, CA 92102'</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>231</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>nonprofit_partner: generated 'Bedford' -&gt; manual 'Bedford Affordable Housing Foundation'</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>231</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>address: generated '160 S. Virgil Avenue, Los Angeles' -&gt; manual '160 S Virgil Ave, Los Angeles, CA 90004'</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>address: generated '926 S. Kingsley Drive, Los Angeles, CA' -&gt; manual '926 S Kingsley Dr, Los Angeles, CA 90006'</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>term_years: generated '55' -&gt; manual '10'</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>234</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>address: generated '939 S. Kingsley Drive, Los Angeles, CA' -&gt; manual '939 S Kingsley Dr, Los Angeles, CA 90006'</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>235</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>address: generated '3950 W. Ingraham Street, Los Angeles, CA' -&gt; manual '3950 Ingraham St, San Diego, CA 92109'</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>236</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>total_units: generated '136' -&gt; manual '108'</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>236</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>address: generated '6985 S. Centinela Avenue, Los Angeles, CA' -&gt; manual '6985 S. Centinela Avenue, Los Angeles, CA 90045'</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>237</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>address: generated '1178 N. Edgemont Street, Los Angeles, CA' -&gt; manual '1178 N Edgemont St, Los Angeles, CA 90029'</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>225</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>entity: generated 'CG Bennington, LP and JSP Bennington, LP' -&gt; manual 'CG Bennington, LP / JSP Bennington, LP'</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>override-conflict</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>225</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>term_years: generated '30' -&gt; manual '55'</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>la-fetch-fallback</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>AIN 6020022027 has no current roll data; using manual value</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>AIN 6020022027 (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>la-fetch-fallback</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>AIN 5036031006 has no current roll data; using manual value</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>la-fetch-fallback</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>AIN 4262018026 has no current roll data; using manual value</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>la-fetch-fallback</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>132</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>AIN 6020022027 has no current roll data; using manual value</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>la-fetch-fallback</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>AIN 2125017014 has no current roll data; using manual value</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>143</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>AIN 41416654 (Alameda): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>147</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>AIN 41416654 (Alameda): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>158</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>AIN 5036031006 (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>194</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>196</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>199</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>201</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>AIN (none) (Santa Barbara): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>203</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>AIN (none) (Sacramento): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>205</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>AIN (none) (Contra Costa): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>207</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>208</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>AIN (none) (San Diego): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>211</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>213</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>AIN (none) (Sacramento): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>214</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>216</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>AIN (none) (San Diego): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>217</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>218</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>219</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>221</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>222</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>AIN (none) (Alameda): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>223</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>AIN (none) (Alameda): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>224</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>AIN (none) (Contra Costa): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>228</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>AIN (none) (San Diego): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>231</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>234</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>235</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>236</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>237</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>AIN 46745075 (Santa Clara): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>AIN 46745074 (Santa Clara): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>AIN 46745073 (Santa Clara): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>198</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>AIN (none) (Santa Clara): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>202</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>AIN (none) (Santa Cruz): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>AIN 128101150 (Solano): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>AIN 128101050 (Solano): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>AIN 128105060 (Solano): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>parcel-no-values</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>225</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>AIN (none) (Solano): no roll values from any source</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>missing-parcels</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>238</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Heritage Park Apartments Livermore: authorized, not dead, no parcel rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>shared-ain</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>143/147</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>AIN 41416654 assigned to multiple projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>shared-ain</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>182/76</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>AIN 5036031006 assigned to multiple projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>shared-ain</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>130/179</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>AIN 5080006008 assigned to multiple projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>shared-ain</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>126/173</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>AIN 5094005005 assigned to multiple projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>shared-ain</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>127/174</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>AIN 5094006003 assigned to multiple projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>shared-ain</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>122/165</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>AIN 5094017020 assigned to multiple projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>shared-ain</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>124/169</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>AIN 5094023025 assigned to multiple projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>shared-ain</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>128/175</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>AIN 5502019004 assigned to multiple projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>shared-ain</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>125/170</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>AIN 5503024012 assigned to multiple projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>shared-ain</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>129/177</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>AIN 5517005016 assigned to multiple projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>shared-ain</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>121/162</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>AIN 5518013024 assigned to multiple projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>shared-ain</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>123/168</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>AIN 5518020021 assigned to multiple projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>shared-ain</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>10/132</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>AIN 6020022027 assigned to multiple projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>shared-ain</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>152/181</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>AIN 7157012017 assigned to multiple projects</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Automate Solano County roll values via the assessor's PublicAccessNow portal
Two public JSON endpoints (QuickSearch resolves parcel id -> Altkey;
the Value History DataDisplay module returns per-tax-year assessment
rows). 60 of 63 assigned Solano parcels now carry current 2026 roll
values (source solano-county-portal); 3 parcels have no value history
in the portal. Assigned Bennington Apartments (#225) its parcel
(0168150010, the single Real Property record at its situs) as a
manual-repo-edit. build_dataset now merges any output/pipeline/
*_roll_values.csv, so further counties drop in as fetchers.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -34477,7 +34477,7 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="25" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
@@ -58019,14 +58019,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N329" t="inlineStr">
-        <is>
-          <t>7595</t>
-        </is>
-      </c>
-      <c r="R329" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K329" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L329" s="2" t="inlineStr">
+        <is>
+          <t>8875.0</t>
+        </is>
+      </c>
+      <c r="M329" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N329" s="2" t="inlineStr">
+        <is>
+          <t>8875.0</t>
+        </is>
+      </c>
+      <c r="O329" s="2" t="inlineStr">
+        <is>
+          <t>1569.0</t>
+        </is>
+      </c>
+      <c r="R329" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S329" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58066,14 +58091,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N330" t="inlineStr">
-        <is>
-          <t>7606</t>
-        </is>
-      </c>
-      <c r="R330" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K330" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L330" s="2" t="inlineStr">
+        <is>
+          <t>8888.0</t>
+        </is>
+      </c>
+      <c r="M330" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N330" s="2" t="inlineStr">
+        <is>
+          <t>8888.0</t>
+        </is>
+      </c>
+      <c r="O330" s="2" t="inlineStr">
+        <is>
+          <t>1535.0</t>
+        </is>
+      </c>
+      <c r="R330" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S330" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58113,14 +58163,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N331" t="inlineStr">
-        <is>
-          <t>7619</t>
-        </is>
-      </c>
-      <c r="R331" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K331" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L331" s="2" t="inlineStr">
+        <is>
+          <t>8903.0</t>
+        </is>
+      </c>
+      <c r="M331" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N331" s="2" t="inlineStr">
+        <is>
+          <t>8903.0</t>
+        </is>
+      </c>
+      <c r="O331" s="2" t="inlineStr">
+        <is>
+          <t>1514.0</t>
+        </is>
+      </c>
+      <c r="R331" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S331" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58160,14 +58235,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N332" t="inlineStr">
-        <is>
-          <t>7631</t>
-        </is>
-      </c>
-      <c r="R332" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K332" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L332" s="2" t="inlineStr">
+        <is>
+          <t>8918.0</t>
+        </is>
+      </c>
+      <c r="M332" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N332" s="2" t="inlineStr">
+        <is>
+          <t>8918.0</t>
+        </is>
+      </c>
+      <c r="O332" s="2" t="inlineStr">
+        <is>
+          <t>1541.0</t>
+        </is>
+      </c>
+      <c r="R332" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S332" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58207,14 +58307,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N333" t="inlineStr">
-        <is>
-          <t>30262</t>
-        </is>
-      </c>
-      <c r="R333" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K333" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L333" s="2" t="inlineStr">
+        <is>
+          <t>30867.0</t>
+        </is>
+      </c>
+      <c r="M333" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N333" s="2" t="inlineStr">
+        <is>
+          <t>30867.0</t>
+        </is>
+      </c>
+      <c r="O333" s="2" t="inlineStr">
+        <is>
+          <t>5457.0</t>
+        </is>
+      </c>
+      <c r="R333" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S333" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58254,14 +58379,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N334" t="inlineStr">
-        <is>
-          <t>30426</t>
-        </is>
-      </c>
-      <c r="R334" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K334" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L334" s="2" t="inlineStr">
+        <is>
+          <t>31033.0</t>
+        </is>
+      </c>
+      <c r="M334" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N334" s="2" t="inlineStr">
+        <is>
+          <t>31033.0</t>
+        </is>
+      </c>
+      <c r="O334" s="2" t="inlineStr">
+        <is>
+          <t>5362.0</t>
+        </is>
+      </c>
+      <c r="R334" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S334" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58301,14 +58451,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N335" t="inlineStr">
-        <is>
-          <t>31967</t>
-        </is>
-      </c>
-      <c r="R335" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K335" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L335" s="2" t="inlineStr">
+        <is>
+          <t>32605.0</t>
+        </is>
+      </c>
+      <c r="M335" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N335" s="2" t="inlineStr">
+        <is>
+          <t>32605.0</t>
+        </is>
+      </c>
+      <c r="O335" s="2" t="inlineStr">
+        <is>
+          <t>5546.0</t>
+        </is>
+      </c>
+      <c r="R335" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S335" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58348,14 +58523,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N336" t="inlineStr">
-        <is>
-          <t>35714</t>
-        </is>
-      </c>
-      <c r="R336" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K336" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L336" s="2" t="inlineStr">
+        <is>
+          <t>36427.0</t>
+        </is>
+      </c>
+      <c r="M336" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N336" s="2" t="inlineStr">
+        <is>
+          <t>36427.0</t>
+        </is>
+      </c>
+      <c r="O336" s="2" t="inlineStr">
+        <is>
+          <t>6294.0</t>
+        </is>
+      </c>
+      <c r="R336" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S336" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58395,14 +58595,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N337" t="inlineStr">
-        <is>
-          <t>40196</t>
-        </is>
-      </c>
-      <c r="R337" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K337" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L337" s="2" t="inlineStr">
+        <is>
+          <t>40997.0</t>
+        </is>
+      </c>
+      <c r="M337" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N337" s="2" t="inlineStr">
+        <is>
+          <t>40997.0</t>
+        </is>
+      </c>
+      <c r="O337" s="2" t="inlineStr">
+        <is>
+          <t>7248.0</t>
+        </is>
+      </c>
+      <c r="R337" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S337" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58479,14 +58704,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N339" t="inlineStr">
-        <is>
-          <t>66586</t>
-        </is>
-      </c>
-      <c r="R339" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K339" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L339" s="2" t="inlineStr">
+        <is>
+          <t>67916.0</t>
+        </is>
+      </c>
+      <c r="M339" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N339" s="2" t="inlineStr">
+        <is>
+          <t>67916.0</t>
+        </is>
+      </c>
+      <c r="O339" s="2" t="inlineStr">
+        <is>
+          <t>11735.0</t>
+        </is>
+      </c>
+      <c r="R339" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S339" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58526,14 +58776,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N340" t="inlineStr">
-        <is>
-          <t>61921</t>
-        </is>
-      </c>
-      <c r="R340" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K340" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L340" s="2" t="inlineStr">
+        <is>
+          <t>63157.0</t>
+        </is>
+      </c>
+      <c r="M340" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N340" s="2" t="inlineStr">
+        <is>
+          <t>63157.0</t>
+        </is>
+      </c>
+      <c r="O340" s="2" t="inlineStr">
+        <is>
+          <t>10743.0</t>
+        </is>
+      </c>
+      <c r="R340" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S340" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58573,14 +58848,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N341" t="inlineStr">
-        <is>
-          <t>49211</t>
-        </is>
-      </c>
-      <c r="R341" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K341" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L341" s="2" t="inlineStr">
+        <is>
+          <t>50192.0</t>
+        </is>
+      </c>
+      <c r="M341" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N341" s="2" t="inlineStr">
+        <is>
+          <t>50192.0</t>
+        </is>
+      </c>
+      <c r="O341" s="2" t="inlineStr">
+        <is>
+          <t>8873.0</t>
+        </is>
+      </c>
+      <c r="R341" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S341" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58620,14 +58920,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N342" t="inlineStr">
-        <is>
-          <t>99051</t>
-        </is>
-      </c>
-      <c r="R342" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K342" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L342" s="2" t="inlineStr">
+        <is>
+          <t>101032.0</t>
+        </is>
+      </c>
+      <c r="M342" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N342" s="2" t="inlineStr">
+        <is>
+          <t>101032.0</t>
+        </is>
+      </c>
+      <c r="O342" s="2" t="inlineStr">
+        <is>
+          <t>17458.0</t>
+        </is>
+      </c>
+      <c r="R342" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S342" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58667,14 +58992,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N343" t="inlineStr">
-        <is>
-          <t>1360</t>
-        </is>
-      </c>
-      <c r="R343" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K343" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L343" s="2" t="inlineStr">
+        <is>
+          <t>51705.0</t>
+        </is>
+      </c>
+      <c r="M343" s="2" t="inlineStr">
+        <is>
+          <t>561000.0</t>
+        </is>
+      </c>
+      <c r="N343" s="2" t="inlineStr">
+        <is>
+          <t>612705.0</t>
+        </is>
+      </c>
+      <c r="O343" s="2" t="inlineStr">
+        <is>
+          <t>108006.0</t>
+        </is>
+      </c>
+      <c r="R343" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S343" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58714,14 +59064,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N344" t="inlineStr">
-        <is>
-          <t>1201</t>
-        </is>
-      </c>
-      <c r="R344" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K344" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L344" s="2" t="inlineStr">
+        <is>
+          <t>50439.0</t>
+        </is>
+      </c>
+      <c r="M344" s="2" t="inlineStr">
+        <is>
+          <t>571000.0</t>
+        </is>
+      </c>
+      <c r="N344" s="2" t="inlineStr">
+        <is>
+          <t>621439.0</t>
+        </is>
+      </c>
+      <c r="O344" s="2" t="inlineStr">
+        <is>
+          <t>115237.0</t>
+        </is>
+      </c>
+      <c r="R344" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S344" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58761,14 +59136,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N345" t="inlineStr">
-        <is>
-          <t>1201</t>
-        </is>
-      </c>
-      <c r="R345" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K345" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L345" s="2" t="inlineStr">
+        <is>
+          <t>50439.0</t>
+        </is>
+      </c>
+      <c r="M345" s="2" t="inlineStr">
+        <is>
+          <t>561000.0</t>
+        </is>
+      </c>
+      <c r="N345" s="2" t="inlineStr">
+        <is>
+          <t>611439.0</t>
+        </is>
+      </c>
+      <c r="O345" s="2" t="inlineStr">
+        <is>
+          <t>107787.0</t>
+        </is>
+      </c>
+      <c r="R345" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S345" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58808,14 +59208,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N346" t="inlineStr">
-        <is>
-          <t>1202</t>
-        </is>
-      </c>
-      <c r="R346" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K346" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L346" s="2" t="inlineStr">
+        <is>
+          <t>50439.0</t>
+        </is>
+      </c>
+      <c r="M346" s="2" t="inlineStr">
+        <is>
+          <t>605000.0</t>
+        </is>
+      </c>
+      <c r="N346" s="2" t="inlineStr">
+        <is>
+          <t>655439.0</t>
+        </is>
+      </c>
+      <c r="O346" s="2" t="inlineStr">
+        <is>
+          <t>118205.0</t>
+        </is>
+      </c>
+      <c r="R346" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S346" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58855,14 +59280,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N347" t="inlineStr">
-        <is>
-          <t>1202</t>
-        </is>
-      </c>
-      <c r="R347" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K347" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L347" s="2" t="inlineStr">
+        <is>
+          <t>9639.0</t>
+        </is>
+      </c>
+      <c r="M347" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N347" s="2" t="inlineStr">
+        <is>
+          <t>9639.0</t>
+        </is>
+      </c>
+      <c r="O347" s="2" t="inlineStr">
+        <is>
+          <t>1665.0</t>
+        </is>
+      </c>
+      <c r="R347" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S347" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58902,14 +59352,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N348" t="inlineStr">
-        <is>
-          <t>1202</t>
-        </is>
-      </c>
-      <c r="R348" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K348" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L348" s="2" t="inlineStr">
+        <is>
+          <t>9639.0</t>
+        </is>
+      </c>
+      <c r="M348" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N348" s="2" t="inlineStr">
+        <is>
+          <t>9639.0</t>
+        </is>
+      </c>
+      <c r="O348" s="2" t="inlineStr">
+        <is>
+          <t>1704.0</t>
+        </is>
+      </c>
+      <c r="R348" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S348" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58949,14 +59424,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N349" t="inlineStr">
-        <is>
-          <t>32653</t>
-        </is>
-      </c>
-      <c r="R349" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K349" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L349" s="2" t="inlineStr">
+        <is>
+          <t>33305.0</t>
+        </is>
+      </c>
+      <c r="M349" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N349" s="2" t="inlineStr">
+        <is>
+          <t>33305.0</t>
+        </is>
+      </c>
+      <c r="O349" s="2" t="inlineStr">
+        <is>
+          <t>5755.0</t>
+        </is>
+      </c>
+      <c r="R349" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S349" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -58996,14 +59496,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N350" t="inlineStr">
-        <is>
-          <t>32653</t>
-        </is>
-      </c>
-      <c r="R350" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K350" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L350" s="2" t="inlineStr">
+        <is>
+          <t>33305.0</t>
+        </is>
+      </c>
+      <c r="M350" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N350" s="2" t="inlineStr">
+        <is>
+          <t>33305.0</t>
+        </is>
+      </c>
+      <c r="O350" s="2" t="inlineStr">
+        <is>
+          <t>5888.0</t>
+        </is>
+      </c>
+      <c r="R350" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S350" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59043,14 +59568,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N351" t="inlineStr">
-        <is>
-          <t>32697</t>
-        </is>
-      </c>
-      <c r="R351" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K351" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L351" s="2" t="inlineStr">
+        <is>
+          <t>33350.0</t>
+        </is>
+      </c>
+      <c r="M351" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N351" s="2" t="inlineStr">
+        <is>
+          <t>33350.0</t>
+        </is>
+      </c>
+      <c r="O351" s="2" t="inlineStr">
+        <is>
+          <t>5762.0</t>
+        </is>
+      </c>
+      <c r="R351" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S351" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59090,14 +59640,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N352" t="inlineStr">
-        <is>
-          <t>32612</t>
-        </is>
-      </c>
-      <c r="R352" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K352" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L352" s="2" t="inlineStr">
+        <is>
+          <t>33263.0</t>
+        </is>
+      </c>
+      <c r="M352" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N352" s="2" t="inlineStr">
+        <is>
+          <t>33263.0</t>
+        </is>
+      </c>
+      <c r="O352" s="2" t="inlineStr">
+        <is>
+          <t>5658.0</t>
+        </is>
+      </c>
+      <c r="R352" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S352" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59137,14 +59712,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N353" t="inlineStr">
-        <is>
-          <t>40431</t>
-        </is>
-      </c>
-      <c r="R353" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K353" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L353" s="2" t="inlineStr">
+        <is>
+          <t>41238.0</t>
+        </is>
+      </c>
+      <c r="M353" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N353" s="2" t="inlineStr">
+        <is>
+          <t>41238.0</t>
+        </is>
+      </c>
+      <c r="O353" s="2" t="inlineStr">
+        <is>
+          <t>7125.0</t>
+        </is>
+      </c>
+      <c r="R353" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S353" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59184,14 +59784,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N354" t="inlineStr">
-        <is>
-          <t>47216</t>
-        </is>
-      </c>
-      <c r="R354" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K354" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L354" s="2" t="inlineStr">
+        <is>
+          <t>88958.0</t>
+        </is>
+      </c>
+      <c r="M354" s="2" t="inlineStr">
+        <is>
+          <t>561000.0</t>
+        </is>
+      </c>
+      <c r="N354" s="2" t="inlineStr">
+        <is>
+          <t>649958.0</t>
+        </is>
+      </c>
+      <c r="O354" s="2" t="inlineStr">
+        <is>
+          <t>114443.0</t>
+        </is>
+      </c>
+      <c r="R354" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S354" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59231,14 +59856,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N355" t="inlineStr">
-        <is>
-          <t>29071</t>
-        </is>
-      </c>
-      <c r="R355" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K355" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L355" s="2" t="inlineStr">
+        <is>
+          <t>70451.0</t>
+        </is>
+      </c>
+      <c r="M355" s="2" t="inlineStr">
+        <is>
+          <t>605000.0</t>
+        </is>
+      </c>
+      <c r="N355" s="2" t="inlineStr">
+        <is>
+          <t>675451.0</t>
+        </is>
+      </c>
+      <c r="O355" s="2" t="inlineStr">
+        <is>
+          <t>448773.0</t>
+        </is>
+      </c>
+      <c r="R355" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S355" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59278,14 +59928,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N356" t="inlineStr">
-        <is>
-          <t>29025</t>
-        </is>
-      </c>
-      <c r="R356" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K356" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L356" s="2" t="inlineStr">
+        <is>
+          <t>70404.0</t>
+        </is>
+      </c>
+      <c r="M356" s="2" t="inlineStr">
+        <is>
+          <t>561000.0</t>
+        </is>
+      </c>
+      <c r="N356" s="2" t="inlineStr">
+        <is>
+          <t>631404.0</t>
+        </is>
+      </c>
+      <c r="O356" s="2" t="inlineStr">
+        <is>
+          <t>111237.0</t>
+        </is>
+      </c>
+      <c r="R356" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S356" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59325,14 +60000,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N357" t="inlineStr">
-        <is>
-          <t>29025</t>
-        </is>
-      </c>
-      <c r="R357" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K357" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L357" s="2" t="inlineStr">
+        <is>
+          <t>70404.0</t>
+        </is>
+      </c>
+      <c r="M357" s="2" t="inlineStr">
+        <is>
+          <t>605000.0</t>
+        </is>
+      </c>
+      <c r="N357" s="2" t="inlineStr">
+        <is>
+          <t>675404.0</t>
+        </is>
+      </c>
+      <c r="O357" s="2" t="inlineStr">
+        <is>
+          <t>121601.0</t>
+        </is>
+      </c>
+      <c r="R357" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S357" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59372,14 +60072,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N358" t="inlineStr">
-        <is>
-          <t>29025</t>
-        </is>
-      </c>
-      <c r="R358" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K358" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L358" s="2" t="inlineStr">
+        <is>
+          <t>70404.0</t>
+        </is>
+      </c>
+      <c r="M358" s="2" t="inlineStr">
+        <is>
+          <t>561000.0</t>
+        </is>
+      </c>
+      <c r="N358" s="2" t="inlineStr">
+        <is>
+          <t>631404.0</t>
+        </is>
+      </c>
+      <c r="O358" s="2" t="inlineStr">
+        <is>
+          <t>111237.0</t>
+        </is>
+      </c>
+      <c r="R358" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S358" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59419,14 +60144,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N359" t="inlineStr">
-        <is>
-          <t>7331</t>
-        </is>
-      </c>
-      <c r="R359" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K359" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L359" s="2" t="inlineStr">
+        <is>
+          <t>49366.0</t>
+        </is>
+      </c>
+      <c r="M359" s="2" t="inlineStr">
+        <is>
+          <t>571000.0</t>
+        </is>
+      </c>
+      <c r="N359" s="2" t="inlineStr">
+        <is>
+          <t>620366.0</t>
+        </is>
+      </c>
+      <c r="O359" s="2" t="inlineStr">
+        <is>
+          <t>113937.0</t>
+        </is>
+      </c>
+      <c r="R359" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S359" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59466,14 +60216,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N360" t="inlineStr">
-        <is>
-          <t>7331</t>
-        </is>
-      </c>
-      <c r="R360" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K360" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L360" s="2" t="inlineStr">
+        <is>
+          <t>49366.0</t>
+        </is>
+      </c>
+      <c r="M360" s="2" t="inlineStr">
+        <is>
+          <t>561000.0</t>
+        </is>
+      </c>
+      <c r="N360" s="2" t="inlineStr">
+        <is>
+          <t>610366.0</t>
+        </is>
+      </c>
+      <c r="O360" s="2" t="inlineStr">
+        <is>
+          <t>107602.0</t>
+        </is>
+      </c>
+      <c r="R360" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S360" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59513,14 +60288,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N361" t="inlineStr">
-        <is>
-          <t>6988</t>
-        </is>
-      </c>
-      <c r="R361" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K361" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L361" s="2" t="inlineStr">
+        <is>
+          <t>48965.0</t>
+        </is>
+      </c>
+      <c r="M361" s="2" t="inlineStr">
+        <is>
+          <t>605000.0</t>
+        </is>
+      </c>
+      <c r="N361" s="2" t="inlineStr">
+        <is>
+          <t>653965.0</t>
+        </is>
+      </c>
+      <c r="O361" s="2" t="inlineStr">
+        <is>
+          <t>117954.0</t>
+        </is>
+      </c>
+      <c r="R361" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S361" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59560,14 +60360,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N362" t="inlineStr">
-        <is>
-          <t>1018</t>
-        </is>
-      </c>
-      <c r="R362" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K362" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L362" s="2" t="inlineStr">
+        <is>
+          <t>48965.0</t>
+        </is>
+      </c>
+      <c r="M362" s="2" t="inlineStr">
+        <is>
+          <t>561000.0</t>
+        </is>
+      </c>
+      <c r="N362" s="2" t="inlineStr">
+        <is>
+          <t>609965.0</t>
+        </is>
+      </c>
+      <c r="O362" s="2" t="inlineStr">
+        <is>
+          <t>107533.0</t>
+        </is>
+      </c>
+      <c r="R362" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S362" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59607,14 +60432,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N363" t="inlineStr">
-        <is>
-          <t>1223</t>
-        </is>
-      </c>
-      <c r="R363" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K363" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L363" s="2" t="inlineStr">
+        <is>
+          <t>50603.0</t>
+        </is>
+      </c>
+      <c r="M363" s="2" t="inlineStr">
+        <is>
+          <t>571000.0</t>
+        </is>
+      </c>
+      <c r="N363" s="2" t="inlineStr">
+        <is>
+          <t>621603.0</t>
+        </is>
+      </c>
+      <c r="O363" s="2" t="inlineStr">
+        <is>
+          <t>115266.0</t>
+        </is>
+      </c>
+      <c r="R363" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S363" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59654,14 +60504,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N364" t="inlineStr">
-        <is>
-          <t>1507</t>
-        </is>
-      </c>
-      <c r="R364" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K364" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L364" s="2" t="inlineStr">
+        <is>
+          <t>52887.0</t>
+        </is>
+      </c>
+      <c r="M364" s="2" t="inlineStr">
+        <is>
+          <t>561000.0</t>
+        </is>
+      </c>
+      <c r="N364" s="2" t="inlineStr">
+        <is>
+          <t>613887.0</t>
+        </is>
+      </c>
+      <c r="O364" s="2" t="inlineStr">
+        <is>
+          <t>390827.0</t>
+        </is>
+      </c>
+      <c r="R364" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S364" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59701,14 +60576,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N365" t="inlineStr">
-        <is>
-          <t>1101</t>
-        </is>
-      </c>
-      <c r="R365" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K365" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L365" s="2" t="inlineStr">
+        <is>
+          <t>49635.0</t>
+        </is>
+      </c>
+      <c r="M365" s="2" t="inlineStr">
+        <is>
+          <t>571000.0</t>
+        </is>
+      </c>
+      <c r="N365" s="2" t="inlineStr">
+        <is>
+          <t>620635.0</t>
+        </is>
+      </c>
+      <c r="O365" s="2" t="inlineStr">
+        <is>
+          <t>115095.0</t>
+        </is>
+      </c>
+      <c r="R365" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S365" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59748,14 +60648,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N366" t="inlineStr">
-        <is>
-          <t>1101</t>
-        </is>
-      </c>
-      <c r="R366" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K366" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L366" s="2" t="inlineStr">
+        <is>
+          <t>49635.0</t>
+        </is>
+      </c>
+      <c r="M366" s="2" t="inlineStr">
+        <is>
+          <t>561000.0</t>
+        </is>
+      </c>
+      <c r="N366" s="2" t="inlineStr">
+        <is>
+          <t>610635.0</t>
+        </is>
+      </c>
+      <c r="O366" s="2" t="inlineStr">
+        <is>
+          <t>107648.0</t>
+        </is>
+      </c>
+      <c r="R366" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S366" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59795,14 +60720,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N367" t="inlineStr">
-        <is>
-          <t>1101</t>
-        </is>
-      </c>
-      <c r="R367" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K367" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L367" s="2" t="inlineStr">
+        <is>
+          <t>49635.0</t>
+        </is>
+      </c>
+      <c r="M367" s="2" t="inlineStr">
+        <is>
+          <t>605000.0</t>
+        </is>
+      </c>
+      <c r="N367" s="2" t="inlineStr">
+        <is>
+          <t>654635.0</t>
+        </is>
+      </c>
+      <c r="O367" s="2" t="inlineStr">
+        <is>
+          <t>434959.0</t>
+        </is>
+      </c>
+      <c r="R367" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S367" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59842,14 +60792,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N368" t="inlineStr">
-        <is>
-          <t>1101</t>
-        </is>
-      </c>
-      <c r="R368" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K368" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L368" s="2" t="inlineStr">
+        <is>
+          <t>49635.0</t>
+        </is>
+      </c>
+      <c r="M368" s="2" t="inlineStr">
+        <is>
+          <t>561000.0</t>
+        </is>
+      </c>
+      <c r="N368" s="2" t="inlineStr">
+        <is>
+          <t>610635.0</t>
+        </is>
+      </c>
+      <c r="O368" s="2" t="inlineStr">
+        <is>
+          <t>107648.0</t>
+        </is>
+      </c>
+      <c r="R368" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S368" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59889,14 +60864,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N369" t="inlineStr">
-        <is>
-          <t>29932</t>
-        </is>
-      </c>
-      <c r="R369" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K369" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L369" s="2" t="inlineStr">
+        <is>
+          <t>71329.0</t>
+        </is>
+      </c>
+      <c r="M369" s="2" t="inlineStr">
+        <is>
+          <t>571000.0</t>
+        </is>
+      </c>
+      <c r="N369" s="2" t="inlineStr">
+        <is>
+          <t>642329.0</t>
+        </is>
+      </c>
+      <c r="O369" s="2" t="inlineStr">
+        <is>
+          <t>118930.0</t>
+        </is>
+      </c>
+      <c r="R369" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S369" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59936,14 +60936,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N370" t="inlineStr">
-        <is>
-          <t>29932</t>
-        </is>
-      </c>
-      <c r="R370" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K370" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L370" s="2" t="inlineStr">
+        <is>
+          <t>30529.0</t>
+        </is>
+      </c>
+      <c r="M370" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N370" s="2" t="inlineStr">
+        <is>
+          <t>30529.0</t>
+        </is>
+      </c>
+      <c r="O370" s="2" t="inlineStr">
+        <is>
+          <t>5275.0</t>
+        </is>
+      </c>
+      <c r="R370" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S370" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -59983,14 +61008,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N371" t="inlineStr">
-        <is>
-          <t>29932</t>
-        </is>
-      </c>
-      <c r="R371" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K371" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L371" s="2" t="inlineStr">
+        <is>
+          <t>30529.0</t>
+        </is>
+      </c>
+      <c r="M371" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N371" s="2" t="inlineStr">
+        <is>
+          <t>30529.0</t>
+        </is>
+      </c>
+      <c r="O371" s="2" t="inlineStr">
+        <is>
+          <t>5397.0</t>
+        </is>
+      </c>
+      <c r="R371" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S371" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60030,14 +61080,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N372" t="inlineStr">
-        <is>
-          <t>55923</t>
-        </is>
-      </c>
-      <c r="R372" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K372" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L372" s="2" t="inlineStr">
+        <is>
+          <t>97840.0</t>
+        </is>
+      </c>
+      <c r="M372" s="2" t="inlineStr">
+        <is>
+          <t>561000.0</t>
+        </is>
+      </c>
+      <c r="N372" s="2" t="inlineStr">
+        <is>
+          <t>658840.0</t>
+        </is>
+      </c>
+      <c r="O372" s="2" t="inlineStr">
+        <is>
+          <t>419134.0</t>
+        </is>
+      </c>
+      <c r="R372" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S372" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60077,14 +61152,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N373" t="inlineStr">
-        <is>
-          <t>47738</t>
-        </is>
-      </c>
-      <c r="R373" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K373" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L373" s="2" t="inlineStr">
+        <is>
+          <t>89491.0</t>
+        </is>
+      </c>
+      <c r="M373" s="2" t="inlineStr">
+        <is>
+          <t>572220.0</t>
+        </is>
+      </c>
+      <c r="N373" s="2" t="inlineStr">
+        <is>
+          <t>661711.0</t>
+        </is>
+      </c>
+      <c r="O373" s="2" t="inlineStr">
+        <is>
+          <t>116518.0</t>
+        </is>
+      </c>
+      <c r="R373" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S373" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60124,14 +61224,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N374" t="inlineStr">
-        <is>
-          <t>27211</t>
-        </is>
-      </c>
-      <c r="R374" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K374" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L374" s="2" t="inlineStr">
+        <is>
+          <t>68555.0</t>
+        </is>
+      </c>
+      <c r="M374" s="2" t="inlineStr">
+        <is>
+          <t>582420.0</t>
+        </is>
+      </c>
+      <c r="N374" s="2" t="inlineStr">
+        <is>
+          <t>650975.0</t>
+        </is>
+      </c>
+      <c r="O374" s="2" t="inlineStr">
+        <is>
+          <t>351865.0</t>
+        </is>
+      </c>
+      <c r="R374" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S374" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60171,14 +61296,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N375" t="inlineStr">
-        <is>
-          <t>27211</t>
-        </is>
-      </c>
-      <c r="R375" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K375" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L375" s="2" t="inlineStr">
+        <is>
+          <t>68555.0</t>
+        </is>
+      </c>
+      <c r="M375" s="2" t="inlineStr">
+        <is>
+          <t>617100.0</t>
+        </is>
+      </c>
+      <c r="N375" s="2" t="inlineStr">
+        <is>
+          <t>685655.0</t>
+        </is>
+      </c>
+      <c r="O375" s="2" t="inlineStr">
+        <is>
+          <t>123479.0</t>
+        </is>
+      </c>
+      <c r="R375" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S375" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60218,14 +61368,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N376" t="inlineStr">
-        <is>
-          <t>27211</t>
-        </is>
-      </c>
-      <c r="R376" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K376" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L376" s="2" t="inlineStr">
+        <is>
+          <t>68555.0</t>
+        </is>
+      </c>
+      <c r="M376" s="2" t="inlineStr">
+        <is>
+          <t>572220.0</t>
+        </is>
+      </c>
+      <c r="N376" s="2" t="inlineStr">
+        <is>
+          <t>640775.0</t>
+        </is>
+      </c>
+      <c r="O376" s="2" t="inlineStr">
+        <is>
+          <t>112900.0</t>
+        </is>
+      </c>
+      <c r="R376" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S376" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60265,14 +61440,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N377" t="inlineStr">
-        <is>
-          <t>6874</t>
-        </is>
-      </c>
-      <c r="R377" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K377" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L377" s="2" t="inlineStr">
+        <is>
+          <t>48832.0</t>
+        </is>
+      </c>
+      <c r="M377" s="2" t="inlineStr">
+        <is>
+          <t>582420.0</t>
+        </is>
+      </c>
+      <c r="N377" s="2" t="inlineStr">
+        <is>
+          <t>631252.0</t>
+        </is>
+      </c>
+      <c r="O377" s="2" t="inlineStr">
+        <is>
+          <t>341301.0</t>
+        </is>
+      </c>
+      <c r="R377" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S377" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60312,14 +61512,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N378" t="inlineStr">
-        <is>
-          <t>6874</t>
-        </is>
-      </c>
-      <c r="R378" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K378" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L378" s="2" t="inlineStr">
+        <is>
+          <t>8032.0</t>
+        </is>
+      </c>
+      <c r="M378" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N378" s="2" t="inlineStr">
+        <is>
+          <t>8032.0</t>
+        </is>
+      </c>
+      <c r="O378" s="2" t="inlineStr">
+        <is>
+          <t>1366.0</t>
+        </is>
+      </c>
+      <c r="R378" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S378" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60359,14 +61584,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N379" t="inlineStr">
-        <is>
-          <t>6874</t>
-        </is>
-      </c>
-      <c r="R379" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K379" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L379" s="2" t="inlineStr">
+        <is>
+          <t>48832.0</t>
+        </is>
+      </c>
+      <c r="M379" s="2" t="inlineStr">
+        <is>
+          <t>572220.0</t>
+        </is>
+      </c>
+      <c r="N379" s="2" t="inlineStr">
+        <is>
+          <t>621052.0</t>
+        </is>
+      </c>
+      <c r="O379" s="2" t="inlineStr">
+        <is>
+          <t>109492.0</t>
+        </is>
+      </c>
+      <c r="R379" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S379" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60406,14 +61656,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N380" t="inlineStr">
-        <is>
-          <t>6874</t>
-        </is>
-      </c>
-      <c r="R380" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K380" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L380" s="2" t="inlineStr">
+        <is>
+          <t>48832.0</t>
+        </is>
+      </c>
+      <c r="M380" s="2" t="inlineStr">
+        <is>
+          <t>582420.0</t>
+        </is>
+      </c>
+      <c r="N380" s="2" t="inlineStr">
+        <is>
+          <t>631252.0</t>
+        </is>
+      </c>
+      <c r="O380" s="2" t="inlineStr">
+        <is>
+          <t>341301.0</t>
+        </is>
+      </c>
+      <c r="R380" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S380" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60453,14 +61728,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N381" t="inlineStr">
-        <is>
-          <t>8329</t>
-        </is>
-      </c>
-      <c r="R381" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K381" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L381" s="2" t="inlineStr">
+        <is>
+          <t>50532.0</t>
+        </is>
+      </c>
+      <c r="M381" s="2" t="inlineStr">
+        <is>
+          <t>572220.0</t>
+        </is>
+      </c>
+      <c r="N381" s="2" t="inlineStr">
+        <is>
+          <t>622752.0</t>
+        </is>
+      </c>
+      <c r="O381" s="2" t="inlineStr">
+        <is>
+          <t>622752.0</t>
+        </is>
+      </c>
+      <c r="R381" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S381" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60537,14 +61837,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N383" t="inlineStr">
-        <is>
-          <t>11538</t>
-        </is>
-      </c>
-      <c r="R383" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K383" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L383" s="2" t="inlineStr">
+        <is>
+          <t>54282.0</t>
+        </is>
+      </c>
+      <c r="M383" s="2" t="inlineStr">
+        <is>
+          <t>408000.0</t>
+        </is>
+      </c>
+      <c r="N383" s="2" t="inlineStr">
+        <is>
+          <t>462282.0</t>
+        </is>
+      </c>
+      <c r="O383" s="2" t="inlineStr">
+        <is>
+          <t>132718.0</t>
+        </is>
+      </c>
+      <c r="R383" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S383" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60584,14 +61909,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N384" t="inlineStr">
-        <is>
-          <t>11625</t>
-        </is>
-      </c>
-      <c r="R384" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K384" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L384" s="2" t="inlineStr">
+        <is>
+          <t>54384.0</t>
+        </is>
+      </c>
+      <c r="M384" s="2" t="inlineStr">
+        <is>
+          <t>397800.0</t>
+        </is>
+      </c>
+      <c r="N384" s="2" t="inlineStr">
+        <is>
+          <t>452184.0</t>
+        </is>
+      </c>
+      <c r="O384" s="2" t="inlineStr">
+        <is>
+          <t>452184.0</t>
+        </is>
+      </c>
+      <c r="R384" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S384" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60631,14 +61981,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N385" t="inlineStr">
-        <is>
-          <t>11618</t>
-        </is>
-      </c>
-      <c r="R385" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K385" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L385" s="2" t="inlineStr">
+        <is>
+          <t>13574.0</t>
+        </is>
+      </c>
+      <c r="M385" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N385" s="2" t="inlineStr">
+        <is>
+          <t>13574.0</t>
+        </is>
+      </c>
+      <c r="O385" s="2" t="inlineStr">
+        <is>
+          <t>3743.0</t>
+        </is>
+      </c>
+      <c r="R385" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S385" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60678,14 +62053,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N386" t="inlineStr">
-        <is>
-          <t>11609</t>
-        </is>
-      </c>
-      <c r="R386" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K386" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L386" s="2" t="inlineStr">
+        <is>
+          <t>54364.0</t>
+        </is>
+      </c>
+      <c r="M386" s="2" t="inlineStr">
+        <is>
+          <t>397800.0</t>
+        </is>
+      </c>
+      <c r="N386" s="2" t="inlineStr">
+        <is>
+          <t>452164.0</t>
+        </is>
+      </c>
+      <c r="O386" s="2" t="inlineStr">
+        <is>
+          <t>161808.0</t>
+        </is>
+      </c>
+      <c r="R386" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S386" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60725,14 +62125,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N387" t="inlineStr">
-        <is>
-          <t>11771</t>
-        </is>
-      </c>
-      <c r="R387" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K387" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L387" s="2" t="inlineStr">
+        <is>
+          <t>54554.0</t>
+        </is>
+      </c>
+      <c r="M387" s="2" t="inlineStr">
+        <is>
+          <t>408000.0</t>
+        </is>
+      </c>
+      <c r="N387" s="2" t="inlineStr">
+        <is>
+          <t>462554.0</t>
+        </is>
+      </c>
+      <c r="O387" s="2" t="inlineStr">
+        <is>
+          <t>132793.0</t>
+        </is>
+      </c>
+      <c r="R387" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S387" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60772,14 +62197,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N388" t="inlineStr">
-        <is>
-          <t>56604</t>
-        </is>
-      </c>
-      <c r="R388" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K388" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L388" s="2" t="inlineStr">
+        <is>
+          <t>98534.0</t>
+        </is>
+      </c>
+      <c r="M388" s="2" t="inlineStr">
+        <is>
+          <t>572220.0</t>
+        </is>
+      </c>
+      <c r="N388" s="2" t="inlineStr">
+        <is>
+          <t>670754.0</t>
+        </is>
+      </c>
+      <c r="O388" s="2" t="inlineStr">
+        <is>
+          <t>362111.0</t>
+        </is>
+      </c>
+      <c r="R388" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S388" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60819,14 +62269,39 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N389" t="inlineStr">
-        <is>
-          <t>60404</t>
-        </is>
-      </c>
-      <c r="R389" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K389" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L389" s="2" t="inlineStr">
+        <is>
+          <t>61611.0</t>
+        </is>
+      </c>
+      <c r="M389" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N389" s="2" t="inlineStr">
+        <is>
+          <t>61611.0</t>
+        </is>
+      </c>
+      <c r="O389" s="2" t="inlineStr">
+        <is>
+          <t>24570.0</t>
+        </is>
+      </c>
+      <c r="R389" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S389" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60846,6 +62321,21 @@
           <t>Bennington Apartments</t>
         </is>
       </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>168150010</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>0168-150-010</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>2780 NORTH TEXAS STREET FAIRFIELD</t>
+        </is>
+      </c>
       <c r="G390" t="inlineStr">
         <is>
           <t>False</t>
@@ -60853,7 +62343,47 @@
       </c>
       <c r="H390" t="inlineStr">
         <is>
-          <t>collaborator-sheet</t>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>Single Real Property parcel at the project situs per Solano assessor portal search 2026-08-22 (other hits are business accounts)</t>
+        </is>
+      </c>
+      <c r="K390" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L390" s="2" t="inlineStr">
+        <is>
+          <t>5338692.0</t>
+        </is>
+      </c>
+      <c r="M390" s="2" t="inlineStr">
+        <is>
+          <t>23942991.0</t>
+        </is>
+      </c>
+      <c r="N390" s="2" t="inlineStr">
+        <is>
+          <t>29281683.0</t>
+        </is>
+      </c>
+      <c r="O390" s="2" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="R390" s="2" t="inlineStr">
+        <is>
+          <t>solano-county-portal</t>
+        </is>
+      </c>
+      <c r="S390" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -60925,7 +62455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C201"/>
+  <dimension ref="A1:C200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -63129,7 +64659,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>la-fetch-fallback</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -63139,7 +64669,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>AIN 6020022027 has no current roll data; using manual value</t>
+          <t>AIN 6020022027 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
@@ -63163,7 +64693,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>la-fetch-fallback</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -63173,14 +64703,14 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>AIN 5036031006 has no current roll data; using manual value</t>
+          <t>AIN 5036031006 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>la-fetch-fallback</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -63190,14 +64720,14 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>AIN 4262018026 has no current roll data; using manual value</t>
+          <t>AIN 4262018026 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>la-fetch-fallback</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -63207,14 +64737,14 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>AIN 6020022027 has no current roll data; using manual value</t>
+          <t>AIN 6020022027 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>la-fetch-fallback</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -63224,7 +64754,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>AIN 2125017014 has no current roll data; using manual value</t>
+          <t>AIN 2125017014 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
@@ -64081,34 +65611,34 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>missing-parcels</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>238</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>AIN (none) (Solano): no roll values from any source</t>
+          <t>Heritage Park Apartments Livermore: authorized, not dead, no parcel rows</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>missing-parcels</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>238</t>
+          <t>143/147</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Heritage Park Apartments Livermore: authorized, not dead, no parcel rows</t>
+          <t>AIN 41416654 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -64120,12 +65650,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>143/147</t>
+          <t>182/76</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>AIN 41416654 assigned to multiple projects</t>
+          <t>AIN 5036031006 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -64137,12 +65667,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>182/76</t>
+          <t>130/179</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>AIN 5036031006 assigned to multiple projects</t>
+          <t>AIN 5080006008 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -64154,12 +65684,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>130/179</t>
+          <t>126/173</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>AIN 5080006008 assigned to multiple projects</t>
+          <t>AIN 5094005005 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -64171,12 +65701,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>126/173</t>
+          <t>127/174</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>AIN 5094005005 assigned to multiple projects</t>
+          <t>AIN 5094006003 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -64188,12 +65718,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>127/174</t>
+          <t>122/165</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>AIN 5094006003 assigned to multiple projects</t>
+          <t>AIN 5094017020 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -64205,12 +65735,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>122/165</t>
+          <t>124/169</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>AIN 5094017020 assigned to multiple projects</t>
+          <t>AIN 5094023025 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -64222,12 +65752,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>124/169</t>
+          <t>128/175</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>AIN 5094023025 assigned to multiple projects</t>
+          <t>AIN 5502019004 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -64239,12 +65769,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>128/175</t>
+          <t>125/170</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>AIN 5502019004 assigned to multiple projects</t>
+          <t>AIN 5503024012 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -64256,12 +65786,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>125/170</t>
+          <t>129/177</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>AIN 5503024012 assigned to multiple projects</t>
+          <t>AIN 5517005016 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -64273,12 +65803,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>129/177</t>
+          <t>121/162</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>AIN 5517005016 assigned to multiple projects</t>
+          <t>AIN 5518013024 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -64290,12 +65820,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>121/162</t>
+          <t>123/168</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>AIN 5518013024 assigned to multiple projects</t>
+          <t>AIN 5518020021 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -64307,12 +65837,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>123/168</t>
+          <t>10/132</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>AIN 5518020021 assigned to multiple projects</t>
+          <t>AIN 6020022027 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -64324,27 +65854,10 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>10/132</t>
+          <t>152/181</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
-        <is>
-          <t>AIN 6020022027 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B201" t="inlineStr">
-        <is>
-          <t>152/181</t>
-        </is>
-      </c>
-      <c r="C201" t="inlineStr">
         <is>
           <t>AIN 7157012017 assigned to multiple projects</t>
         </is>

</xml_diff>

<commit_message>
Automate San Diego County assessed values via SANDAG parcels layer
geo.sandag.org hosted Parcels feature layer (maintained from county
ARCC data, last edited Aug 2026) supplies asr_land/asr_impr/asr_total
for all 13 assigned San Diego APNs. The layer publishes no exemption
field, so build_dataset now falls back field-level to the manual
exemption for a parcel when the value source lacks one (provenance-
recorded). Probed Santa Clara (Cloudflare-walled everywhere), San
Mateo and Alameda (no public value services found) — those counties
stay manual for now.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -34903,14 +34903,44 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>9316117</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>2202858</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>7489628</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>9692486</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>sandag-parcels</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -35844,14 +35874,44 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>32460480</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>9568699</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>24203182</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>33771881</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>sandag-parcels</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -40766,14 +40826,44 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N75" t="inlineStr">
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>13158000</t>
+        </is>
+      </c>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>204000</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="inlineStr">
         <is>
           <t>13362000</t>
         </is>
       </c>
-      <c r="R75" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="P75" s="2" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="Q75" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="R75" s="2" t="inlineStr">
+        <is>
+          <t>sandag-parcels</t>
+        </is>
+      </c>
+      <c r="S75" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -41172,14 +41262,44 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N83" t="inlineStr">
-        <is>
-          <t>53339453</t>
-        </is>
-      </c>
-      <c r="R83" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L83" s="2" t="inlineStr">
+        <is>
+          <t>18360000</t>
+        </is>
+      </c>
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>50003178</t>
+        </is>
+      </c>
+      <c r="N83" s="2" t="inlineStr">
+        <is>
+          <t>68363178</t>
+        </is>
+      </c>
+      <c r="P83" s="2" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="Q83" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="R83" s="2" t="inlineStr">
+        <is>
+          <t>sandag-parcels</t>
+        </is>
+      </c>
+      <c r="S83" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -41219,14 +41339,44 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N84" t="inlineStr">
-        <is>
-          <t>5832864</t>
-        </is>
-      </c>
-      <c r="R84" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>2142762</t>
+        </is>
+      </c>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>3925748</t>
+        </is>
+      </c>
+      <c r="N84" s="2" t="inlineStr">
+        <is>
+          <t>6068510</t>
+        </is>
+      </c>
+      <c r="P84" s="2" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="Q84" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="R84" s="2" t="inlineStr">
+        <is>
+          <t>sandag-parcels</t>
+        </is>
+      </c>
+      <c r="S84" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -46298,14 +46448,44 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N146" t="inlineStr">
-        <is>
-          <t>2804259</t>
-        </is>
-      </c>
-      <c r="R146" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K146" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L146" s="2" t="inlineStr">
+        <is>
+          <t>4462500</t>
+        </is>
+      </c>
+      <c r="M146" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N146" s="2" t="inlineStr">
+        <is>
+          <t>4462500</t>
+        </is>
+      </c>
+      <c r="P146" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  </t>
+        </is>
+      </c>
+      <c r="Q146" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="R146" s="2" t="inlineStr">
+        <is>
+          <t>sandag-parcels</t>
+        </is>
+      </c>
+      <c r="S146" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -46345,14 +46525,44 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N147" t="inlineStr">
-        <is>
-          <t>30350548</t>
-        </is>
-      </c>
-      <c r="R147" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K147" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L147" s="2" t="inlineStr">
+        <is>
+          <t>23383000</t>
+        </is>
+      </c>
+      <c r="M147" s="2" t="inlineStr">
+        <is>
+          <t>10021000</t>
+        </is>
+      </c>
+      <c r="N147" s="2" t="inlineStr">
+        <is>
+          <t>33404000</t>
+        </is>
+      </c>
+      <c r="P147" s="2" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="Q147" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="R147" s="2" t="inlineStr">
+        <is>
+          <t>sandag-parcels</t>
+        </is>
+      </c>
+      <c r="S147" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -47831,14 +48041,44 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N165" t="inlineStr">
-        <is>
-          <t>51548563</t>
-        </is>
-      </c>
-      <c r="R165" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K165" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L165" s="2" t="inlineStr">
+        <is>
+          <t>30000000</t>
+        </is>
+      </c>
+      <c r="M165" s="2" t="inlineStr">
+        <is>
+          <t>43424100</t>
+        </is>
+      </c>
+      <c r="N165" s="2" t="inlineStr">
+        <is>
+          <t>73424100</t>
+        </is>
+      </c>
+      <c r="P165" s="2" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="Q165" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="R165" s="2" t="inlineStr">
+        <is>
+          <t>sandag-parcels</t>
+        </is>
+      </c>
+      <c r="S165" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -52860,14 +53100,44 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N227" t="inlineStr">
-        <is>
-          <t>12540125</t>
-        </is>
-      </c>
-      <c r="R227" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K227" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L227" s="2" t="inlineStr">
+        <is>
+          <t>5116369</t>
+        </is>
+      </c>
+      <c r="M227" s="2" t="inlineStr">
+        <is>
+          <t>7674557</t>
+        </is>
+      </c>
+      <c r="N227" s="2" t="inlineStr">
+        <is>
+          <t>12790926</t>
+        </is>
+      </c>
+      <c r="P227" s="2" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="Q227" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="R227" s="2" t="inlineStr">
+        <is>
+          <t>sandag-parcels</t>
+        </is>
+      </c>
+      <c r="S227" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -52907,14 +53177,44 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N228" t="inlineStr">
-        <is>
-          <t>41107952</t>
-        </is>
-      </c>
-      <c r="R228" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K228" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L228" s="2" t="inlineStr">
+        <is>
+          <t>20621754</t>
+        </is>
+      </c>
+      <c r="M228" s="2" t="inlineStr">
+        <is>
+          <t>21308356</t>
+        </is>
+      </c>
+      <c r="N228" s="2" t="inlineStr">
+        <is>
+          <t>41930110</t>
+        </is>
+      </c>
+      <c r="P228" s="2" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="Q228" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="R228" s="2" t="inlineStr">
+        <is>
+          <t>sandag-parcels</t>
+        </is>
+      </c>
+      <c r="S228" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -52954,14 +53254,44 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N229" t="inlineStr">
-        <is>
-          <t>18982539</t>
-        </is>
-      </c>
-      <c r="R229" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K229" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L229" s="2" t="inlineStr">
+        <is>
+          <t>7937360</t>
+        </is>
+      </c>
+      <c r="M229" s="2" t="inlineStr">
+        <is>
+          <t>11424829</t>
+        </is>
+      </c>
+      <c r="N229" s="2" t="inlineStr">
+        <is>
+          <t>19362189</t>
+        </is>
+      </c>
+      <c r="P229" s="2" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="Q229" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="R229" s="2" t="inlineStr">
+        <is>
+          <t>sandag-parcels</t>
+        </is>
+      </c>
+      <c r="S229" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -53001,14 +53331,44 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N230" t="inlineStr">
-        <is>
-          <t>12540125</t>
-        </is>
-      </c>
-      <c r="R230" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="K230" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L230" s="2" t="inlineStr">
+        <is>
+          <t>5116369</t>
+        </is>
+      </c>
+      <c r="M230" s="2" t="inlineStr">
+        <is>
+          <t>7674557</t>
+        </is>
+      </c>
+      <c r="N230" s="2" t="inlineStr">
+        <is>
+          <t>12790926</t>
+        </is>
+      </c>
+      <c r="P230" s="2" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="Q230" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="R230" s="2" t="inlineStr">
+        <is>
+          <t>sandag-parcels</t>
+        </is>
+      </c>
+      <c r="S230" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>
@@ -55776,19 +56136,49 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
-      <c r="N265" t="inlineStr">
-        <is>
-          <t>49668778</t>
-        </is>
-      </c>
-      <c r="O265" t="inlineStr">
+      <c r="K265" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L265" s="2" t="inlineStr">
+        <is>
+          <t>30308100</t>
+        </is>
+      </c>
+      <c r="M265" s="2" t="inlineStr">
+        <is>
+          <t>20354053</t>
+        </is>
+      </c>
+      <c r="N265" s="2" t="inlineStr">
+        <is>
+          <t>50662153</t>
+        </is>
+      </c>
+      <c r="O265" s="2" t="inlineStr">
         <is>
           <t>49157189</t>
         </is>
       </c>
-      <c r="R265" t="inlineStr">
-        <is>
-          <t>collaborator-sheet</t>
+      <c r="P265" s="2" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="Q265" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="R265" s="2" t="inlineStr">
+        <is>
+          <t>sandag-parcels</t>
+        </is>
+      </c>
+      <c r="S265" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Resolve parcels for Park View, Bluwater, Guava Gardens, Verdana; record 3 addresses
Addresses for Baird / Hazelhurst / Park View recorded as manual
overrides (Drew). Situs lookups: Park View -> LA AIN 5157007028;
Bluwater Crossing -> SANDAG 2146500200 (66 units, $49.3M); Guava
Gardens -> 4701122500; Verdana -> 4441201300 + 4441201800. Hazelhurst
is North Hollywood (not Bonita); no exact 6144 situs exists — 6142 /
6146 are the candidate parcels, left for manual pick, as is Baird
(no 6840; block has 6838/6852/6804).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -24937,6 +24937,11 @@
           <t>Grant up to $10,000 (Charitable Affordable Housing)</t>
         </is>
       </c>
+      <c r="T199" t="inlineStr">
+        <is>
+          <t>6840 Baird Ave, Los Angeles, CA 91335</t>
+        </is>
+      </c>
       <c r="AD199" t="inlineStr">
         <is>
           <t>operative</t>
@@ -24954,7 +24959,7 @@
       </c>
       <c r="AH199" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>restricted_units:collaborator-sheet; city_cut:collaborator-sheet; address:manual-repo-edit</t>
         </is>
       </c>
     </row>
@@ -25527,6 +25532,11 @@
           <t>Grant up to $10,000 (Charitable Affordable Housing)</t>
         </is>
       </c>
+      <c r="T204" t="inlineStr">
+        <is>
+          <t>6144 Hazelhurst Place, North Hollywood, CA 91606</t>
+        </is>
+      </c>
       <c r="W204" t="inlineStr">
         <is>
           <t>YES</t>
@@ -25549,7 +25559,7 @@
       </c>
       <c r="AH204" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:manual-repo-edit</t>
         </is>
       </c>
     </row>
@@ -27033,6 +27043,11 @@
           <t>Grant up to $10,000 (Charitable Affordable Housing)</t>
         </is>
       </c>
+      <c r="T217" t="inlineStr">
+        <is>
+          <t>217 N. Park View Street, Los Angeles, CA 90026</t>
+        </is>
+      </c>
       <c r="W217" t="inlineStr">
         <is>
           <t>YES</t>
@@ -27055,7 +27070,7 @@
       </c>
       <c r="AH217" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:manual-repo-edit</t>
         </is>
       </c>
     </row>
@@ -36124,7 +36139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T392"/>
+  <dimension ref="A1:T394"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42491,7 +42506,7 @@
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4284000</t>
         </is>
       </c>
       <c r="P70" s="2" t="inlineStr">
@@ -59787,6 +59802,21 @@
           <t>Bluwater Crossing Apartments</t>
         </is>
       </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>2146500200</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>214-650-02-00</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>6790 EMBARCADERO LN CARLSBAD CA 92011</t>
+        </is>
+      </c>
       <c r="G279" t="inlineStr">
         <is>
           <t>False</t>
@@ -59794,7 +59824,52 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>collaborator-sheet</t>
+          <t>script-situs-match (2026-08-22)</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>Exact situs match, SANDAG; 66-unit apartment parcel</t>
+        </is>
+      </c>
+      <c r="K279" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L279" s="2" t="inlineStr">
+        <is>
+          <t>15568767</t>
+        </is>
+      </c>
+      <c r="M279" s="2" t="inlineStr">
+        <is>
+          <t>33766648</t>
+        </is>
+      </c>
+      <c r="N279" s="2" t="inlineStr">
+        <is>
+          <t>49335415</t>
+        </is>
+      </c>
+      <c r="P279" s="2" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="Q279" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="R279" s="2" t="inlineStr">
+        <is>
+          <t>sandag-parcels</t>
+        </is>
+      </c>
+      <c r="S279" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="T279" t="inlineStr">
@@ -60216,6 +60291,21 @@
           <t>Guava Gardens Apartments</t>
         </is>
       </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>4701122500</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>470-112-25-00</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>5035 GUAVA AVE LA MESA CA 91942</t>
+        </is>
+      </c>
       <c r="G286" t="inlineStr">
         <is>
           <t>False</t>
@@ -60223,7 +60313,52 @@
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>collaborator-sheet</t>
+          <t>script-situs-match (2026-08-22)</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>Exact situs match, SANDAG; 81-unit apartment parcel</t>
+        </is>
+      </c>
+      <c r="K286" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L286" s="2" t="inlineStr">
+        <is>
+          <t>2033407</t>
+        </is>
+      </c>
+      <c r="M286" s="2" t="inlineStr">
+        <is>
+          <t>3050116</t>
+        </is>
+      </c>
+      <c r="N286" s="2" t="inlineStr">
+        <is>
+          <t>5083523</t>
+        </is>
+      </c>
+      <c r="P286" s="2" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="Q286" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="R286" s="2" t="inlineStr">
+        <is>
+          <t>sandag-parcels</t>
+        </is>
+      </c>
+      <c r="S286" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="T286" t="inlineStr">
@@ -60248,6 +60383,21 @@
           <t>Park View by Angeleno Apartments</t>
         </is>
       </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>5157007028</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>5157-007-028</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>217 N PARK VIEW ST LOS ANGELES CA 90026</t>
+        </is>
+      </c>
       <c r="G287" t="inlineStr">
         <is>
           <t>False</t>
@@ -60255,7 +60405,57 @@
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>collaborator-sheet</t>
+          <t>script-situs-match (2026-08-22)</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>Exact situs match, LA parcel API; use still "Single" (pre-development)</t>
+        </is>
+      </c>
+      <c r="K287" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L287" s="2" t="inlineStr">
+        <is>
+          <t>938400</t>
+        </is>
+      </c>
+      <c r="M287" s="2" t="inlineStr">
+        <is>
+          <t>234600</t>
+        </is>
+      </c>
+      <c r="N287" s="2" t="inlineStr">
+        <is>
+          <t>1173000</t>
+        </is>
+      </c>
+      <c r="O287" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P287" s="2" t="inlineStr">
+        <is>
+          <t>1911</t>
+        </is>
+      </c>
+      <c r="Q287" s="2" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="R287" s="2" t="inlineStr">
+        <is>
+          <t>la-county-api</t>
+        </is>
+      </c>
+      <c r="S287" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="T287" t="inlineStr">
@@ -67511,6 +67711,200 @@
       <c r="T392" t="inlineStr">
         <is>
           <t>230</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>369</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Verdana Apartments</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>4441201300</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>444-120-13-00</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>438 CAMINO DEL RIO S SAN DIEGO CA 92108</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>script-situs-match (2026-08-22)</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>situs-match</t>
+        </is>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>Exact situs match, SANDAG; pre-development parcels per staff report address</t>
+        </is>
+      </c>
+      <c r="K393" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L393" s="2" t="inlineStr">
+        <is>
+          <t>2427182</t>
+        </is>
+      </c>
+      <c r="M393" s="2" t="inlineStr">
+        <is>
+          <t>1490976</t>
+        </is>
+      </c>
+      <c r="N393" s="2" t="inlineStr">
+        <is>
+          <t>3918158</t>
+        </is>
+      </c>
+      <c r="P393" s="2" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="Q393" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="R393" s="2" t="inlineStr">
+        <is>
+          <t>sandag-parcels</t>
+        </is>
+      </c>
+      <c r="S393" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="T393" t="inlineStr">
+        <is>
+          <t>369</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>369</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Verdana Apartments</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>4441201800</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>444-120-18-00</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>480 CAMINO DEL RIO S SAN DIEGO CA 92108</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>script-situs-match (2026-08-22)</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>situs-match</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>Exact situs match, SANDAG; pre-development parcels per staff report address</t>
+        </is>
+      </c>
+      <c r="K394" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L394" s="2" t="inlineStr">
+        <is>
+          <t>1884643</t>
+        </is>
+      </c>
+      <c r="M394" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N394" s="2" t="inlineStr">
+        <is>
+          <t>1884643</t>
+        </is>
+      </c>
+      <c r="P394" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  </t>
+        </is>
+      </c>
+      <c r="Q394" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="R394" s="2" t="inlineStr">
+        <is>
+          <t>sandag-parcels</t>
+        </is>
+      </c>
+      <c r="S394" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="T394" t="inlineStr">
+        <is>
+          <t>369</t>
         </is>
       </c>
     </row>
@@ -67525,7 +67919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C187"/>
+  <dimension ref="A1:C183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -70074,12 +70468,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>213</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>AIN (none) (San Diego): no roll values from any source</t>
+          <t>AIN (none) (Sacramento): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70091,12 +70485,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>213</t>
+          <t>215</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>AIN (none) (Sacramento): no roll values from any source</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70108,7 +70502,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>215</t>
+          <t>221</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -70125,12 +70519,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>216</t>
+          <t>222</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>AIN (none) (San Diego): no roll values from any source</t>
+          <t>AIN (none) (Alameda): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70142,12 +70536,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>217</t>
+          <t>223</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN (none) (Alameda): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70159,12 +70553,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>221</t>
+          <t>226</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN (none) (Contra Costa): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70176,12 +70570,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>229</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>AIN (none) (Alameda): no roll values from any source</t>
+          <t>AIN (none) (San Diego): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70193,12 +70587,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>223</t>
+          <t>235</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>AIN (none) (Alameda): no roll values from any source</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70210,12 +70604,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>236</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>AIN (none) (Contra Costa): no roll values from any source</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70227,12 +70621,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>189</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>AIN (none) (San Diego): no roll values from any source</t>
+          <t>AIN 46745075 (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70244,12 +70638,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>235</t>
+          <t>189</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN 46745074 (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70261,12 +70655,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>189</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN 46745073 (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70278,12 +70672,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>198</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>AIN 46745075 (Santa Clara): no roll values from any source</t>
+          <t>AIN (none) (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70295,12 +70689,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>202</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>AIN 46745074 (Santa Clara): no roll values from any source</t>
+          <t>AIN (none) (Santa Cruz): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70312,12 +70706,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>AIN 46745073 (Santa Clara): no roll values from any source</t>
+          <t>AIN 128101150 (Solano): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70329,12 +70723,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>198</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>AIN (none) (Santa Clara): no roll values from any source</t>
+          <t>AIN 128101050 (Solano): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70346,97 +70740,97 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>202</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>AIN (none) (Santa Cruz): no roll values from any source</t>
+          <t>AIN 128105060 (Solano): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>missing-parcels</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>238</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>AIN 128101150 (Solano): no roll values from any source</t>
+          <t>Heritage Park Apartments Livermore (Alameda): operative authorization, not dead, no parcels anywhere in its property group</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>143/147</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>AIN 128101050 (Solano): no roll values from any source</t>
+          <t>AIN 41416654 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>182/76</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>AIN 128105060 (Solano): no roll values from any source</t>
+          <t>AIN 5036031006 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>missing-parcels</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>238</t>
+          <t>200/218</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Heritage Park Apartments Livermore (Alameda): operative authorization, not dead, no parcels anywhere in its property group</t>
+          <t>AIN 5040021006 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>missing-parcels</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>369</t>
+          <t>130/179</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Verdana Apartments (San Diego): operative authorization, not dead, no parcels anywhere in its property group</t>
+          <t>AIN 5080006008 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70448,12 +70842,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>143/147</t>
+          <t>126/173</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>AIN 41416654 assigned to multiple projects</t>
+          <t>AIN 5094005005 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70465,12 +70859,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>182/76</t>
+          <t>127/174</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>AIN 5036031006 assigned to multiple projects</t>
+          <t>AIN 5094006003 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70482,12 +70876,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>200/218</t>
+          <t>122/165</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>AIN 5040021006 assigned to multiple projects</t>
+          <t>AIN 5094017020 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70499,12 +70893,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>130/179</t>
+          <t>124/169</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>AIN 5080006008 assigned to multiple projects</t>
+          <t>AIN 5094023025 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70516,12 +70910,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>126/173</t>
+          <t>128/175</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>AIN 5094005005 assigned to multiple projects</t>
+          <t>AIN 5502019004 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70533,12 +70927,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>127/174</t>
+          <t>125/170</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>AIN 5094006003 assigned to multiple projects</t>
+          <t>AIN 5503024012 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70550,12 +70944,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>122/165</t>
+          <t>129/177</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>AIN 5094017020 assigned to multiple projects</t>
+          <t>AIN 5517005016 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70567,12 +70961,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>124/169</t>
+          <t>121/162</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>AIN 5094023025 assigned to multiple projects</t>
+          <t>AIN 5518013024 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70584,12 +70978,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>128/175</t>
+          <t>123/168</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>AIN 5502019004 assigned to multiple projects</t>
+          <t>AIN 5518020021 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70601,12 +70995,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>125/170</t>
+          <t>135/220</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>AIN 5503024012 assigned to multiple projects</t>
+          <t>AIN 5518026004 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70618,12 +71012,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>129/177</t>
+          <t>10/132</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>AIN 5517005016 assigned to multiple projects</t>
+          <t>AIN 6020022027 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70635,78 +71029,10 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>121/162</t>
+          <t>152/181</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
-        <is>
-          <t>AIN 5518013024 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>123/168</t>
-        </is>
-      </c>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>AIN 5518020021 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>135/220</t>
-        </is>
-      </c>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>AIN 5518026004 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>10/132</t>
-        </is>
-      </c>
-      <c r="C186" t="inlineStr">
-        <is>
-          <t>AIN 6020022027 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>152/181</t>
-        </is>
-      </c>
-      <c r="C187" t="inlineStr">
         <is>
           <t>AIN 7157012017 assigned to multiple projects</t>
         </is>

</xml_diff>

<commit_message>
Assign Baird (6838 Baird Ave) and Hazelhurst (6142 Hazelhurst Pl) parcels
Manual picks by Drew; exact grant addresses (6840/6144) have no
county situs. Noted that assessor unit counts can't disambiguate
proposed projects. Both now valued from the LA parcel API.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -59454,6 +59454,21 @@
           <t>Baird Affordable Housing Apartments</t>
         </is>
       </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>2126022021</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>2126-022-021</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>6838 BAIRD AVE LOS ANGELES CA 91335</t>
+        </is>
+      </c>
       <c r="G270" t="inlineStr">
         <is>
           <t>False</t>
@@ -59461,7 +59476,57 @@
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>collaborator-sheet</t>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>Drew 2026-08-22: project aligns to 6838 Baird Ave (no 6840 situs exists). Assessor unit counts not usable to disambiguate — proposed project may differ.</t>
+        </is>
+      </c>
+      <c r="K270" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L270" s="2" t="inlineStr">
+        <is>
+          <t>833472</t>
+        </is>
+      </c>
+      <c r="M270" s="2" t="inlineStr">
+        <is>
+          <t>552040</t>
+        </is>
+      </c>
+      <c r="N270" s="2" t="inlineStr">
+        <is>
+          <t>1385512</t>
+        </is>
+      </c>
+      <c r="O270" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P270" s="2" t="inlineStr">
+        <is>
+          <t>1952</t>
+        </is>
+      </c>
+      <c r="Q270" s="2" t="inlineStr">
+        <is>
+          <t>Two Units</t>
+        </is>
+      </c>
+      <c r="R270" s="2" t="inlineStr">
+        <is>
+          <t>la-county-api</t>
+        </is>
+      </c>
+      <c r="S270" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="T270" t="inlineStr">
@@ -59642,6 +59707,21 @@
           <t>Hazelhurst Affordable Housing Apartments</t>
         </is>
       </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>2338006014</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>2338-006-014</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>6142 HAZELHURST PL LOS ANGELES CA 91606</t>
+        </is>
+      </c>
       <c r="G274" t="inlineStr">
         <is>
           <t>False</t>
@@ -59649,7 +59729,57 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>collaborator-sheet</t>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>Drew 2026-08-22: development parcel is 6142 (no 6144 situs exists). Assessor unit counts not usable to disambiguate — proposed project may differ.</t>
+        </is>
+      </c>
+      <c r="K274" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L274" s="2" t="inlineStr">
+        <is>
+          <t>688500</t>
+        </is>
+      </c>
+      <c r="M274" s="2" t="inlineStr">
+        <is>
+          <t>1224000</t>
+        </is>
+      </c>
+      <c r="N274" s="2" t="inlineStr">
+        <is>
+          <t>1912500</t>
+        </is>
+      </c>
+      <c r="O274" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P274" s="2" t="inlineStr">
+        <is>
+          <t>1952</t>
+        </is>
+      </c>
+      <c r="Q274" s="2" t="inlineStr">
+        <is>
+          <t>Two Units</t>
+        </is>
+      </c>
+      <c r="R274" s="2" t="inlineStr">
+        <is>
+          <t>la-county-api</t>
+        </is>
+      </c>
+      <c r="S274" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="T274" t="inlineStr">
@@ -67919,7 +68049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C183"/>
+  <dimension ref="A1:C181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -70332,12 +70462,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>201</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN (none) (Santa Barbara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70349,12 +70479,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>201</t>
+          <t>203</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>AIN (none) (Santa Barbara): no roll values from any source</t>
+          <t>AIN (none) (Sacramento): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70366,12 +70496,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>205</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>AIN (none) (Sacramento): no roll values from any source</t>
+          <t>AIN (none) (Contra Costa): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70383,7 +70513,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>206</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -70400,12 +70530,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>205</t>
+          <t>207</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>AIN (none) (Contra Costa): no roll values from any source</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70417,7 +70547,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>208</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -70434,12 +70564,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>213</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN (none) (Sacramento): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70451,7 +70581,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>208</t>
+          <t>215</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -70468,12 +70598,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>213</t>
+          <t>221</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>AIN (none) (Sacramento): no roll values from any source</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70485,12 +70615,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>215</t>
+          <t>222</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN (none) (Alameda): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70502,12 +70632,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>221</t>
+          <t>223</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN (none) (Alameda): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70519,12 +70649,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>226</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>AIN (none) (Alameda): no roll values from any source</t>
+          <t>AIN (none) (Contra Costa): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70536,12 +70666,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>223</t>
+          <t>229</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>AIN (none) (Alameda): no roll values from any source</t>
+          <t>AIN (none) (San Diego): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70553,12 +70683,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>235</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>AIN (none) (Contra Costa): no roll values from any source</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70570,12 +70700,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>236</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>AIN (none) (San Diego): no roll values from any source</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70587,12 +70717,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>235</t>
+          <t>189</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN 46745075 (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70604,12 +70734,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>189</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN 46745074 (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70626,7 +70756,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>AIN 46745075 (Santa Clara): no roll values from any source</t>
+          <t>AIN 46745073 (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70638,12 +70768,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>198</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>AIN 46745074 (Santa Clara): no roll values from any source</t>
+          <t>AIN (none) (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70655,12 +70785,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>202</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>AIN 46745073 (Santa Clara): no roll values from any source</t>
+          <t>AIN (none) (Santa Cruz): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70672,12 +70802,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>198</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>AIN (none) (Santa Clara): no roll values from any source</t>
+          <t>AIN 128101150 (Solano): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70689,12 +70819,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>202</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>AIN (none) (Santa Cruz): no roll values from any source</t>
+          <t>AIN 128101050 (Solano): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70711,58 +70841,58 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>AIN 128101150 (Solano): no roll values from any source</t>
+          <t>AIN 128105060 (Solano): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>missing-parcels</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>238</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>AIN 128101050 (Solano): no roll values from any source</t>
+          <t>Heritage Park Apartments Livermore (Alameda): operative authorization, not dead, no parcels anywhere in its property group</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>143/147</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>AIN 128105060 (Solano): no roll values from any source</t>
+          <t>AIN 41416654 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>missing-parcels</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>238</t>
+          <t>182/76</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Heritage Park Apartments Livermore (Alameda): operative authorization, not dead, no parcels anywhere in its property group</t>
+          <t>AIN 5036031006 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70774,12 +70904,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>143/147</t>
+          <t>200/218</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>AIN 41416654 assigned to multiple projects</t>
+          <t>AIN 5040021006 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70791,12 +70921,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>182/76</t>
+          <t>130/179</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>AIN 5036031006 assigned to multiple projects</t>
+          <t>AIN 5080006008 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70808,12 +70938,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>200/218</t>
+          <t>126/173</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>AIN 5040021006 assigned to multiple projects</t>
+          <t>AIN 5094005005 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70825,12 +70955,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>130/179</t>
+          <t>127/174</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>AIN 5080006008 assigned to multiple projects</t>
+          <t>AIN 5094006003 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70842,12 +70972,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>126/173</t>
+          <t>122/165</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>AIN 5094005005 assigned to multiple projects</t>
+          <t>AIN 5094017020 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70859,12 +70989,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>127/174</t>
+          <t>124/169</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>AIN 5094006003 assigned to multiple projects</t>
+          <t>AIN 5094023025 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70876,12 +71006,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>122/165</t>
+          <t>128/175</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>AIN 5094017020 assigned to multiple projects</t>
+          <t>AIN 5502019004 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70893,12 +71023,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>124/169</t>
+          <t>125/170</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>AIN 5094023025 assigned to multiple projects</t>
+          <t>AIN 5503024012 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70910,12 +71040,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>128/175</t>
+          <t>129/177</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>AIN 5502019004 assigned to multiple projects</t>
+          <t>AIN 5517005016 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70927,12 +71057,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>125/170</t>
+          <t>121/162</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>AIN 5503024012 assigned to multiple projects</t>
+          <t>AIN 5518013024 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70944,12 +71074,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>129/177</t>
+          <t>123/168</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>AIN 5517005016 assigned to multiple projects</t>
+          <t>AIN 5518020021 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70961,12 +71091,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>121/162</t>
+          <t>135/220</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>AIN 5518013024 assigned to multiple projects</t>
+          <t>AIN 5518026004 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70978,12 +71108,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>123/168</t>
+          <t>10/132</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>AIN 5518020021 assigned to multiple projects</t>
+          <t>AIN 6020022027 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70995,44 +71125,10 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>135/220</t>
+          <t>152/181</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
-        <is>
-          <t>AIN 5518026004 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>10/132</t>
-        </is>
-      </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>AIN 6020022027 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>152/181</t>
-        </is>
-      </c>
-      <c r="C183" t="inlineStr">
         <is>
           <t>AIN 7157012017 assigned to multiple projects</t>
         </is>

</xml_diff>

<commit_message>
Assign LA parcels for 3950 Ingraham, 511 Hoover, Banner Ave, Park Playa
Drew via assessor portal map view (new construction lots without
county situs records). Ingraham, Banner (situs 6223), and Park Playa
(parking-lot use, odd lot) valued from the 2026 roll; 511 Hoover's
AIN 5539028040 is not yet in the county parcel layer — values will
appear when the county publishes it.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -36151,7 +36151,7 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
@@ -60389,6 +60389,21 @@
           <t>511 Hoover Street Apartments</t>
         </is>
       </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>5539028040</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>5539-028-040</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>511 N HOOVER ST (no county situs; AIN from assessor portal map)</t>
+        </is>
+      </c>
       <c r="G285" t="inlineStr">
         <is>
           <t>False</t>
@@ -60396,7 +60411,12 @@
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>collaborator-sheet</t>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>Drew 2026-08-22 via assessor portal map view; new construction, situs not yet keyed.</t>
         </is>
       </c>
       <c r="T285" t="inlineStr">
@@ -60886,6 +60906,21 @@
           <t>Banner Avenue Apartments</t>
         </is>
       </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>5534006026</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>5534-006-026</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>6219 BANNER AVE (no county situs; AIN from assessor portal map)</t>
+        </is>
+      </c>
       <c r="G291" t="inlineStr">
         <is>
           <t>False</t>
@@ -60893,7 +60928,57 @@
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>collaborator-sheet</t>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>Drew 2026-08-22 via assessor portal map view; Banner Ave parcels not situs-keyed.</t>
+        </is>
+      </c>
+      <c r="K291" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L291" s="2" t="inlineStr">
+        <is>
+          <t>3459330</t>
+        </is>
+      </c>
+      <c r="M291" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N291" s="2" t="inlineStr">
+        <is>
+          <t>3459330</t>
+        </is>
+      </c>
+      <c r="O291" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P291" s="2" t="inlineStr">
+        <is>
+          <t>0000</t>
+        </is>
+      </c>
+      <c r="Q291" s="2" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="R291" s="2" t="inlineStr">
+        <is>
+          <t>la-county-api</t>
+        </is>
+      </c>
+      <c r="S291" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="T291" t="inlineStr">
@@ -61779,6 +61864,21 @@
           <t>3950 Ingraham Apartments</t>
         </is>
       </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>5092029007</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>5092-029-007</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>3950 INGRAHAM ST LOS ANGELES CA 90005</t>
+        </is>
+      </c>
       <c r="G305" t="inlineStr">
         <is>
           <t>False</t>
@@ -61786,7 +61886,52 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>collaborator-sheet</t>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>Drew confirmed 2026-08-22: staff report "3950 W. Ingraham" has spurious W; single Ingraham St in LA. Pre-development "Four Units" lot.</t>
+        </is>
+      </c>
+      <c r="K305" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L305" s="2" t="inlineStr">
+        <is>
+          <t>1237872</t>
+        </is>
+      </c>
+      <c r="M305" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N305" s="2" t="inlineStr">
+        <is>
+          <t>1237872</t>
+        </is>
+      </c>
+      <c r="O305" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q305" s="2" t="inlineStr">
+        <is>
+          <t>Four Units (Any Combination)</t>
+        </is>
+      </c>
+      <c r="R305" s="2" t="inlineStr">
+        <is>
+          <t>la-county-api</t>
+        </is>
+      </c>
+      <c r="S305" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="T305" t="inlineStr">
@@ -61811,6 +61956,21 @@
           <t>Park Playa Apartments</t>
         </is>
       </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>4211011047</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>4211-011-047</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>6985 S CENTINELA AVE (no county situs; AIN from assessor portal map)</t>
+        </is>
+      </c>
       <c r="G306" t="inlineStr">
         <is>
           <t>False</t>
@@ -61818,7 +61978,52 @@
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>collaborator-sheet</t>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>Drew 2026-08-22 via assessor portal map view; odd lot shape, best-fit parcel.</t>
+        </is>
+      </c>
+      <c r="K306" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L306" s="2" t="inlineStr">
+        <is>
+          <t>5234013</t>
+        </is>
+      </c>
+      <c r="M306" s="2" t="inlineStr">
+        <is>
+          <t>28443</t>
+        </is>
+      </c>
+      <c r="N306" s="2" t="inlineStr">
+        <is>
+          <t>5262456</t>
+        </is>
+      </c>
+      <c r="O306" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q306" s="2" t="inlineStr">
+        <is>
+          <t>Parking Lots (Commercial Use Properties)</t>
+        </is>
+      </c>
+      <c r="R306" s="2" t="inlineStr">
+        <is>
+          <t>la-county-api</t>
+        </is>
+      </c>
+      <c r="S306" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="T306" t="inlineStr">
@@ -68049,7 +68254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C181"/>
+  <dimension ref="A1:C178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -70586,7 +70791,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN 5539028040 (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70598,12 +70803,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>221</t>
+          <t>222</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN (none) (Alameda): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70615,7 +70820,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>223</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -70632,12 +70837,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>223</t>
+          <t>226</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>AIN (none) (Alameda): no roll values from any source</t>
+          <t>AIN (none) (Contra Costa): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70649,12 +70854,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>229</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>AIN (none) (Contra Costa): no roll values from any source</t>
+          <t>AIN (none) (San Diego): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70666,12 +70871,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>189</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>AIN (none) (San Diego): no roll values from any source</t>
+          <t>AIN 46745075 (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70683,12 +70888,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>235</t>
+          <t>189</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN 46745074 (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70700,12 +70905,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>189</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN 46745073 (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70717,12 +70922,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>198</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>AIN 46745075 (Santa Clara): no roll values from any source</t>
+          <t>AIN (none) (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70734,12 +70939,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>202</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>AIN 46745074 (Santa Clara): no roll values from any source</t>
+          <t>AIN (none) (Santa Cruz): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70751,12 +70956,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>AIN 46745073 (Santa Clara): no roll values from any source</t>
+          <t>AIN 128101150 (Solano): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70768,12 +70973,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>198</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>AIN (none) (Santa Clara): no roll values from any source</t>
+          <t>AIN 128101050 (Solano): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70785,80 +70990,80 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>202</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>AIN (none) (Santa Cruz): no roll values from any source</t>
+          <t>AIN 128105060 (Solano): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>missing-parcels</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>238</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>AIN 128101150 (Solano): no roll values from any source</t>
+          <t>Heritage Park Apartments Livermore (Alameda): operative authorization, not dead, no parcels anywhere in its property group</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>143/147</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>AIN 128101050 (Solano): no roll values from any source</t>
+          <t>AIN 41416654 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>182/76</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>AIN 128105060 (Solano): no roll values from any source</t>
+          <t>AIN 5036031006 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>missing-parcels</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>238</t>
+          <t>200/218</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Heritage Park Apartments Livermore (Alameda): operative authorization, not dead, no parcels anywhere in its property group</t>
+          <t>AIN 5040021006 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70870,12 +71075,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>143/147</t>
+          <t>130/179</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>AIN 41416654 assigned to multiple projects</t>
+          <t>AIN 5080006008 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70887,12 +71092,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>182/76</t>
+          <t>126/173</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>AIN 5036031006 assigned to multiple projects</t>
+          <t>AIN 5094005005 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70904,12 +71109,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>200/218</t>
+          <t>127/174</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>AIN 5040021006 assigned to multiple projects</t>
+          <t>AIN 5094006003 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70921,12 +71126,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>130/179</t>
+          <t>122/165</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>AIN 5080006008 assigned to multiple projects</t>
+          <t>AIN 5094017020 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70938,12 +71143,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>126/173</t>
+          <t>124/169</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>AIN 5094005005 assigned to multiple projects</t>
+          <t>AIN 5094023025 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70955,12 +71160,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>127/174</t>
+          <t>128/175</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>AIN 5094006003 assigned to multiple projects</t>
+          <t>AIN 5502019004 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70972,12 +71177,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>122/165</t>
+          <t>125/170</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>AIN 5094017020 assigned to multiple projects</t>
+          <t>AIN 5503024012 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -70989,12 +71194,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>124/169</t>
+          <t>129/177</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>AIN 5094023025 assigned to multiple projects</t>
+          <t>AIN 5517005016 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -71006,12 +71211,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>128/175</t>
+          <t>121/162</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>AIN 5502019004 assigned to multiple projects</t>
+          <t>AIN 5518013024 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -71023,12 +71228,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>125/170</t>
+          <t>123/168</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>AIN 5503024012 assigned to multiple projects</t>
+          <t>AIN 5518020021 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -71040,12 +71245,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>129/177</t>
+          <t>135/220</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>AIN 5517005016 assigned to multiple projects</t>
+          <t>AIN 5518026004 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -71057,12 +71262,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>121/162</t>
+          <t>10/132</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>AIN 5518013024 assigned to multiple projects</t>
+          <t>AIN 6020022027 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -71074,61 +71279,10 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>123/168</t>
+          <t>152/181</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
-        <is>
-          <t>AIN 5518020021 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>135/220</t>
-        </is>
-      </c>
-      <c r="C179" t="inlineStr">
-        <is>
-          <t>AIN 5518026004 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>10/132</t>
-        </is>
-      </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>AIN 6020022027 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>152/181</t>
-        </is>
-      </c>
-      <c r="C181" t="inlineStr">
         <is>
           <t>AIN 7157012017 assigned to multiple projects</t>
         </is>

</xml_diff>

<commit_message>
Manual parcel values: Santa Cruz, Sacramento, Alameda (Drew, assessor portals)
La Posada 9.78M; Sierra Village 8.88M; Bent Tree 15.69M; Bayfair
11.14M; 2121 Wood St 71.93M with a 56.40M welfare exemption on the
roll; Heritage Park Livermore 47.39M with a 19.52M exemption.
Coliseum Connections (41416654) shows $0 assessed at the county —
recorded as such. All roll year 2026, source manual-repo-edit.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -36139,7 +36139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T394"/>
+  <dimension ref="A1:T395"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -36151,7 +36151,7 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
@@ -54924,6 +54924,26 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="N215" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R215" t="inlineStr">
+        <is>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
       <c r="T215" t="inlineStr">
         <is>
           <t>147</t>
@@ -59675,6 +59695,21 @@
           <t>Bent Tree Apartments</t>
         </is>
       </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>21900420330000</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>219-0042-033-0000</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>4350 GALBRATH DR SACRAMENTO CA 95842</t>
+        </is>
+      </c>
       <c r="G273" t="inlineStr">
         <is>
           <t>False</t>
@@ -59682,7 +59717,32 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>collaborator-sheet</t>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>Drew 2026-08-22 via Sacramento assessor lookup</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="N273" t="inlineStr">
+        <is>
+          <t>15693765</t>
+        </is>
+      </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R273" t="inlineStr">
+        <is>
+          <t>manual-repo-edit</t>
         </is>
       </c>
       <c r="T273" t="inlineStr">
@@ -60265,6 +60325,21 @@
           <t>Sierra Village</t>
         </is>
       </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>22800420320000</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>228-0042-032-0000</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>5416 JACKSON ST NORTH HIGHLANDS CA 95660</t>
+        </is>
+      </c>
       <c r="G283" t="inlineStr">
         <is>
           <t>False</t>
@@ -60272,7 +60347,32 @@
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>collaborator-sheet</t>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>Drew 2026-08-22 via Sacramento assessor lookup</t>
+        </is>
+      </c>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="N283" t="inlineStr">
+        <is>
+          <t>8878476</t>
+        </is>
+      </c>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R283" t="inlineStr">
+        <is>
+          <t>manual-repo-edit</t>
         </is>
       </c>
       <c r="T283" t="inlineStr">
@@ -61003,6 +61103,21 @@
           <t>Bayfair Apartments</t>
         </is>
       </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>80C49562</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>80C-495-6-2</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>16077 ASHLAND AVE SAN LORENZO CA 94580</t>
+        </is>
+      </c>
       <c r="G292" t="inlineStr">
         <is>
           <t>False</t>
@@ -61010,7 +61125,32 @@
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>collaborator-sheet</t>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>Drew 2026-08-22 via Alameda assessor lookup</t>
+        </is>
+      </c>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="N292" t="inlineStr">
+        <is>
+          <t>11141147</t>
+        </is>
+      </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R292" t="inlineStr">
+        <is>
+          <t>manual-repo-edit</t>
         </is>
       </c>
       <c r="T292" t="inlineStr">
@@ -61035,6 +61175,21 @@
           <t>2121 Wood St</t>
         </is>
       </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>1831016</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>18-310-16</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>2121 WOOD ST OAKLAND CA 94607</t>
+        </is>
+      </c>
       <c r="G293" t="inlineStr">
         <is>
           <t>False</t>
@@ -61042,7 +61197,32 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>collaborator-sheet</t>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>Drew 2026-08-22 via Alameda assessor lookup</t>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="N293" t="inlineStr">
+        <is>
+          <t>71934357</t>
+        </is>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>56403868</t>
+        </is>
+      </c>
+      <c r="R293" t="inlineStr">
+        <is>
+          <t>manual-repo-edit</t>
         </is>
       </c>
       <c r="T293" t="inlineStr">
@@ -63118,6 +63298,16 @@
           <t>La Posada Apartments</t>
         </is>
       </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>01125105</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>011-251-05</t>
+        </is>
+      </c>
       <c r="G327" t="inlineStr">
         <is>
           <t>False</t>
@@ -63125,7 +63315,32 @@
       </c>
       <c r="H327" t="inlineStr">
         <is>
-          <t>collaborator-sheet</t>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>Drew 2026-08-22 via Santa Cruz assessor lookup, 609 Frederick St</t>
+        </is>
+      </c>
+      <c r="K327" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="N327" t="inlineStr">
+        <is>
+          <t>9776112</t>
+        </is>
+      </c>
+      <c r="O327" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R327" t="inlineStr">
+        <is>
+          <t>manual-repo-edit</t>
         </is>
       </c>
       <c r="T327" t="inlineStr">
@@ -68240,6 +68455,78 @@
       <c r="T394" t="inlineStr">
         <is>
           <t>369</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>238</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Alameda</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Heritage Park Apartments Livermore</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>9917523</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>99-175-23</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>900 E STANLEY BLVD LIVERMORE CA 94550</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>Drew 2026-08-22 via Alameda assessor lookup</t>
+        </is>
+      </c>
+      <c r="K395" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="N395" t="inlineStr">
+        <is>
+          <t>47387387</t>
+        </is>
+      </c>
+      <c r="O395" t="inlineStr">
+        <is>
+          <t>19523603</t>
+        </is>
+      </c>
+      <c r="R395" t="inlineStr">
+        <is>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="T395" t="inlineStr">
+        <is>
+          <t>238</t>
         </is>
       </c>
     </row>
@@ -68254,7 +68541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C178"/>
+  <dimension ref="A1:C171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -70582,12 +70869,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>158</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>AIN 41416654 (Alameda): no roll values from any source</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70599,12 +70886,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>182</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN 5036031006 (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70616,12 +70903,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>182</t>
+          <t>196</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>AIN 5036031006 (Los Angeles): no roll values from any source</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70633,7 +70920,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>197</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -70650,12 +70937,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>197</t>
+          <t>201</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN (none) (Santa Barbara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70667,12 +70954,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>201</t>
+          <t>205</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>AIN (none) (Santa Barbara): no roll values from any source</t>
+          <t>AIN (none) (Contra Costa): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70684,12 +70971,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>206</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>AIN (none) (Sacramento): no roll values from any source</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70701,12 +70988,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>205</t>
+          <t>207</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>AIN (none) (Contra Costa): no roll values from any source</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70718,7 +71005,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>208</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -70735,12 +71022,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>215</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN 5539028040 (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70752,12 +71039,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>208</t>
+          <t>226</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN (none) (Contra Costa): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70769,12 +71056,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>213</t>
+          <t>229</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>AIN (none) (Sacramento): no roll values from any source</t>
+          <t>AIN (none) (San Diego): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70786,12 +71073,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>215</t>
+          <t>189</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>AIN 5539028040 (Los Angeles): no roll values from any source</t>
+          <t>AIN 46745075 (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70803,12 +71090,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>189</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>AIN (none) (Alameda): no roll values from any source</t>
+          <t>AIN 46745074 (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70820,12 +71107,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>223</t>
+          <t>189</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>AIN (none) (Alameda): no roll values from any source</t>
+          <t>AIN 46745073 (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70837,12 +71124,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>198</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>AIN (none) (Contra Costa): no roll values from any source</t>
+          <t>AIN (none) (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70854,12 +71141,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>AIN (none) (San Diego): no roll values from any source</t>
+          <t>AIN 128101150 (Solano): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70871,12 +71158,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>AIN 46745075 (Santa Clara): no roll values from any source</t>
+          <t>AIN 128101050 (Solano): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -70888,131 +71175,131 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>AIN 46745074 (Santa Clara): no roll values from any source</t>
+          <t>AIN 128105060 (Solano): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>143/147</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>AIN 46745073 (Santa Clara): no roll values from any source</t>
+          <t>AIN 41416654 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>198</t>
+          <t>182/76</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>AIN (none) (Santa Clara): no roll values from any source</t>
+          <t>AIN 5036031006 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>202</t>
+          <t>200/218</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>AIN (none) (Santa Cruz): no roll values from any source</t>
+          <t>AIN 5040021006 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>130/179</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>AIN 128101150 (Solano): no roll values from any source</t>
+          <t>AIN 5080006008 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>126/173</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>AIN 128101050 (Solano): no roll values from any source</t>
+          <t>AIN 5094005005 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>127/174</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>AIN 128105060 (Solano): no roll values from any source</t>
+          <t>AIN 5094006003 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>missing-parcels</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>238</t>
+          <t>122/165</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Heritage Park Apartments Livermore (Alameda): operative authorization, not dead, no parcels anywhere in its property group</t>
+          <t>AIN 5094017020 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -71024,12 +71311,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>143/147</t>
+          <t>124/169</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>AIN 41416654 assigned to multiple projects</t>
+          <t>AIN 5094023025 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -71041,12 +71328,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>182/76</t>
+          <t>128/175</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>AIN 5036031006 assigned to multiple projects</t>
+          <t>AIN 5502019004 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -71058,12 +71345,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>200/218</t>
+          <t>125/170</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>AIN 5040021006 assigned to multiple projects</t>
+          <t>AIN 5503024012 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -71075,12 +71362,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>130/179</t>
+          <t>129/177</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>AIN 5080006008 assigned to multiple projects</t>
+          <t>AIN 5517005016 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -71092,12 +71379,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>126/173</t>
+          <t>121/162</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>AIN 5094005005 assigned to multiple projects</t>
+          <t>AIN 5518013024 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -71109,12 +71396,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>127/174</t>
+          <t>123/168</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>AIN 5094006003 assigned to multiple projects</t>
+          <t>AIN 5518020021 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -71126,12 +71413,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>122/165</t>
+          <t>135/220</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>AIN 5094017020 assigned to multiple projects</t>
+          <t>AIN 5518026004 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -71143,12 +71430,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>124/169</t>
+          <t>10/132</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>AIN 5094023025 assigned to multiple projects</t>
+          <t>AIN 6020022027 assigned to multiple projects</t>
         </is>
       </c>
     </row>
@@ -71160,129 +71447,10 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>128/175</t>
+          <t>152/181</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
-        <is>
-          <t>AIN 5502019004 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>125/170</t>
-        </is>
-      </c>
-      <c r="C172" t="inlineStr">
-        <is>
-          <t>AIN 5503024012 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>129/177</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>AIN 5517005016 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>121/162</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>AIN 5518013024 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>123/168</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>AIN 5518020021 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>135/220</t>
-        </is>
-      </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>AIN 5518026004 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>10/132</t>
-        </is>
-      </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>AIN 6020022027 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>152/181</t>
-        </is>
-      </c>
-      <c r="C178" t="inlineStr">
         <is>
           <t>AIN 7157012017 assigned to multiple projects</t>
         </is>

</xml_diff>

<commit_message>
Montessa common-area parcels recorded as $0 (government-owned)
All three quiet Montessa AINs (0128101050/1150, 0128105060) are use
code 9800 Governmental & Miscellaneous, Government Owned=YS, $0
values, no site address — dedicated common-area lots, correctly
non-taxable. Bent Tree exemption-free confirmed by Drew.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -63326,6 +63326,31 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>Government-owned common-area parcel (use code 9800, $0 values) — Drew via Solano GIS 2026-08-22</t>
+        </is>
+      </c>
+      <c r="K326" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="N326" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O326" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R326" t="inlineStr">
+        <is>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
       <c r="T326" t="inlineStr">
         <is>
           <t>16</t>
@@ -64061,6 +64086,31 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>Government-owned common-area parcel (use code 9800, Government Owned=YS, no site address, $0 values) — Drew via Solano GIS 2026-08-22</t>
+        </is>
+      </c>
+      <c r="K336" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="N336" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O336" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R336" t="inlineStr">
+        <is>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
       <c r="T336" t="inlineStr">
         <is>
           <t>16</t>
@@ -67412,6 +67462,31 @@
       <c r="H380" t="inlineStr">
         <is>
           <t>collaborator-sheet</t>
+        </is>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>Government-owned common-area parcel (use code 9800, $0 values) — Drew via Solano GIS 2026-08-22</t>
+        </is>
+      </c>
+      <c r="K380" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="N380" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O380" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R380" t="inlineStr">
+        <is>
+          <t>manual-repo-edit</t>
         </is>
       </c>
       <c r="T380" t="inlineStr">
@@ -71043,7 +71118,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -71053,14 +71128,14 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>AIN 128101150 (Solano): no roll values from any source</t>
+          <t>AIN 128101150 (Solano) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -71070,14 +71145,14 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>AIN 128101050 (Solano): no roll values from any source</t>
+          <t>AIN 128101050 (Solano) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -71087,7 +71162,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>AIN 128105060 (Solano): no roll values from any source</t>
+          <t>AIN 128105060 (Solano) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plumb restricted_units through extraction; prune redundant overrides
The staff-report parser always extracted restricted unit counts but
ExtractedGrant never carried the field, so the dataset's
restricted_units came entirely from collaborator overrides. Now
generated at 93% coverage for CMFA; 182 overrides that matched the
newly generated values were dropped, keeping 50 (12 genuine
corrections + rows with no generated value).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -727,7 +727,7 @@
           <t>24</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>24</t>
         </is>
@@ -774,7 +774,7 @@
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -849,7 +849,7 @@
           <t>15</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="R3" s="2" t="inlineStr">
         <is>
           <t>14</t>
         </is>
@@ -901,7 +901,7 @@
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>built:collaborator-sheet; scc_filed:collaborator-sheet; investor_1:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>built:collaborator-sheet; scc_filed:collaborator-sheet; investor_1:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
           <t>48</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>48</t>
         </is>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1327,7 @@
           <t>32</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="R7" s="2" t="inlineStr">
         <is>
           <t>13</t>
         </is>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>manual_status:collaborator-sheet; city:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>manual_status:collaborator-sheet; city:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -1444,7 +1444,7 @@
           <t>61</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="R8" s="2" t="inlineStr">
         <is>
           <t>61</t>
         </is>
@@ -1491,7 +1491,7 @@
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>leasing_link:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>leasing_link:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1566,7 @@
           <t>147</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="R9" s="2" t="inlineStr">
         <is>
           <t>147</t>
         </is>
@@ -1613,7 +1613,7 @@
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -1693,7 +1693,7 @@
           <t>227</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="R10" s="2" t="inlineStr">
         <is>
           <t>227</t>
         </is>
@@ -1735,7 +1735,7 @@
       </c>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_2:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -1927,7 +1927,7 @@
           <t>166</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="R12" s="2" t="inlineStr">
         <is>
           <t>166</t>
         </is>
@@ -1979,7 +1979,7 @@
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; entity:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
           <t>66</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
+      <c r="R14" s="2" t="inlineStr">
         <is>
           <t>27</t>
         </is>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_2:collaborator-sheet; manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -2308,7 +2308,7 @@
           <t>89</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
+      <c r="R15" s="2" t="inlineStr">
         <is>
           <t>40</t>
         </is>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>leasing_link:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>leasing_link:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
           <t>69</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
+      <c r="R16" s="2" t="inlineStr">
         <is>
           <t>69</t>
         </is>
@@ -2487,7 +2487,7 @@
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>built:collaborator-sheet; manual_status:collaborator-sheet; entity:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>built:collaborator-sheet; manual_status:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -2562,7 +2562,7 @@
           <t>169</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="R17" s="2" t="inlineStr">
         <is>
           <t>58</t>
         </is>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; entity:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2689,7 @@
           <t>111</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="R18" s="2" t="inlineStr">
         <is>
           <t>111</t>
         </is>
@@ -2746,7 +2746,7 @@
       </c>
       <c r="AH18" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; built:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; built:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2826,7 @@
           <t>103</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="R19" s="2" t="inlineStr">
         <is>
           <t>102</t>
         </is>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; built:collaborator-sheet; scc_filed:collaborator-sheet; city:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>investor_2:collaborator-sheet; built:collaborator-sheet; scc_filed:collaborator-sheet; city:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -2958,7 +2958,7 @@
           <t>160</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr">
+      <c r="R20" s="2" t="inlineStr">
         <is>
           <t>160</t>
         </is>
@@ -3010,7 +3010,7 @@
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; built:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_2:collaborator-sheet; built:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -3085,7 +3085,7 @@
           <t>58</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
+      <c r="R21" s="2" t="inlineStr">
         <is>
           <t>58</t>
         </is>
@@ -3142,7 +3142,7 @@
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>acquisition_price_m:collaborator-sheet; acquisition_date:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>acquisition_price_m:collaborator-sheet; acquisition_date:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3217,7 @@
           <t>52</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
+      <c r="R22" s="2" t="inlineStr">
         <is>
           <t>52</t>
         </is>
@@ -3274,7 +3274,7 @@
       </c>
       <c r="AH22" t="inlineStr">
         <is>
-          <t>acquisition_price_m:collaborator-sheet; acquisition_date:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>acquisition_price_m:collaborator-sheet; acquisition_date:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -3349,7 +3349,7 @@
           <t>225</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr">
+      <c r="R23" s="2" t="inlineStr">
         <is>
           <t>225</t>
         </is>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>built:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>built:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -3476,7 +3476,7 @@
           <t>74</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
+      <c r="R24" s="2" t="inlineStr">
         <is>
           <t>74</t>
         </is>
@@ -3523,7 +3523,7 @@
       </c>
       <c r="AH24" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -3593,7 +3593,7 @@
           <t>25</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr">
+      <c r="R25" s="2" t="inlineStr">
         <is>
           <t>24</t>
         </is>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>scc_filed:collaborator-sheet; resolution:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>scc_filed:collaborator-sheet; resolution:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -3710,7 +3710,7 @@
           <t>29</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr">
+      <c r="R26" s="2" t="inlineStr">
         <is>
           <t>28</t>
         </is>
@@ -3757,7 +3757,7 @@
       </c>
       <c r="AH26" t="inlineStr">
         <is>
-          <t>scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -3832,7 +3832,7 @@
           <t>93</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr">
+      <c r="R27" s="2" t="inlineStr">
         <is>
           <t>93</t>
         </is>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="AH27" t="inlineStr">
         <is>
-          <t>built:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>built:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -3959,7 +3959,7 @@
           <t>52</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr">
+      <c r="R28" s="2" t="inlineStr">
         <is>
           <t>32</t>
         </is>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="AH28" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; built:collaborator-sheet; acquisition_price_m:collaborator-sheet; acquisition_date:collaborator-sheet; link:collaborator-sheet; scc_filed:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; built:collaborator-sheet; acquisition_price_m:collaborator-sheet; acquisition_date:collaborator-sheet; link:collaborator-sheet; scc_filed:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
           <t>72</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr">
+      <c r="R29" s="2" t="inlineStr">
         <is>
           <t>49</t>
         </is>
@@ -4153,7 +4153,7 @@
       </c>
       <c r="AH29" t="inlineStr">
         <is>
-          <t>scc_filed:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>scc_filed:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -4228,7 +4228,7 @@
           <t>48</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr">
+      <c r="R30" s="2" t="inlineStr">
         <is>
           <t>29</t>
         </is>
@@ -4275,7 +4275,7 @@
       </c>
       <c r="AH30" t="inlineStr">
         <is>
-          <t>scc_filed:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>scc_filed:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -4350,7 +4350,7 @@
           <t>26</t>
         </is>
       </c>
-      <c r="R31" t="inlineStr">
+      <c r="R31" s="2" t="inlineStr">
         <is>
           <t>25</t>
         </is>
@@ -4402,7 +4402,7 @@
       </c>
       <c r="AH31" t="inlineStr">
         <is>
-          <t>built:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>built:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -4477,7 +4477,7 @@
           <t>26</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr">
+      <c r="R32" s="2" t="inlineStr">
         <is>
           <t>25</t>
         </is>
@@ -4534,7 +4534,7 @@
       </c>
       <c r="AH32" t="inlineStr">
         <is>
-          <t>acquisition_price_m:collaborator-sheet; acquisition_date:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>acquisition_price_m:collaborator-sheet; acquisition_date:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -4609,7 +4609,7 @@
           <t>165</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr">
+      <c r="R33" s="2" t="inlineStr">
         <is>
           <t>98</t>
         </is>
@@ -4661,7 +4661,7 @@
       </c>
       <c r="AH33" t="inlineStr">
         <is>
-          <t>built:collaborator-sheet; scc_filed:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>built:collaborator-sheet; scc_filed:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -4746,7 +4746,7 @@
           <t>79</t>
         </is>
       </c>
-      <c r="R34" t="inlineStr">
+      <c r="R34" s="2" t="inlineStr">
         <is>
           <t>48</t>
         </is>
@@ -4793,7 +4793,7 @@
       </c>
       <c r="AH34" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -4868,7 +4868,7 @@
           <t>41</t>
         </is>
       </c>
-      <c r="R35" t="inlineStr">
+      <c r="R35" s="2" t="inlineStr">
         <is>
           <t>41</t>
         </is>
@@ -4915,7 +4915,7 @@
       </c>
       <c r="AH35" t="inlineStr">
         <is>
-          <t>scc_filed:collaborator-sheet; city:collaborator-sheet; county:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>scc_filed:collaborator-sheet; city:collaborator-sheet; county:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -4985,7 +4985,7 @@
           <t>104</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr">
+      <c r="R36" s="2" t="inlineStr">
         <is>
           <t>104</t>
         </is>
@@ -5032,7 +5032,7 @@
       </c>
       <c r="AH36" t="inlineStr">
         <is>
-          <t>scc_filed:collaborator-sheet; city:collaborator-sheet; resolution:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>scc_filed:collaborator-sheet; city:collaborator-sheet; resolution:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -5102,7 +5102,7 @@
           <t>80</t>
         </is>
       </c>
-      <c r="R37" t="inlineStr">
+      <c r="R37" s="2" t="inlineStr">
         <is>
           <t>80</t>
         </is>
@@ -5150,7 +5150,7 @@
       </c>
       <c r="AH37" t="inlineStr">
         <is>
-          <t>scc_filed:collaborator-sheet; resolution:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>scc_filed:collaborator-sheet; resolution:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
           <t>53</t>
         </is>
       </c>
-      <c r="R38" t="inlineStr">
+      <c r="R38" s="2" t="inlineStr">
         <is>
           <t>53</t>
         </is>
@@ -5272,7 +5272,7 @@
       </c>
       <c r="AH38" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; property_name:collaborator-sheet; resolution:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; property_name:collaborator-sheet; resolution:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -5347,7 +5347,7 @@
           <t>236</t>
         </is>
       </c>
-      <c r="R39" t="inlineStr">
+      <c r="R39" s="2" t="inlineStr">
         <is>
           <t>236</t>
         </is>
@@ -5404,7 +5404,7 @@
       </c>
       <c r="AH39" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; built:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; built:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -5474,7 +5474,7 @@
           <t>66</t>
         </is>
       </c>
-      <c r="R40" t="inlineStr">
+      <c r="R40" s="2" t="inlineStr">
         <is>
           <t>51</t>
         </is>
@@ -5526,7 +5526,7 @@
       </c>
       <c r="AH40" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; resolution:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; resolution:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -5606,7 +5606,7 @@
           <t>68</t>
         </is>
       </c>
-      <c r="R41" t="inlineStr">
+      <c r="R41" s="2" t="inlineStr">
         <is>
           <t>14</t>
         </is>
@@ -5653,7 +5653,7 @@
       </c>
       <c r="AH41" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; resolution:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; resolution:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -5728,7 +5728,7 @@
           <t>188</t>
         </is>
       </c>
-      <c r="R42" t="inlineStr">
+      <c r="R42" s="2" t="inlineStr">
         <is>
           <t>111</t>
         </is>
@@ -5775,7 +5775,7 @@
       </c>
       <c r="AH42" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -5855,7 +5855,7 @@
           <t>90</t>
         </is>
       </c>
-      <c r="R43" t="inlineStr">
+      <c r="R43" s="2" t="inlineStr">
         <is>
           <t>71</t>
         </is>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="AH43" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -5987,7 +5987,7 @@
           <t>99</t>
         </is>
       </c>
-      <c r="R44" t="inlineStr">
+      <c r="R44" s="2" t="inlineStr">
         <is>
           <t>99</t>
         </is>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="AH44" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -6109,7 +6109,7 @@
           <t>41</t>
         </is>
       </c>
-      <c r="R45" t="inlineStr">
+      <c r="R45" s="2" t="inlineStr">
         <is>
           <t>40</t>
         </is>
@@ -6161,7 +6161,7 @@
       </c>
       <c r="AH45" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; nonprofit_partner:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -6241,7 +6241,7 @@
           <t>406</t>
         </is>
       </c>
-      <c r="R46" t="inlineStr">
+      <c r="R46" s="2" t="inlineStr">
         <is>
           <t>406</t>
         </is>
@@ -6293,7 +6293,7 @@
       </c>
       <c r="AH46" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -6373,7 +6373,7 @@
           <t>53</t>
         </is>
       </c>
-      <c r="R47" t="inlineStr">
+      <c r="R47" s="2" t="inlineStr">
         <is>
           <t>53</t>
         </is>
@@ -6420,7 +6420,7 @@
       </c>
       <c r="AH47" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -6495,7 +6495,7 @@
           <t>488</t>
         </is>
       </c>
-      <c r="R48" t="inlineStr">
+      <c r="R48" s="2" t="inlineStr">
         <is>
           <t>483</t>
         </is>
@@ -6547,7 +6547,7 @@
       </c>
       <c r="AH48" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -6627,7 +6627,7 @@
           <t>697</t>
         </is>
       </c>
-      <c r="R49" t="inlineStr">
+      <c r="R49" s="2" t="inlineStr">
         <is>
           <t>697</t>
         </is>
@@ -6679,7 +6679,7 @@
       </c>
       <c r="AH49" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; scc_filed:collaborator-sheet; investor_1:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; scc_filed:collaborator-sheet; investor_1:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -6749,7 +6749,7 @@
           <t>162</t>
         </is>
       </c>
-      <c r="R50" t="inlineStr">
+      <c r="R50" s="2" t="inlineStr">
         <is>
           <t>162</t>
         </is>
@@ -6796,7 +6796,7 @@
       </c>
       <c r="AH50" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; property_name:collaborator-sheet; entity:collaborator-sheet; investor_1:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; property_name:collaborator-sheet; entity:collaborator-sheet; investor_1:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -6871,7 +6871,7 @@
           <t>229</t>
         </is>
       </c>
-      <c r="R51" t="inlineStr">
+      <c r="R51" s="2" t="inlineStr">
         <is>
           <t>229</t>
         </is>
@@ -6923,7 +6923,7 @@
       </c>
       <c r="AH51" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -7008,7 +7008,7 @@
           <t>145</t>
         </is>
       </c>
-      <c r="R52" t="inlineStr">
+      <c r="R52" s="2" t="inlineStr">
         <is>
           <t>144</t>
         </is>
@@ -7060,7 +7060,7 @@
       </c>
       <c r="AH52" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; built:collaborator-sheet; manual_status:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; built:collaborator-sheet; manual_status:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -7140,7 +7140,7 @@
           <t>63</t>
         </is>
       </c>
-      <c r="R53" t="inlineStr">
+      <c r="R53" s="2" t="inlineStr">
         <is>
           <t>62</t>
         </is>
@@ -7187,7 +7187,7 @@
       </c>
       <c r="AH53" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; city:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; city:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -7267,7 +7267,7 @@
           <t>198</t>
         </is>
       </c>
-      <c r="R54" t="inlineStr">
+      <c r="R54" s="2" t="inlineStr">
         <is>
           <t>198</t>
         </is>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="AH54" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; built:collaborator-sheet; manual_status:collaborator-sheet; city:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; built:collaborator-sheet; manual_status:collaborator-sheet; city:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -7389,7 +7389,7 @@
           <t>356</t>
         </is>
       </c>
-      <c r="R55" t="inlineStr">
+      <c r="R55" s="2" t="inlineStr">
         <is>
           <t>144</t>
         </is>
@@ -7441,7 +7441,7 @@
       </c>
       <c r="AH55" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; resolution:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; resolution:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -7521,7 +7521,7 @@
           <t>377</t>
         </is>
       </c>
-      <c r="R56" t="inlineStr">
+      <c r="R56" s="2" t="inlineStr">
         <is>
           <t>151</t>
         </is>
@@ -7573,7 +7573,7 @@
       </c>
       <c r="AH56" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -7648,7 +7648,7 @@
           <t>94</t>
         </is>
       </c>
-      <c r="R57" t="inlineStr">
+      <c r="R57" s="2" t="inlineStr">
         <is>
           <t>71</t>
         </is>
@@ -7695,7 +7695,7 @@
       </c>
       <c r="AH57" t="inlineStr">
         <is>
-          <t>leasing_link:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>leasing_link:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -7775,7 +7775,7 @@
           <t>193</t>
         </is>
       </c>
-      <c r="R58" t="inlineStr">
+      <c r="R58" s="2" t="inlineStr">
         <is>
           <t>193</t>
         </is>
@@ -7852,7 +7852,7 @@
       </c>
       <c r="AH58" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; built:collaborator-sheet; acquisition_price_m:collaborator-sheet; acquisition_date:collaborator-sheet; link:collaborator-sheet; leasing_link:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; built:collaborator-sheet; acquisition_price_m:collaborator-sheet; acquisition_date:collaborator-sheet; link:collaborator-sheet; leasing_link:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -7927,7 +7927,7 @@
           <t>296</t>
         </is>
       </c>
-      <c r="R59" t="inlineStr">
+      <c r="R59" s="2" t="inlineStr">
         <is>
           <t>296</t>
         </is>
@@ -7979,7 +7979,7 @@
       </c>
       <c r="AH59" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -8049,7 +8049,7 @@
           <t>193</t>
         </is>
       </c>
-      <c r="R60" t="inlineStr">
+      <c r="R60" s="2" t="inlineStr">
         <is>
           <t>100</t>
         </is>
@@ -8106,7 +8106,7 @@
       </c>
       <c r="AH60" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; built:collaborator-sheet; scc_filed:collaborator-sheet; city:collaborator-sheet; resolution:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; built:collaborator-sheet; scc_filed:collaborator-sheet; city:collaborator-sheet; resolution:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -8181,7 +8181,7 @@
           <t>196</t>
         </is>
       </c>
-      <c r="R61" t="inlineStr">
+      <c r="R61" s="2" t="inlineStr">
         <is>
           <t>29</t>
         </is>
@@ -8228,7 +8228,7 @@
       </c>
       <c r="AH61" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; entity:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; entity:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -8415,7 +8415,7 @@
           <t>116</t>
         </is>
       </c>
-      <c r="R63" t="inlineStr">
+      <c r="R63" s="2" t="inlineStr">
         <is>
           <t>115</t>
         </is>
@@ -8467,7 +8467,7 @@
       </c>
       <c r="AH63" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -8537,7 +8537,7 @@
           <t>32</t>
         </is>
       </c>
-      <c r="R64" t="inlineStr">
+      <c r="R64" s="2" t="inlineStr">
         <is>
           <t>32</t>
         </is>
@@ -8584,7 +8584,7 @@
       </c>
       <c r="AH64" t="inlineStr">
         <is>
-          <t>scc_filed:collaborator-sheet; resolution:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>scc_filed:collaborator-sheet; resolution:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -8766,7 +8766,7 @@
           <t>272</t>
         </is>
       </c>
-      <c r="R66" t="inlineStr">
+      <c r="R66" s="2" t="inlineStr">
         <is>
           <t>270</t>
         </is>
@@ -8823,7 +8823,7 @@
       </c>
       <c r="AH66" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; built:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; built:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -8903,7 +8903,7 @@
           <t>13</t>
         </is>
       </c>
-      <c r="R67" t="inlineStr">
+      <c r="R67" s="2" t="inlineStr">
         <is>
           <t>13</t>
         </is>
@@ -8945,7 +8945,7 @@
       </c>
       <c r="AH67" t="inlineStr">
         <is>
-          <t>manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -9020,7 +9020,7 @@
           <t>169</t>
         </is>
       </c>
-      <c r="R68" t="inlineStr">
+      <c r="R68" s="2" t="inlineStr">
         <is>
           <t>68</t>
         </is>
@@ -9067,7 +9067,7 @@
       </c>
       <c r="AH68" t="inlineStr">
         <is>
-          <t>scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -9142,7 +9142,7 @@
           <t>189</t>
         </is>
       </c>
-      <c r="R69" t="inlineStr">
+      <c r="R69" s="2" t="inlineStr">
         <is>
           <t>189</t>
         </is>
@@ -9199,7 +9199,7 @@
       </c>
       <c r="AH69" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; built:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; built:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -9279,7 +9279,7 @@
           <t>50</t>
         </is>
       </c>
-      <c r="R70" t="inlineStr">
+      <c r="R70" s="2" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -9321,7 +9321,7 @@
       </c>
       <c r="AH70" t="inlineStr">
         <is>
-          <t>manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -9401,6 +9401,11 @@
           <t>122</t>
         </is>
       </c>
+      <c r="R71" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="S71" s="2" t="inlineStr">
         <is>
           <t>20% at 60% AMI; 80% at 80% AMI</t>
@@ -9772,7 +9777,7 @@
           <t>189</t>
         </is>
       </c>
-      <c r="R74" t="inlineStr">
+      <c r="R74" s="2" t="inlineStr">
         <is>
           <t>148</t>
         </is>
@@ -9824,7 +9829,7 @@
       </c>
       <c r="AH74" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -10031,7 +10036,7 @@
           <t>203</t>
         </is>
       </c>
-      <c r="R76" t="inlineStr">
+      <c r="R76" s="2" t="inlineStr">
         <is>
           <t>203</t>
         </is>
@@ -10078,7 +10083,7 @@
       </c>
       <c r="AH76" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -10153,7 +10158,7 @@
           <t>50</t>
         </is>
       </c>
-      <c r="R77" t="inlineStr">
+      <c r="R77" s="2" t="inlineStr">
         <is>
           <t>49</t>
         </is>
@@ -10200,7 +10205,7 @@
       </c>
       <c r="AH77" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; entity:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -10275,7 +10280,7 @@
           <t>84</t>
         </is>
       </c>
-      <c r="R78" t="inlineStr">
+      <c r="R78" s="2" t="inlineStr">
         <is>
           <t>17</t>
         </is>
@@ -10322,7 +10327,7 @@
       </c>
       <c r="AH78" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -10534,7 +10539,7 @@
           <t>29</t>
         </is>
       </c>
-      <c r="R80" t="inlineStr">
+      <c r="R80" s="2" t="inlineStr">
         <is>
           <t>28</t>
         </is>
@@ -10581,7 +10586,7 @@
       </c>
       <c r="AH80" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; entity:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -10656,7 +10661,7 @@
           <t>36</t>
         </is>
       </c>
-      <c r="R81" t="inlineStr">
+      <c r="R81" s="2" t="inlineStr">
         <is>
           <t>35</t>
         </is>
@@ -10703,7 +10708,7 @@
       </c>
       <c r="AH81" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -10900,7 +10905,7 @@
           <t>20</t>
         </is>
       </c>
-      <c r="R83" t="inlineStr">
+      <c r="R83" s="2" t="inlineStr">
         <is>
           <t>19</t>
         </is>
@@ -10947,7 +10952,7 @@
       </c>
       <c r="AH83" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -11022,7 +11027,7 @@
           <t>28</t>
         </is>
       </c>
-      <c r="R84" t="inlineStr">
+      <c r="R84" s="2" t="inlineStr">
         <is>
           <t>27</t>
         </is>
@@ -11069,7 +11074,7 @@
       </c>
       <c r="AH84" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -11144,7 +11149,7 @@
           <t>21</t>
         </is>
       </c>
-      <c r="R85" t="inlineStr">
+      <c r="R85" s="2" t="inlineStr">
         <is>
           <t>20</t>
         </is>
@@ -11191,7 +11196,7 @@
       </c>
       <c r="AH85" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -11266,7 +11271,7 @@
           <t>48</t>
         </is>
       </c>
-      <c r="R86" t="inlineStr">
+      <c r="R86" s="2" t="inlineStr">
         <is>
           <t>47</t>
         </is>
@@ -11313,7 +11318,7 @@
       </c>
       <c r="AH86" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; entity:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -11388,7 +11393,7 @@
           <t>28</t>
         </is>
       </c>
-      <c r="R87" t="inlineStr">
+      <c r="R87" s="2" t="inlineStr">
         <is>
           <t>27</t>
         </is>
@@ -11435,7 +11440,7 @@
       </c>
       <c r="AH87" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; entity:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -11515,7 +11520,7 @@
           <t>687</t>
         </is>
       </c>
-      <c r="R88" t="inlineStr">
+      <c r="R88" s="2" t="inlineStr">
         <is>
           <t>687</t>
         </is>
@@ -11567,7 +11572,7 @@
       </c>
       <c r="AH88" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; scc_filed:collaborator-sheet; investor_1:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; scc_filed:collaborator-sheet; investor_1:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -11642,7 +11647,7 @@
           <t>69</t>
         </is>
       </c>
-      <c r="R89" t="inlineStr">
+      <c r="R89" s="2" t="inlineStr">
         <is>
           <t>68</t>
         </is>
@@ -11689,7 +11694,7 @@
       </c>
       <c r="AH89" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -11764,7 +11769,7 @@
           <t>230</t>
         </is>
       </c>
-      <c r="R90" t="inlineStr">
+      <c r="R90" s="2" t="inlineStr">
         <is>
           <t>230</t>
         </is>
@@ -11811,7 +11816,7 @@
       </c>
       <c r="AH90" t="inlineStr">
         <is>
-          <t>acquisition_date:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>acquisition_date:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -11886,7 +11891,7 @@
           <t>84</t>
         </is>
       </c>
-      <c r="R91" t="inlineStr">
+      <c r="R91" s="2" t="inlineStr">
         <is>
           <t>84</t>
         </is>
@@ -11933,7 +11938,7 @@
       </c>
       <c r="AH91" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -12008,7 +12013,7 @@
           <t>38</t>
         </is>
       </c>
-      <c r="R92" t="inlineStr">
+      <c r="R92" s="2" t="inlineStr">
         <is>
           <t>37</t>
         </is>
@@ -12055,7 +12060,7 @@
       </c>
       <c r="AH92" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -12130,7 +12135,7 @@
           <t>177</t>
         </is>
       </c>
-      <c r="R93" t="inlineStr">
+      <c r="R93" s="2" t="inlineStr">
         <is>
           <t>177</t>
         </is>
@@ -12182,7 +12187,7 @@
       </c>
       <c r="AH93" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -12252,7 +12257,7 @@
           <t>148</t>
         </is>
       </c>
-      <c r="R94" t="inlineStr">
+      <c r="R94" s="2" t="inlineStr">
         <is>
           <t>148</t>
         </is>
@@ -12299,7 +12304,7 @@
       </c>
       <c r="AH94" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; resolution:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; resolution:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -12374,7 +12379,7 @@
           <t>183</t>
         </is>
       </c>
-      <c r="R95" t="inlineStr">
+      <c r="R95" s="2" t="inlineStr">
         <is>
           <t>183</t>
         </is>
@@ -12431,7 +12436,7 @@
       </c>
       <c r="AH95" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; built:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; built:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -12506,7 +12511,7 @@
           <t>164</t>
         </is>
       </c>
-      <c r="R96" t="inlineStr">
+      <c r="R96" s="2" t="inlineStr">
         <is>
           <t>164</t>
         </is>
@@ -12563,7 +12568,7 @@
       </c>
       <c r="AH96" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; acquisition_date:collaborator-sheet; link:collaborator-sheet; scc_filed:collaborator-sheet; resolution:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_2:collaborator-sheet; acquisition_date:collaborator-sheet; link:collaborator-sheet; scc_filed:collaborator-sheet; resolution:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -12643,7 +12648,7 @@
           <t>948</t>
         </is>
       </c>
-      <c r="R97" t="inlineStr">
+      <c r="R97" s="2" t="inlineStr">
         <is>
           <t>948</t>
         </is>
@@ -12705,7 +12710,7 @@
       </c>
       <c r="AH97" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; built:collaborator-sheet; acquisition_price_m:collaborator-sheet; acquisition_date:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_2:collaborator-sheet; built:collaborator-sheet; acquisition_price_m:collaborator-sheet; acquisition_date:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -12780,7 +12785,7 @@
           <t>112</t>
         </is>
       </c>
-      <c r="R98" t="inlineStr">
+      <c r="R98" s="2" t="inlineStr">
         <is>
           <t>112</t>
         </is>
@@ -12827,7 +12832,7 @@
       </c>
       <c r="AH98" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -12907,7 +12912,7 @@
           <t>192</t>
         </is>
       </c>
-      <c r="R99" t="inlineStr">
+      <c r="R99" s="2" t="inlineStr">
         <is>
           <t>192</t>
         </is>
@@ -12959,7 +12964,7 @@
       </c>
       <c r="AH99" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; leasing_link:collaborator-sheet; manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; leasing_link:collaborator-sheet; manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -13161,7 +13166,7 @@
           <t>72</t>
         </is>
       </c>
-      <c r="R101" t="inlineStr">
+      <c r="R101" s="2" t="inlineStr">
         <is>
           <t>71</t>
         </is>
@@ -13213,7 +13218,7 @@
       </c>
       <c r="AH101" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -13288,7 +13293,7 @@
           <t>73</t>
         </is>
       </c>
-      <c r="R102" t="inlineStr">
+      <c r="R102" s="2" t="inlineStr">
         <is>
           <t>72</t>
         </is>
@@ -13340,7 +13345,7 @@
       </c>
       <c r="AH102" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -13415,7 +13420,7 @@
           <t>53</t>
         </is>
       </c>
-      <c r="R103" t="inlineStr">
+      <c r="R103" s="2" t="inlineStr">
         <is>
           <t>52</t>
         </is>
@@ -13467,7 +13472,7 @@
       </c>
       <c r="AH103" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -13542,7 +13547,7 @@
           <t>25</t>
         </is>
       </c>
-      <c r="R104" t="inlineStr">
+      <c r="R104" s="2" t="inlineStr">
         <is>
           <t>25</t>
         </is>
@@ -13589,7 +13594,7 @@
       </c>
       <c r="AH104" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -13664,7 +13669,7 @@
           <t>27</t>
         </is>
       </c>
-      <c r="R105" t="inlineStr">
+      <c r="R105" s="2" t="inlineStr">
         <is>
           <t>27</t>
         </is>
@@ -13711,7 +13716,7 @@
       </c>
       <c r="AH105" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -13786,7 +13791,7 @@
           <t>49</t>
         </is>
       </c>
-      <c r="R106" t="inlineStr">
+      <c r="R106" s="2" t="inlineStr">
         <is>
           <t>49</t>
         </is>
@@ -13833,7 +13838,7 @@
       </c>
       <c r="AH106" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -13908,7 +13913,7 @@
           <t>48</t>
         </is>
       </c>
-      <c r="R107" t="inlineStr">
+      <c r="R107" s="2" t="inlineStr">
         <is>
           <t>48</t>
         </is>
@@ -13955,7 +13960,7 @@
       </c>
       <c r="AH107" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -14030,7 +14035,7 @@
           <t>43</t>
         </is>
       </c>
-      <c r="R108" t="inlineStr">
+      <c r="R108" s="2" t="inlineStr">
         <is>
           <t>43</t>
         </is>
@@ -14077,7 +14082,7 @@
       </c>
       <c r="AH108" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -14152,7 +14157,7 @@
           <t>38</t>
         </is>
       </c>
-      <c r="R109" t="inlineStr">
+      <c r="R109" s="2" t="inlineStr">
         <is>
           <t>38</t>
         </is>
@@ -14199,7 +14204,7 @@
       </c>
       <c r="AH109" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -14274,7 +14279,7 @@
           <t>32</t>
         </is>
       </c>
-      <c r="R110" t="inlineStr">
+      <c r="R110" s="2" t="inlineStr">
         <is>
           <t>32</t>
         </is>
@@ -14321,7 +14326,7 @@
       </c>
       <c r="AH110" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -14630,7 +14635,7 @@
           <t>40</t>
         </is>
       </c>
-      <c r="R113" t="inlineStr">
+      <c r="R113" s="2" t="inlineStr">
         <is>
           <t>40</t>
         </is>
@@ -14677,7 +14682,7 @@
       </c>
       <c r="AH113" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -14752,7 +14757,7 @@
           <t>32</t>
         </is>
       </c>
-      <c r="R114" t="inlineStr">
+      <c r="R114" s="2" t="inlineStr">
         <is>
           <t>32</t>
         </is>
@@ -14799,7 +14804,7 @@
       </c>
       <c r="AH114" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -14874,7 +14879,7 @@
           <t>20</t>
         </is>
       </c>
-      <c r="R115" t="inlineStr">
+      <c r="R115" s="2" t="inlineStr">
         <is>
           <t>20</t>
         </is>
@@ -14921,7 +14926,7 @@
       </c>
       <c r="AH115" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -14996,7 +15001,7 @@
           <t>60</t>
         </is>
       </c>
-      <c r="R116" t="inlineStr">
+      <c r="R116" s="2" t="inlineStr">
         <is>
           <t>60</t>
         </is>
@@ -15043,7 +15048,7 @@
       </c>
       <c r="AH116" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -15118,7 +15123,7 @@
           <t>73</t>
         </is>
       </c>
-      <c r="R117" t="inlineStr">
+      <c r="R117" s="2" t="inlineStr">
         <is>
           <t>73</t>
         </is>
@@ -15165,7 +15170,7 @@
       </c>
       <c r="AH117" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -15240,7 +15245,7 @@
           <t>55</t>
         </is>
       </c>
-      <c r="R118" t="inlineStr">
+      <c r="R118" s="2" t="inlineStr">
         <is>
           <t>55</t>
         </is>
@@ -15287,7 +15292,7 @@
       </c>
       <c r="AH118" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -15362,7 +15367,7 @@
           <t>40</t>
         </is>
       </c>
-      <c r="R119" t="inlineStr">
+      <c r="R119" s="2" t="inlineStr">
         <is>
           <t>40</t>
         </is>
@@ -15409,7 +15414,7 @@
       </c>
       <c r="AH119" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -15596,7 +15601,7 @@
           <t>272</t>
         </is>
       </c>
-      <c r="R121" t="inlineStr">
+      <c r="R121" s="2" t="inlineStr">
         <is>
           <t>272</t>
         </is>
@@ -15648,7 +15653,7 @@
       </c>
       <c r="AH121" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; city:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; city:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -15845,7 +15850,7 @@
           <t>39</t>
         </is>
       </c>
-      <c r="R123" t="inlineStr">
+      <c r="R123" s="2" t="inlineStr">
         <is>
           <t>39</t>
         </is>
@@ -15892,7 +15897,7 @@
       </c>
       <c r="AH123" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -15972,7 +15977,7 @@
           <t>48</t>
         </is>
       </c>
-      <c r="R124" t="inlineStr">
+      <c r="R124" s="2" t="inlineStr">
         <is>
           <t>48</t>
         </is>
@@ -16019,7 +16024,7 @@
       </c>
       <c r="AH124" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -16099,7 +16104,7 @@
           <t>18</t>
         </is>
       </c>
-      <c r="R125" t="inlineStr">
+      <c r="R125" s="2" t="inlineStr">
         <is>
           <t>18</t>
         </is>
@@ -16146,7 +16151,7 @@
       </c>
       <c r="AH125" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -16226,7 +16231,7 @@
           <t>45</t>
         </is>
       </c>
-      <c r="R126" t="inlineStr">
+      <c r="R126" s="2" t="inlineStr">
         <is>
           <t>45</t>
         </is>
@@ -16273,7 +16278,7 @@
       </c>
       <c r="AH126" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; property_name:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; property_name:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -16353,7 +16358,7 @@
           <t>40</t>
         </is>
       </c>
-      <c r="R127" t="inlineStr">
+      <c r="R127" s="2" t="inlineStr">
         <is>
           <t>40</t>
         </is>
@@ -16400,7 +16405,7 @@
       </c>
       <c r="AH127" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -16480,7 +16485,7 @@
           <t>23</t>
         </is>
       </c>
-      <c r="R128" t="inlineStr">
+      <c r="R128" s="2" t="inlineStr">
         <is>
           <t>23</t>
         </is>
@@ -16527,7 +16532,7 @@
       </c>
       <c r="AH128" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -16607,7 +16612,7 @@
           <t>48</t>
         </is>
       </c>
-      <c r="R129" t="inlineStr">
+      <c r="R129" s="2" t="inlineStr">
         <is>
           <t>48</t>
         </is>
@@ -16654,7 +16659,7 @@
       </c>
       <c r="AH129" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -16734,7 +16739,7 @@
           <t>32</t>
         </is>
       </c>
-      <c r="R130" t="inlineStr">
+      <c r="R130" s="2" t="inlineStr">
         <is>
           <t>32</t>
         </is>
@@ -16781,7 +16786,7 @@
       </c>
       <c r="AH130" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -16861,7 +16866,7 @@
           <t>76</t>
         </is>
       </c>
-      <c r="R131" t="inlineStr">
+      <c r="R131" s="2" t="inlineStr">
         <is>
           <t>76</t>
         </is>
@@ -16908,7 +16913,7 @@
       </c>
       <c r="AH131" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -16983,7 +16988,7 @@
           <t>37</t>
         </is>
       </c>
-      <c r="R132" t="inlineStr">
+      <c r="R132" s="2" t="inlineStr">
         <is>
           <t>37</t>
         </is>
@@ -17030,7 +17035,7 @@
       </c>
       <c r="AH132" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -17105,7 +17110,7 @@
           <t>79</t>
         </is>
       </c>
-      <c r="R133" t="inlineStr">
+      <c r="R133" s="2" t="inlineStr">
         <is>
           <t>78</t>
         </is>
@@ -17147,7 +17152,7 @@
       </c>
       <c r="AH133" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -17222,7 +17227,7 @@
           <t>68</t>
         </is>
       </c>
-      <c r="R134" t="inlineStr">
+      <c r="R134" s="2" t="inlineStr">
         <is>
           <t>68</t>
         </is>
@@ -17269,7 +17274,7 @@
       </c>
       <c r="AH134" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -17349,7 +17354,7 @@
           <t>52</t>
         </is>
       </c>
-      <c r="R135" t="inlineStr">
+      <c r="R135" s="2" t="inlineStr">
         <is>
           <t>52</t>
         </is>
@@ -17396,7 +17401,7 @@
       </c>
       <c r="AH135" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -17573,7 +17578,7 @@
           <t>41</t>
         </is>
       </c>
-      <c r="R137" t="inlineStr">
+      <c r="R137" s="2" t="inlineStr">
         <is>
           <t>41</t>
         </is>
@@ -17620,7 +17625,7 @@
       </c>
       <c r="AH137" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -17695,7 +17700,7 @@
           <t>114</t>
         </is>
       </c>
-      <c r="R138" t="inlineStr">
+      <c r="R138" s="2" t="inlineStr">
         <is>
           <t>114</t>
         </is>
@@ -17747,7 +17752,7 @@
       </c>
       <c r="AH138" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; city:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; city:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -17822,7 +17827,7 @@
           <t>286</t>
         </is>
       </c>
-      <c r="R139" t="inlineStr">
+      <c r="R139" s="2" t="inlineStr">
         <is>
           <t>286</t>
         </is>
@@ -17869,7 +17874,7 @@
       </c>
       <c r="AH139" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; nonprofit_partner:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -17944,7 +17949,7 @@
           <t>148</t>
         </is>
       </c>
-      <c r="R140" t="inlineStr">
+      <c r="R140" s="2" t="inlineStr">
         <is>
           <t>148</t>
         </is>
@@ -17991,7 +17996,7 @@
       </c>
       <c r="AH140" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -18061,7 +18066,7 @@
           <t>278</t>
         </is>
       </c>
-      <c r="R141" t="inlineStr">
+      <c r="R141" s="2" t="inlineStr">
         <is>
           <t>278</t>
         </is>
@@ -18113,7 +18118,7 @@
       </c>
       <c r="AH141" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; built:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; built:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -18183,7 +18188,7 @@
           <t>116</t>
         </is>
       </c>
-      <c r="R142" t="inlineStr">
+      <c r="R142" s="2" t="inlineStr">
         <is>
           <t>116</t>
         </is>
@@ -18225,7 +18230,7 @@
       </c>
       <c r="AH142" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -18427,7 +18432,7 @@
           <t>460</t>
         </is>
       </c>
-      <c r="R144" t="inlineStr">
+      <c r="R144" s="2" t="inlineStr">
         <is>
           <t>460</t>
         </is>
@@ -18474,7 +18479,7 @@
       </c>
       <c r="AH144" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; property_name:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; property_name:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -18544,7 +18549,7 @@
           <t>110</t>
         </is>
       </c>
-      <c r="R145" t="inlineStr">
+      <c r="R145" s="2" t="inlineStr">
         <is>
           <t>110</t>
         </is>
@@ -18591,7 +18596,7 @@
       </c>
       <c r="AH145" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -18925,7 +18930,7 @@
           <t>170</t>
         </is>
       </c>
-      <c r="R148" t="inlineStr">
+      <c r="R148" s="2" t="inlineStr">
         <is>
           <t>170</t>
         </is>
@@ -18977,7 +18982,7 @@
       </c>
       <c r="AH148" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; built:collaborator-sheet; manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; built:collaborator-sheet; manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -19057,7 +19062,7 @@
           <t>61</t>
         </is>
       </c>
-      <c r="R149" t="inlineStr">
+      <c r="R149" s="2" t="inlineStr">
         <is>
           <t>61</t>
         </is>
@@ -19104,7 +19109,7 @@
       </c>
       <c r="AH149" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -19184,7 +19189,7 @@
           <t>181</t>
         </is>
       </c>
-      <c r="R150" t="inlineStr">
+      <c r="R150" s="2" t="inlineStr">
         <is>
           <t>181</t>
         </is>
@@ -19231,7 +19236,7 @@
       </c>
       <c r="AH150" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; property_name:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; property_name:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -19311,7 +19316,7 @@
           <t>74</t>
         </is>
       </c>
-      <c r="R151" t="inlineStr">
+      <c r="R151" s="2" t="inlineStr">
         <is>
           <t>74</t>
         </is>
@@ -19358,7 +19363,7 @@
       </c>
       <c r="AH151" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; property_name:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; property_name:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -19433,7 +19438,7 @@
           <t>152</t>
         </is>
       </c>
-      <c r="R152" t="inlineStr">
+      <c r="R152" s="2" t="inlineStr">
         <is>
           <t>152</t>
         </is>
@@ -19480,7 +19485,7 @@
       </c>
       <c r="AH152" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -19555,7 +19560,7 @@
           <t>101</t>
         </is>
       </c>
-      <c r="R153" t="inlineStr">
+      <c r="R153" s="2" t="inlineStr">
         <is>
           <t>101</t>
         </is>
@@ -19607,7 +19612,7 @@
       </c>
       <c r="AH153" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; built:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; built:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -19682,7 +19687,7 @@
           <t>482</t>
         </is>
       </c>
-      <c r="R154" t="inlineStr">
+      <c r="R154" s="2" t="inlineStr">
         <is>
           <t>216</t>
         </is>
@@ -19729,7 +19734,7 @@
       </c>
       <c r="AH154" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -19804,7 +19809,7 @@
           <t>120</t>
         </is>
       </c>
-      <c r="R155" t="inlineStr">
+      <c r="R155" s="2" t="inlineStr">
         <is>
           <t>120</t>
         </is>
@@ -19856,7 +19861,7 @@
       </c>
       <c r="AH155" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; built:collaborator-sheet; entity:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; built:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -19931,7 +19936,7 @@
           <t>170</t>
         </is>
       </c>
-      <c r="R156" t="inlineStr">
+      <c r="R156" s="2" t="inlineStr">
         <is>
           <t>170</t>
         </is>
@@ -19983,7 +19988,7 @@
       </c>
       <c r="AH156" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; built:collaborator-sheet; entity:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; built:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -20150,7 +20155,7 @@
           <t>29</t>
         </is>
       </c>
-      <c r="R158" t="inlineStr">
+      <c r="R158" s="2" t="inlineStr">
         <is>
           <t>29</t>
         </is>
@@ -20192,7 +20197,7 @@
       </c>
       <c r="AH158" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; total_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -20267,7 +20272,7 @@
           <t>290</t>
         </is>
       </c>
-      <c r="R159" t="inlineStr">
+      <c r="R159" s="2" t="inlineStr">
         <is>
           <t>290</t>
         </is>
@@ -20309,7 +20314,7 @@
       </c>
       <c r="AH159" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -20389,7 +20394,7 @@
           <t>16</t>
         </is>
       </c>
-      <c r="R160" t="inlineStr">
+      <c r="R160" s="2" t="inlineStr">
         <is>
           <t>16</t>
         </is>
@@ -20436,7 +20441,7 @@
       </c>
       <c r="AH160" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -20511,7 +20516,7 @@
           <t>40</t>
         </is>
       </c>
-      <c r="R161" t="inlineStr">
+      <c r="R161" s="2" t="inlineStr">
         <is>
           <t>40</t>
         </is>
@@ -20553,7 +20558,7 @@
       </c>
       <c r="AH161" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -20735,7 +20740,7 @@
           <t>67</t>
         </is>
       </c>
-      <c r="R163" t="inlineStr">
+      <c r="R163" s="2" t="inlineStr">
         <is>
           <t>67</t>
         </is>
@@ -20777,7 +20782,7 @@
       </c>
       <c r="AH163" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -20852,7 +20857,7 @@
           <t>40</t>
         </is>
       </c>
-      <c r="R164" t="inlineStr">
+      <c r="R164" s="2" t="inlineStr">
         <is>
           <t>40</t>
         </is>
@@ -20894,7 +20899,7 @@
       </c>
       <c r="AH164" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -20969,7 +20974,7 @@
           <t>39</t>
         </is>
       </c>
-      <c r="R165" t="inlineStr">
+      <c r="R165" s="2" t="inlineStr">
         <is>
           <t>39</t>
         </is>
@@ -21011,7 +21016,7 @@
       </c>
       <c r="AH165" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -21086,7 +21091,7 @@
           <t>40</t>
         </is>
       </c>
-      <c r="R166" t="inlineStr">
+      <c r="R166" s="2" t="inlineStr">
         <is>
           <t>40</t>
         </is>
@@ -21128,7 +21133,7 @@
       </c>
       <c r="AH166" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -21203,7 +21208,7 @@
           <t>20</t>
         </is>
       </c>
-      <c r="R167" t="inlineStr">
+      <c r="R167" s="2" t="inlineStr">
         <is>
           <t>20</t>
         </is>
@@ -21245,7 +21250,7 @@
       </c>
       <c r="AH167" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -21320,7 +21325,7 @@
           <t>48</t>
         </is>
       </c>
-      <c r="R168" t="inlineStr">
+      <c r="R168" s="2" t="inlineStr">
         <is>
           <t>48</t>
         </is>
@@ -21362,7 +21367,7 @@
       </c>
       <c r="AH168" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -21437,7 +21442,7 @@
           <t>18</t>
         </is>
       </c>
-      <c r="R169" t="inlineStr">
+      <c r="R169" s="2" t="inlineStr">
         <is>
           <t>18</t>
         </is>
@@ -21479,7 +21484,7 @@
       </c>
       <c r="AH169" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -21554,7 +21559,7 @@
           <t>45</t>
         </is>
       </c>
-      <c r="R170" t="inlineStr">
+      <c r="R170" s="2" t="inlineStr">
         <is>
           <t>45</t>
         </is>
@@ -21596,7 +21601,7 @@
       </c>
       <c r="AH170" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -21671,7 +21676,7 @@
           <t>42</t>
         </is>
       </c>
-      <c r="R171" t="inlineStr">
+      <c r="R171" s="2" t="inlineStr">
         <is>
           <t>42</t>
         </is>
@@ -21713,7 +21718,7 @@
       </c>
       <c r="AH171" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -21895,7 +21900,7 @@
           <t>40</t>
         </is>
       </c>
-      <c r="R173" t="inlineStr">
+      <c r="R173" s="2" t="inlineStr">
         <is>
           <t>40</t>
         </is>
@@ -21937,7 +21942,7 @@
       </c>
       <c r="AH173" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -22012,7 +22017,7 @@
           <t>23</t>
         </is>
       </c>
-      <c r="R174" t="inlineStr">
+      <c r="R174" s="2" t="inlineStr">
         <is>
           <t>23</t>
         </is>
@@ -22054,7 +22059,7 @@
       </c>
       <c r="AH174" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -22129,7 +22134,7 @@
           <t>48</t>
         </is>
       </c>
-      <c r="R175" t="inlineStr">
+      <c r="R175" s="2" t="inlineStr">
         <is>
           <t>48</t>
         </is>
@@ -22171,7 +22176,7 @@
       </c>
       <c r="AH175" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -22246,7 +22251,7 @@
           <t>31</t>
         </is>
       </c>
-      <c r="R176" t="inlineStr">
+      <c r="R176" s="2" t="inlineStr">
         <is>
           <t>31</t>
         </is>
@@ -22288,7 +22293,7 @@
       </c>
       <c r="AH176" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -22363,7 +22368,7 @@
           <t>32</t>
         </is>
       </c>
-      <c r="R177" t="inlineStr">
+      <c r="R177" s="2" t="inlineStr">
         <is>
           <t>32</t>
         </is>
@@ -22405,7 +22410,7 @@
       </c>
       <c r="AH177" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -22480,7 +22485,7 @@
           <t>40</t>
         </is>
       </c>
-      <c r="R178" t="inlineStr">
+      <c r="R178" s="2" t="inlineStr">
         <is>
           <t>40</t>
         </is>
@@ -22522,7 +22527,7 @@
       </c>
       <c r="AH178" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -22597,7 +22602,7 @@
           <t>76</t>
         </is>
       </c>
-      <c r="R179" t="inlineStr">
+      <c r="R179" s="2" t="inlineStr">
         <is>
           <t>76</t>
         </is>
@@ -22639,7 +22644,7 @@
       </c>
       <c r="AH179" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -22826,7 +22831,7 @@
           <t>152</t>
         </is>
       </c>
-      <c r="R181" t="inlineStr">
+      <c r="R181" s="2" t="inlineStr">
         <is>
           <t>152</t>
         </is>
@@ -22868,7 +22873,7 @@
       </c>
       <c r="AH181" t="inlineStr">
         <is>
-          <t>manual_status:collaborator-sheet; city:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>manual_status:collaborator-sheet; city:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -23080,7 +23085,7 @@
           <t>70</t>
         </is>
       </c>
-      <c r="R183" t="inlineStr">
+      <c r="R183" s="2" t="inlineStr">
         <is>
           <t>13</t>
         </is>
@@ -23122,7 +23127,7 @@
       </c>
       <c r="AH183" t="inlineStr">
         <is>
-          <t>manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -23197,7 +23202,7 @@
           <t>30</t>
         </is>
       </c>
-      <c r="R184" t="inlineStr">
+      <c r="R184" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -23244,7 +23249,7 @@
       </c>
       <c r="AH184" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -23319,7 +23324,7 @@
           <t>39</t>
         </is>
       </c>
-      <c r="R185" t="inlineStr">
+      <c r="R185" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
@@ -23366,7 +23371,7 @@
       </c>
       <c r="AH185" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -23441,7 +23446,7 @@
           <t>70</t>
         </is>
       </c>
-      <c r="R186" t="inlineStr">
+      <c r="R186" s="2" t="inlineStr">
         <is>
           <t>14</t>
         </is>
@@ -23488,7 +23493,7 @@
       </c>
       <c r="AH186" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -23563,7 +23568,7 @@
           <t>232</t>
         </is>
       </c>
-      <c r="R187" t="inlineStr">
+      <c r="R187" s="2" t="inlineStr">
         <is>
           <t>232</t>
         </is>
@@ -23610,7 +23615,7 @@
       </c>
       <c r="AH187" t="inlineStr">
         <is>
-          <t>built:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>built:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -23680,7 +23685,7 @@
           <t>135</t>
         </is>
       </c>
-      <c r="R188" t="inlineStr">
+      <c r="R188" s="2" t="inlineStr">
         <is>
           <t>27</t>
         </is>
@@ -23722,7 +23727,7 @@
       </c>
       <c r="AH188" t="inlineStr">
         <is>
-          <t>manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -23792,7 +23797,7 @@
           <t>221</t>
         </is>
       </c>
-      <c r="R189" t="inlineStr">
+      <c r="R189" s="2" t="inlineStr">
         <is>
           <t>221</t>
         </is>
@@ -23844,7 +23849,7 @@
       </c>
       <c r="AH189" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; built:collaborator-sheet; manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; built:collaborator-sheet; manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -23919,7 +23924,7 @@
           <t>293</t>
         </is>
       </c>
-      <c r="R190" t="inlineStr">
+      <c r="R190" s="2" t="inlineStr">
         <is>
           <t>102</t>
         </is>
@@ -23966,7 +23971,7 @@
       </c>
       <c r="AH190" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; entity:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -24332,7 +24337,7 @@
           <t>37</t>
         </is>
       </c>
-      <c r="R194" t="inlineStr">
+      <c r="R194" s="2" t="inlineStr">
         <is>
           <t>36</t>
         </is>
@@ -24379,7 +24384,7 @@
       </c>
       <c r="AH194" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -24454,7 +24459,7 @@
           <t>41</t>
         </is>
       </c>
-      <c r="R195" t="inlineStr">
+      <c r="R195" s="2" t="inlineStr">
         <is>
           <t>41</t>
         </is>
@@ -24501,7 +24506,7 @@
       </c>
       <c r="AH195" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -24683,7 +24688,7 @@
           <t>100</t>
         </is>
       </c>
-      <c r="R197" t="inlineStr">
+      <c r="R197" s="2" t="inlineStr">
         <is>
           <t>100</t>
         </is>
@@ -24730,7 +24735,7 @@
       </c>
       <c r="AH197" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -24795,7 +24800,7 @@
           <t>264</t>
         </is>
       </c>
-      <c r="R198" t="inlineStr">
+      <c r="R198" s="2" t="inlineStr">
         <is>
           <t>264</t>
         </is>
@@ -24842,7 +24847,7 @@
       </c>
       <c r="AH198" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -24917,7 +24922,7 @@
           <t>38</t>
         </is>
       </c>
-      <c r="R199" t="inlineStr">
+      <c r="R199" s="2" t="inlineStr">
         <is>
           <t>37</t>
         </is>
@@ -24959,7 +24964,7 @@
       </c>
       <c r="AH199" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; city_cut:collaborator-sheet; address:manual-repo-edit</t>
+          <t>city_cut:collaborator-sheet; address:manual-repo-edit</t>
         </is>
       </c>
     </row>
@@ -25029,7 +25034,7 @@
           <t>70</t>
         </is>
       </c>
-      <c r="R200" t="inlineStr">
+      <c r="R200" s="2" t="inlineStr">
         <is>
           <t>70</t>
         </is>
@@ -25071,7 +25076,7 @@
       </c>
       <c r="AH200" t="inlineStr">
         <is>
-          <t>resolution:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>resolution:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -25151,7 +25156,7 @@
           <t>197</t>
         </is>
       </c>
-      <c r="R201" t="inlineStr">
+      <c r="R201" s="2" t="inlineStr">
         <is>
           <t>80</t>
         </is>
@@ -25193,7 +25198,7 @@
       </c>
       <c r="AH201" t="inlineStr">
         <is>
-          <t>manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -25268,7 +25273,7 @@
           <t>150</t>
         </is>
       </c>
-      <c r="R202" t="inlineStr">
+      <c r="R202" s="2" t="inlineStr">
         <is>
           <t>150</t>
         </is>
@@ -25320,7 +25325,7 @@
       </c>
       <c r="AH202" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; built:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; built:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -25395,7 +25400,7 @@
           <t>208</t>
         </is>
       </c>
-      <c r="R203" t="inlineStr">
+      <c r="R203" s="2" t="inlineStr">
         <is>
           <t>208</t>
         </is>
@@ -25437,7 +25442,7 @@
       </c>
       <c r="AH203" t="inlineStr">
         <is>
-          <t>city:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>city:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -25512,7 +25517,7 @@
           <t>49</t>
         </is>
       </c>
-      <c r="R204" t="inlineStr">
+      <c r="R204" s="2" t="inlineStr">
         <is>
           <t>49</t>
         </is>
@@ -25559,7 +25564,7 @@
       </c>
       <c r="AH204" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:manual-repo-edit</t>
+          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; address:manual-repo-edit</t>
         </is>
       </c>
     </row>
@@ -25751,7 +25756,7 @@
           <t>123</t>
         </is>
       </c>
-      <c r="R206" t="inlineStr">
+      <c r="R206" s="2" t="inlineStr">
         <is>
           <t>123</t>
         </is>
@@ -25793,7 +25798,7 @@
       </c>
       <c r="AH206" t="inlineStr">
         <is>
-          <t>manual_status:collaborator-sheet; county:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>manual_status:collaborator-sheet; county:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -26087,7 +26092,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="R209" t="inlineStr">
+      <c r="R209" s="2" t="inlineStr">
         <is>
           <t>12</t>
         </is>
@@ -26129,7 +26134,7 @@
       </c>
       <c r="AH209" t="inlineStr">
         <is>
-          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; term_years:collaborator-sheet</t>
+          <t>investor_1:collaborator-sheet; address:collaborator-sheet; term_years:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -26204,7 +26209,7 @@
           <t>211</t>
         </is>
       </c>
-      <c r="R210" t="inlineStr">
+      <c r="R210" s="2" t="inlineStr">
         <is>
           <t>211</t>
         </is>
@@ -26241,7 +26246,7 @@
       </c>
       <c r="AH210" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet; term_years:collaborator-sheet</t>
+          <t>address:collaborator-sheet; term_years:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -26901,7 +26906,7 @@
           <t>81</t>
         </is>
       </c>
-      <c r="R216" t="inlineStr">
+      <c r="R216" s="2" t="inlineStr">
         <is>
           <t>81</t>
         </is>
@@ -26948,7 +26953,7 @@
       </c>
       <c r="AH216" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -27023,7 +27028,7 @@
           <t>34</t>
         </is>
       </c>
-      <c r="R217" t="inlineStr">
+      <c r="R217" s="2" t="inlineStr">
         <is>
           <t>34</t>
         </is>
@@ -27070,7 +27075,7 @@
       </c>
       <c r="AH217" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:manual-repo-edit</t>
+          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; address:manual-repo-edit</t>
         </is>
       </c>
     </row>
@@ -27257,7 +27262,7 @@
           <t>94</t>
         </is>
       </c>
-      <c r="R219" t="inlineStr">
+      <c r="R219" s="2" t="inlineStr">
         <is>
           <t>94</t>
         </is>
@@ -27304,7 +27309,7 @@
       </c>
       <c r="AH219" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -27491,7 +27496,7 @@
           <t>64</t>
         </is>
       </c>
-      <c r="R221" t="inlineStr">
+      <c r="R221" s="2" t="inlineStr">
         <is>
           <t>58</t>
         </is>
@@ -27538,7 +27543,7 @@
       </c>
       <c r="AH221" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -27894,7 +27899,7 @@
           <t>132</t>
         </is>
       </c>
-      <c r="R225" t="inlineStr">
+      <c r="R225" s="2" t="inlineStr">
         <is>
           <t>132</t>
         </is>
@@ -27936,7 +27941,7 @@
       </c>
       <c r="AH225" t="inlineStr">
         <is>
-          <t>entity:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; term_years:collaborator-sheet</t>
+          <t>entity:collaborator-sheet; address:collaborator-sheet; term_years:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -28118,7 +28123,7 @@
           <t>148</t>
         </is>
       </c>
-      <c r="R227" t="inlineStr">
+      <c r="R227" s="2" t="inlineStr">
         <is>
           <t>148</t>
         </is>
@@ -28160,7 +28165,7 @@
       </c>
       <c r="AH227" t="inlineStr">
         <is>
-          <t>restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -29611,6 +29616,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="R241" s="2" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
       <c r="S241" s="2" t="inlineStr">
         <is>
           <t>78% at 80% AMI</t>
@@ -29785,6 +29795,11 @@
           <t>111</t>
         </is>
       </c>
+      <c r="R243" s="2" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
       <c r="S243" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -29892,6 +29907,11 @@
           <t>169</t>
         </is>
       </c>
+      <c r="R244" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
       <c r="S244" s="2" t="inlineStr">
         <is>
           <t>34% at 80% AMI</t>
@@ -29994,6 +30014,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="R245" s="2" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
       <c r="S245" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -30091,6 +30116,11 @@
           <t>697</t>
         </is>
       </c>
+      <c r="R246" s="2" t="inlineStr">
+        <is>
+          <t>697</t>
+        </is>
+      </c>
       <c r="S246" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -30193,6 +30223,11 @@
           <t>488</t>
         </is>
       </c>
+      <c r="R247" s="2" t="inlineStr">
+        <is>
+          <t>483</t>
+        </is>
+      </c>
       <c r="S247" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -30300,6 +30335,11 @@
           <t>406</t>
         </is>
       </c>
+      <c r="R248" s="2" t="inlineStr">
+        <is>
+          <t>406</t>
+        </is>
+      </c>
       <c r="S248" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -30392,6 +30432,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="R249" s="2" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
       <c r="S249" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -30484,6 +30529,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="R250" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="S250" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -30581,6 +30631,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="R251" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="S251" s="2" t="inlineStr">
         <is>
           <t>at 80% AMI</t>
@@ -30673,6 +30728,11 @@
           <t>171</t>
         </is>
       </c>
+      <c r="R252" s="2" t="inlineStr">
+        <is>
+          <t>171</t>
+        </is>
+      </c>
       <c r="S252" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -30760,6 +30820,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="R253" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
       <c r="S253" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -30862,6 +30927,11 @@
           <t>89</t>
         </is>
       </c>
+      <c r="R254" s="2" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
       <c r="S254" s="2" t="inlineStr">
         <is>
           <t>10% at 60% AMI; 90% at 80% AMI</t>
@@ -30954,6 +31024,11 @@
           <t>156</t>
         </is>
       </c>
+      <c r="R255" s="2" t="inlineStr">
+        <is>
+          <t>156</t>
+        </is>
+      </c>
       <c r="S255" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -31046,6 +31121,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="R256" s="2" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
       <c r="S256" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -31138,6 +31218,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="R257" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
       <c r="S257" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -31230,6 +31315,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="R258" s="2" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
       <c r="S258" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -31322,6 +31412,11 @@
           <t>188</t>
         </is>
       </c>
+      <c r="R259" s="2" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
       <c r="S259" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -31414,6 +31509,11 @@
           <t>250</t>
         </is>
       </c>
+      <c r="R260" s="2" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
       <c r="S260" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -31516,6 +31616,11 @@
           <t>99</t>
         </is>
       </c>
+      <c r="R261" s="2" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
       <c r="S261" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -31603,6 +31708,11 @@
           <t>160</t>
         </is>
       </c>
+      <c r="R262" s="2" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
       <c r="S262" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -31695,6 +31805,11 @@
           <t>193</t>
         </is>
       </c>
+      <c r="R263" s="2" t="inlineStr">
+        <is>
+          <t>193</t>
+        </is>
+      </c>
       <c r="S263" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -31787,6 +31902,11 @@
           <t>148</t>
         </is>
       </c>
+      <c r="R264" s="2" t="inlineStr">
+        <is>
+          <t>148</t>
+        </is>
+      </c>
       <c r="S264" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -31879,6 +31999,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="R265" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
       <c r="S265" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -31971,6 +32096,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="R266" s="2" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
       <c r="S266" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -32063,6 +32193,11 @@
           <t>250</t>
         </is>
       </c>
+      <c r="R267" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
       <c r="S267" s="2" t="inlineStr">
         <is>
           <t>40% at 80% AMI</t>
@@ -32170,6 +32305,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="R268" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
       <c r="S268" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -32277,6 +32417,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="R269" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="S269" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -32369,6 +32514,11 @@
           <t>615</t>
         </is>
       </c>
+      <c r="R270" s="2" t="inlineStr">
+        <is>
+          <t>615</t>
+        </is>
+      </c>
       <c r="S270" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -32456,6 +32606,11 @@
           <t>Kingdom Development, Inc.</t>
         </is>
       </c>
+      <c r="R271" s="2" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
       <c r="S271" s="2" t="inlineStr">
         <is>
           <t>40% at 80% AMI</t>
@@ -32558,6 +32713,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="R272" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="S272" s="2" t="inlineStr">
         <is>
           <t>at 80% AMI</t>
@@ -32660,6 +32820,11 @@
           <t>687</t>
         </is>
       </c>
+      <c r="R273" s="2" t="inlineStr">
+        <is>
+          <t>687</t>
+        </is>
+      </c>
       <c r="S273" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -32752,6 +32917,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="R274" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
       <c r="S274" s="2" t="inlineStr">
         <is>
           <t>81% at 80% AMI</t>
@@ -32859,6 +33029,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="R275" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="S275" s="2" t="inlineStr">
         <is>
           <t>at 80% AMI</t>
@@ -32966,6 +33141,11 @@
           <t>687</t>
         </is>
       </c>
+      <c r="R276" s="2" t="inlineStr">
+        <is>
+          <t>687</t>
+        </is>
+      </c>
       <c r="S276" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -33058,6 +33238,11 @@
           <t>302</t>
         </is>
       </c>
+      <c r="R277" s="2" t="inlineStr">
+        <is>
+          <t>302</t>
+        </is>
+      </c>
       <c r="S277" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -33150,6 +33335,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="R278" s="2" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
       <c r="S278" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -33252,6 +33442,11 @@
           <t>99</t>
         </is>
       </c>
+      <c r="R279" s="2" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
       <c r="S279" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -33344,6 +33539,11 @@
           <t>208</t>
         </is>
       </c>
+      <c r="R280" s="2" t="inlineStr">
+        <is>
+          <t>208</t>
+        </is>
+      </c>
       <c r="S280" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -33436,6 +33636,11 @@
           <t>148</t>
         </is>
       </c>
+      <c r="R281" s="2" t="inlineStr">
+        <is>
+          <t>148</t>
+        </is>
+      </c>
       <c r="S281" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -33528,6 +33733,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="R282" s="2" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
       <c r="S282" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -33630,6 +33840,11 @@
           <t>99</t>
         </is>
       </c>
+      <c r="R283" s="2" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
       <c r="S283" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -33727,6 +33942,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="R284" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="S284" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -33819,6 +34039,11 @@
           <t>90</t>
         </is>
       </c>
+      <c r="R285" s="2" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
       <c r="S285" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -33993,6 +34218,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="R287" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
       <c r="S287" s="2" t="inlineStr">
         <is>
           <t>21% at 80% AMI</t>
@@ -34085,6 +34315,11 @@
           <t>101</t>
         </is>
       </c>
+      <c r="R288" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
       <c r="S288" s="2" t="inlineStr">
         <is>
           <t>40% at 80% AMI</t>
@@ -34187,6 +34422,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="R289" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="S289" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -34279,6 +34519,11 @@
           <t>206</t>
         </is>
       </c>
+      <c r="R290" s="2" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
       <c r="S290" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -34371,6 +34616,11 @@
           <t>192</t>
         </is>
       </c>
+      <c r="R291" s="2" t="inlineStr">
+        <is>
+          <t>192</t>
+        </is>
+      </c>
       <c r="S291" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -34525,6 +34775,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="R293" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="S293" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -34617,6 +34872,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="R294" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="S294" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -34709,6 +34969,11 @@
           <t>151</t>
         </is>
       </c>
+      <c r="R295" s="2" t="inlineStr">
+        <is>
+          <t>151</t>
+        </is>
+      </c>
       <c r="S295" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -34883,6 +35148,11 @@
           <t>122</t>
         </is>
       </c>
+      <c r="R297" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="S297" s="2" t="inlineStr">
         <is>
           <t>20% at 60% AMI; 80% at 80% AMI</t>
@@ -34980,6 +35250,11 @@
           <t>112</t>
         </is>
       </c>
+      <c r="R298" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="S298" s="2" t="inlineStr">
         <is>
           <t>20% at 60% AMI; 80% at 80% AMI</t>
@@ -35072,6 +35347,11 @@
           <t>99</t>
         </is>
       </c>
+      <c r="R299" s="2" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
+      </c>
       <c r="S299" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -35164,6 +35444,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="R300" s="2" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
       <c r="S300" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -35261,6 +35546,11 @@
           <t>122</t>
         </is>
       </c>
+      <c r="R301" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="S301" s="2" t="inlineStr">
         <is>
           <t>20% at 60% AMI; 80% at 80% AMI</t>
@@ -35358,6 +35648,11 @@
           <t>112</t>
         </is>
       </c>
+      <c r="R302" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="S302" s="2" t="inlineStr">
         <is>
           <t>20% at 60% AMI; 80% at 80% AMI</t>
@@ -35450,6 +35745,11 @@
           <t>164</t>
         </is>
       </c>
+      <c r="R303" s="2" t="inlineStr">
+        <is>
+          <t>164</t>
+        </is>
+      </c>
       <c r="S303" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -35542,6 +35842,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="R304" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
       <c r="S304" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -35619,6 +35924,11 @@
           <t>128</t>
         </is>
       </c>
+      <c r="R305" s="2" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
       <c r="S305" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -35702,6 +36012,11 @@
         </is>
       </c>
       <c r="Q306" s="2" t="inlineStr">
+        <is>
+          <t>148</t>
+        </is>
+      </c>
+      <c r="R306" s="2" t="inlineStr">
         <is>
           <t>148</t>
         </is>

</xml_diff>

<commit_message>
Split combined investors; prune formatting-noise overrides (Drew-approved)
- 'A / B' applicant strings now split into investor_1/investor_2
  (7 rows; exact two-part ' / ' split only). Nonprofit stays unsplit —
  which half is the nonprofit is a judgment the collaborator makes.
- Dropped 39 overrides whose values matched generated data after
  field-aware normalization (addresses differing only by abbreviation
  or missing city/zip, 'The '-prefix names, legal-suffix variants,
  typos where the DOCUMENT was right) plus 4 made redundant by the
  investor split. Kept genuine corrections: Kingsley (agenda typo),
  #18's investor/nonprofit split attribution, Bedford's full name,
  #78's investor ordering.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -466,7 +466,7 @@
     <col width="38" customWidth="1" min="16" max="16"/>
     <col width="30" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="35" customWidth="1" min="19" max="19"/>
+    <col width="38" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="17" customWidth="1" min="22" max="22"/>
@@ -1984,9 +1984,9 @@
           <t>820 MacArthur Apartments</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2019 Ozone Affordable Housing</t>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2019 Ozone Affordable Housing – 820 MacArthur, LP</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -2532,9 +2532,9 @@
           <t>Premiere Hollywood Apartments</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>OODB2, LP</t>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>OODB2, LP, a Washington Limited Partnership</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>built:collaborator-sheet; manual_status:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
+          <t>built:collaborator-sheet; manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -2669,9 +2669,9 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Affordable Housing Alliance II, Inc. dba Integrity Housing</t>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Affordable Housing Alliance II, Inc., d/b/a Integrity Housing, a Colorado nonprofit corporation</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -3003,21 +3003,21 @@
           <t>2-CMFA-Minutes-06-07-24.pdf</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr">
+      <c r="Q19" s="2" t="inlineStr">
         <is>
           <t>AOF</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>Pacific Affordable Housing Corp.</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
         <is>
           <t>Pacific Affordable Housing Corp</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>Pacific Affordable Housing Corp</t>
-        </is>
-      </c>
       <c r="T19" s="2" t="inlineStr">
         <is>
           <t>103</t>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; built:collaborator-sheet; scc_filed:collaborator-sheet; city:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>built:collaborator-sheet; scc_filed:collaborator-sheet; city:collaborator-sheet; nonprofit_partner:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -6556,9 +6556,9 @@
           <t>Eleos Ventures, LLC</t>
         </is>
       </c>
-      <c r="S45" t="inlineStr">
-        <is>
-          <t>Step Forward Comminities</t>
+      <c r="S45" s="2" t="inlineStr">
+        <is>
+          <t>Step Forward Communities</t>
         </is>
       </c>
       <c r="T45" s="2" t="inlineStr">
@@ -6613,7 +6613,7 @@
       </c>
       <c r="AJ45" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; nonprofit_partner:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -7186,9 +7186,9 @@
           <t>CMFA</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Summerwood Apartments Homes Apartments</t>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Summerwood Apartment Homes</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -7298,7 +7298,7 @@
       </c>
       <c r="AJ50" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; property_name:collaborator-sheet; entity:collaborator-sheet; investor_1:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; entity:collaborator-sheet; investor_1:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -8210,14 +8210,14 @@
           <t>CMFA-Minutes-12-13-2024.pdf</t>
         </is>
       </c>
-      <c r="Q57" t="inlineStr">
-        <is>
-          <t>Bridge Housing</t>
-        </is>
-      </c>
-      <c r="S57" t="inlineStr">
-        <is>
-          <t>Bridge Housing</t>
+      <c r="Q57" s="2" t="inlineStr">
+        <is>
+          <t>BRIDGE Housing Corporation</t>
+        </is>
+      </c>
+      <c r="S57" s="2" t="inlineStr">
+        <is>
+          <t>BRIDGE Housing Corporation</t>
         </is>
       </c>
       <c r="T57" s="2" t="inlineStr">
@@ -8267,7 +8267,7 @@
       </c>
       <c r="AJ57" t="inlineStr">
         <is>
-          <t>leasing_link:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; address:collaborator-sheet</t>
+          <t>leasing_link:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -12068,9 +12068,9 @@
           <t>569 W. 6th Street. Apartments</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>SIOF 5 Properties, LP, California limited partnership</t>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>SIOF 5 Properties, LP, a California limited partnership</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -12180,7 +12180,7 @@
       </c>
       <c r="AJ86" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -12200,9 +12200,9 @@
           <t>685 W. 4th St Apartments</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>2 SIOF 685 W Fourth St, LP, Delaware limited partnership</t>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>2 SIOF 685 W Fourth St, LP, a Delaware limited partnership</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
@@ -12312,7 +12312,7 @@
       </c>
       <c r="AJ87" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -12387,12 +12387,12 @@
           <t>2-CMFA-Minutes-06-27-2025.pdf</t>
         </is>
       </c>
-      <c r="Q88" t="inlineStr">
-        <is>
-          <t>Vintage Housing Holdings</t>
-        </is>
-      </c>
-      <c r="R88" t="inlineStr">
+      <c r="Q88" s="2" t="inlineStr">
+        <is>
+          <t>Vintage Housing Holdings, LLC</t>
+        </is>
+      </c>
+      <c r="R88" s="2" t="inlineStr">
         <is>
           <t>Kennedy Wilson</t>
         </is>
@@ -12454,7 +12454,7 @@
       </c>
       <c r="AJ88" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; scc_filed:collaborator-sheet; investor_1:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -13189,16 +13189,16 @@
           <t>2-CMFA-Minutes-08-08-25.pdf</t>
         </is>
       </c>
-      <c r="Q94" t="inlineStr">
+      <c r="Q94" s="2" t="inlineStr">
+        <is>
+          <t>BRIDGE Housing Corporation</t>
+        </is>
+      </c>
+      <c r="S94" t="inlineStr">
         <is>
           <t>BRIDGE Housing Corp.</t>
         </is>
       </c>
-      <c r="S94" t="inlineStr">
-        <is>
-          <t>BRIDGE Housing Corp.</t>
-        </is>
-      </c>
       <c r="T94" s="2" t="inlineStr">
         <is>
           <t>148</t>
@@ -13246,7 +13246,7 @@
       </c>
       <c r="AJ94" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; resolution:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; resolution:collaborator-sheet; nonprofit_partner:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -13468,9 +13468,9 @@
           <t>Belveron Partners</t>
         </is>
       </c>
-      <c r="S96" t="inlineStr">
-        <is>
-          <t>Las Palmas Housing &amp; Development Corp.</t>
+      <c r="S96" s="2" t="inlineStr">
+        <is>
+          <t>Las Palmas Housing &amp; Development Corporation</t>
         </is>
       </c>
       <c r="T96" s="2" t="inlineStr">
@@ -13530,7 +13530,7 @@
       </c>
       <c r="AJ96" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; acquisition_date:collaborator-sheet; link:collaborator-sheet; scc_filed:collaborator-sheet; resolution:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_2:collaborator-sheet; acquisition_date:collaborator-sheet; link:collaborator-sheet; scc_filed:collaborator-sheet; resolution:collaborator-sheet; investor_1:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -18853,9 +18853,9 @@
           <t>Grant of $5,000</t>
         </is>
       </c>
-      <c r="Z136" t="inlineStr">
-        <is>
-          <t>5805 Charlotte Drive, San Jose, CA 95123</t>
+      <c r="Z136" s="2" t="inlineStr">
+        <is>
+          <t>5805 Charlotte Drive, San Jose, CA</t>
         </is>
       </c>
       <c r="AA136" s="2" t="inlineStr">
@@ -18870,7 +18870,7 @@
       </c>
       <c r="AJ136" t="inlineStr">
         <is>
-          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -19667,9 +19667,9 @@
           <t>CMFA</t>
         </is>
       </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>Coliseum Transit Village</t>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>Coliseum Connections Transit Village Apartments</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
@@ -19789,7 +19789,7 @@
       </c>
       <c r="AJ143" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; property_name:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -20195,9 +20195,9 @@
           <t>CMFA</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>Coliseum Connections</t>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>Coliseum Connections Transit Village Apartments</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
@@ -20322,7 +20322,7 @@
       </c>
       <c r="AJ147" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; manual_status:collaborator-sheet; property_name:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; scc_filed:collaborator-sheet; manual_status:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -20616,9 +20616,9 @@
           <t>CMFA</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>Langham Apartments</t>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>The Langham Apartments</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -20738,7 +20738,7 @@
       </c>
       <c r="AJ150" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; property_name:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -20753,9 +20753,9 @@
           <t>CMFA</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>Piccadilly Apartments</t>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>The Piccadilly Apartments</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -20875,7 +20875,7 @@
       </c>
       <c r="AJ151" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; property_name:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -25761,9 +25761,9 @@
           <t>Highlands Point Apartments</t>
         </is>
       </c>
-      <c r="D190" t="inlineStr">
-        <is>
-          <t>St. Anton Highland, LP</t>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>St. Anton Highlands LP</t>
         </is>
       </c>
       <c r="E190" s="2" t="inlineStr">
@@ -25873,7 +25873,7 @@
       </c>
       <c r="AJ190" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -27945,9 +27945,9 @@
           <t>Grant of $5,000</t>
         </is>
       </c>
-      <c r="Z207" t="inlineStr">
-        <is>
-          <t>2625 Cullen St, Los Angeles, CA 90034</t>
+      <c r="Z207" s="2" t="inlineStr">
+        <is>
+          <t>2625 Cullen Street, Los Angeles, CA</t>
         </is>
       </c>
       <c r="AA207" s="2" t="inlineStr">
@@ -27962,7 +27962,7 @@
       </c>
       <c r="AJ207" t="inlineStr">
         <is>
-          <t>manual_status:collaborator-sheet; investor_1:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>manual_status:collaborator-sheet; investor_1:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -28682,9 +28682,9 @@
           <t>Grant of $5,000</t>
         </is>
       </c>
-      <c r="Z213" t="inlineStr">
-        <is>
-          <t>5416 Jackson St, North Highlands, CA 95660</t>
+      <c r="Z213" s="2" t="inlineStr">
+        <is>
+          <t>5416 Jackson Street, North Highlands</t>
         </is>
       </c>
       <c r="AA213" s="2" t="inlineStr">
@@ -28699,7 +28699,7 @@
       </c>
       <c r="AJ213" t="inlineStr">
         <is>
-          <t>city:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>city:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -28804,9 +28804,9 @@
           <t>Grant of $5,000</t>
         </is>
       </c>
-      <c r="Z214" t="inlineStr">
-        <is>
-          <t>444 N Amelia Ave, San Dimas, CA 91773</t>
+      <c r="Z214" s="2" t="inlineStr">
+        <is>
+          <t>444 North Amelia Avenue, San Dimas</t>
         </is>
       </c>
       <c r="AA214" s="2" t="inlineStr">
@@ -28826,7 +28826,7 @@
       </c>
       <c r="AJ214" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -28936,9 +28936,9 @@
           <t>Grant of $5,000</t>
         </is>
       </c>
-      <c r="Z215" t="inlineStr">
-        <is>
-          <t>511 N. Hoover Street, Los Angeles, California</t>
+      <c r="Z215" s="2" t="inlineStr">
+        <is>
+          <t>511 N. Hoover Street, Los Angeles</t>
         </is>
       </c>
       <c r="AA215" s="2" t="inlineStr">
@@ -28963,7 +28963,7 @@
       </c>
       <c r="AJ215" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; link:collaborator-sheet; resolution:collaborator-sheet; investor_1:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; link:collaborator-sheet; resolution:collaborator-sheet; investor_1:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -29840,9 +29840,9 @@
           <t>Grant of $5,000</t>
         </is>
       </c>
-      <c r="Z222" t="inlineStr">
-        <is>
-          <t>16077 Ashland Ave, San Lorenzo, CA 94580</t>
+      <c r="Z222" s="2" t="inlineStr">
+        <is>
+          <t>16077 Ashland Avenue, San Lorenzo</t>
         </is>
       </c>
       <c r="AA222" s="2" t="inlineStr">
@@ -29857,7 +29857,7 @@
       </c>
       <c r="AJ222" t="inlineStr">
         <is>
-          <t>city:collaborator-sheet; investor_1:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>city:collaborator-sheet; investor_1:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -30019,9 +30019,9 @@
           <t>Grant of $5,000</t>
         </is>
       </c>
-      <c r="Z224" t="inlineStr">
-        <is>
-          <t>1454 W Florence Ave, Los Angeles, CA 90047</t>
+      <c r="Z224" s="2" t="inlineStr">
+        <is>
+          <t>1454 West Florence Avenue, Los Angeles, CA</t>
         </is>
       </c>
       <c r="AA224" s="2" t="inlineStr">
@@ -30041,7 +30041,7 @@
       </c>
       <c r="AJ224" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; investor_1:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; investor_1:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -30061,9 +30061,9 @@
           <t>Bennington Apartments</t>
         </is>
       </c>
-      <c r="D225" t="inlineStr">
-        <is>
-          <t>CG Bennington, LP / JSP Bennington, LP</t>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>CG Bennington, LP and JSP Bennington, LP</t>
         </is>
       </c>
       <c r="E225" s="2" t="inlineStr">
@@ -30158,7 +30158,7 @@
       </c>
       <c r="AJ225" t="inlineStr">
         <is>
-          <t>entity:collaborator-sheet; address:collaborator-sheet; term_years:collaborator-sheet</t>
+          <t>address:collaborator-sheet; term_years:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -30263,9 +30263,9 @@
           <t>Grant of $5,000</t>
         </is>
       </c>
-      <c r="Z226" t="inlineStr">
-        <is>
-          <t>142 Fig Tree Lane, Martinez, CA 94553</t>
+      <c r="Z226" s="2" t="inlineStr">
+        <is>
+          <t>142 Fig Tree Lane, Martinez, CA</t>
         </is>
       </c>
       <c r="AA226" s="2" t="inlineStr">
@@ -30280,7 +30280,7 @@
       </c>
       <c r="AJ226" t="inlineStr">
         <is>
-          <t>manual_status:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; term_years:collaborator-sheet</t>
+          <t>manual_status:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; term_years:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -30467,9 +30467,9 @@
           <t>Positive Investments, Inc.</t>
         </is>
       </c>
-      <c r="S228" t="inlineStr">
-        <is>
-          <t>Foundation for Affordable Housing</t>
+      <c r="S228" s="2" t="inlineStr">
+        <is>
+          <t>The Foundation for Affordable Housing</t>
         </is>
       </c>
       <c r="T228" s="2" t="inlineStr">
@@ -30514,7 +30514,7 @@
       </c>
       <c r="AJ228" t="inlineStr">
         <is>
-          <t>investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; term_years:collaborator-sheet</t>
+          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet; term_years:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -30619,9 +30619,9 @@
           <t>Grant of $5,000</t>
         </is>
       </c>
-      <c r="Z229" t="inlineStr">
-        <is>
-          <t>220 47th St, San Diego, CA 92102</t>
+      <c r="Z229" s="2" t="inlineStr">
+        <is>
+          <t>220 47th Street, San Diego</t>
         </is>
       </c>
       <c r="AA229" s="2" t="inlineStr">
@@ -30636,7 +30636,7 @@
       </c>
       <c r="AJ229" t="inlineStr">
         <is>
-          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -30651,9 +30651,9 @@
           <t>CSCDA</t>
         </is>
       </c>
-      <c r="C230" t="inlineStr">
-        <is>
-          <t>Hansen illage Apartments</t>
+      <c r="C230" s="2" t="inlineStr">
+        <is>
+          <t>Hansen Village Apartments</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -30706,9 +30706,9 @@
           <t>Positive Investments, Inc.</t>
         </is>
       </c>
-      <c r="S230" t="inlineStr">
-        <is>
-          <t>Foundation for Affordable Housing</t>
+      <c r="S230" s="2" t="inlineStr">
+        <is>
+          <t>The Foundation for Affordable Housing</t>
         </is>
       </c>
       <c r="T230" s="2" t="inlineStr">
@@ -30758,7 +30758,7 @@
       </c>
       <c r="AJ230" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; property_name:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; investor_1:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -30863,9 +30863,9 @@
           <t>Grant of $5,000</t>
         </is>
       </c>
-      <c r="Z231" t="inlineStr">
-        <is>
-          <t>160 S Virgil Ave, Los Angeles, CA 90004</t>
+      <c r="Z231" s="2" t="inlineStr">
+        <is>
+          <t>160 S. Virgil Avenue, Los Angeles</t>
         </is>
       </c>
       <c r="AA231" s="2" t="inlineStr">
@@ -30880,7 +30880,7 @@
       </c>
       <c r="AJ231" t="inlineStr">
         <is>
-          <t>investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -30980,9 +30980,9 @@
           <t>Grant of $5,000</t>
         </is>
       </c>
-      <c r="Z232" t="inlineStr">
-        <is>
-          <t>12091 Bayport St, Garden Grove, CA 92840</t>
+      <c r="Z232" s="2" t="inlineStr">
+        <is>
+          <t>12091 Bayport Street, Garden Grove, CA</t>
         </is>
       </c>
       <c r="AA232" s="2" t="inlineStr">
@@ -31007,7 +31007,7 @@
       </c>
       <c r="AJ232" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; link:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; link:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -31112,9 +31112,9 @@
           <t>Grant of $5,000</t>
         </is>
       </c>
-      <c r="Z233" t="inlineStr">
-        <is>
-          <t>926 S Kingsley Dr, Los Angeles, CA 90006</t>
+      <c r="Z233" s="2" t="inlineStr">
+        <is>
+          <t>926 S. Kingsley Drive, Los Angeles, CA</t>
         </is>
       </c>
       <c r="AA233" s="2" t="inlineStr">
@@ -31129,7 +31129,7 @@
       </c>
       <c r="AJ233" t="inlineStr">
         <is>
-          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; term_years:collaborator-sheet</t>
+          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet; term_years:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -31234,9 +31234,9 @@
           <t>Grant of $5,000</t>
         </is>
       </c>
-      <c r="Z234" t="inlineStr">
-        <is>
-          <t>939 S Kingsley Dr, Los Angeles, CA 90006</t>
+      <c r="Z234" s="2" t="inlineStr">
+        <is>
+          <t>939 S. Kingsley Drive, Los Angeles, CA</t>
         </is>
       </c>
       <c r="AA234" s="2" t="inlineStr">
@@ -31251,7 +31251,7 @@
       </c>
       <c r="AJ234" t="inlineStr">
         <is>
-          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -31478,9 +31478,9 @@
           <t>Grant of $5,000</t>
         </is>
       </c>
-      <c r="Z236" t="inlineStr">
-        <is>
-          <t>6985 S. Centinela Avenue, Los Angeles, CA 90045</t>
+      <c r="Z236" s="2" t="inlineStr">
+        <is>
+          <t>6985 S. Centinela Avenue, Los Angeles, CA</t>
         </is>
       </c>
       <c r="AA236" s="2" t="inlineStr">
@@ -31500,7 +31500,7 @@
       </c>
       <c r="AJ236" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; investor_1:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; investor_1:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -31605,9 +31605,9 @@
           <t>Grant of $5,000</t>
         </is>
       </c>
-      <c r="Z237" t="inlineStr">
-        <is>
-          <t>1178 N Edgemont St, Los Angeles, CA 90029</t>
+      <c r="Z237" s="2" t="inlineStr">
+        <is>
+          <t>1178 N. Edgemont Street, Los Angeles, CA</t>
         </is>
       </c>
       <c r="AA237" s="2" t="inlineStr">
@@ -31622,7 +31622,7 @@
       </c>
       <c r="AJ237" t="inlineStr">
         <is>
-          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -35377,7 +35377,12 @@
       </c>
       <c r="Q272" s="2" t="inlineStr">
         <is>
-          <t>Vintage Housing Holdings, LLC / Kennedy Wilson</t>
+          <t>Vintage Housing Holdings, LLC</t>
+        </is>
+      </c>
+      <c r="R272" s="2" t="inlineStr">
+        <is>
+          <t>Kennedy Wilson</t>
         </is>
       </c>
       <c r="S272" s="2" t="inlineStr">
@@ -35494,7 +35499,12 @@
       </c>
       <c r="Q273" s="2" t="inlineStr">
         <is>
-          <t>Vintage Housing Holdings, LLC / Kennedy Wilson</t>
+          <t>Vintage Housing Holdings, LLC</t>
+        </is>
+      </c>
+      <c r="R273" s="2" t="inlineStr">
+        <is>
+          <t>Kennedy Wilson</t>
         </is>
       </c>
       <c r="S273" s="2" t="inlineStr">
@@ -35723,7 +35733,12 @@
       </c>
       <c r="Q275" s="2" t="inlineStr">
         <is>
-          <t>Vintage Housing Holdings, LLC / Kennedy Wilson</t>
+          <t>Vintage Housing Holdings, LLC</t>
+        </is>
+      </c>
+      <c r="R275" s="2" t="inlineStr">
+        <is>
+          <t>Kennedy Wilson</t>
         </is>
       </c>
       <c r="S275" s="2" t="inlineStr">
@@ -35845,7 +35860,12 @@
       </c>
       <c r="Q276" s="2" t="inlineStr">
         <is>
-          <t>Vintage Housing Holdings, LLC / Kennedy Wilson</t>
+          <t>Vintage Housing Holdings, LLC</t>
+        </is>
+      </c>
+      <c r="R276" s="2" t="inlineStr">
+        <is>
+          <t>Kennedy Wilson</t>
         </is>
       </c>
       <c r="S276" s="2" t="inlineStr">
@@ -72484,7 +72504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C168"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -73078,12 +73098,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>entity: generated '2019 Ozone Affordable Housing – 820 MacArthur, LP' -&gt; manual '2019 Ozone Affordable Housing'</t>
+          <t>nonprofit_partner: generated 'AOF / Pacific Affordable Housing Corp.' -&gt; manual 'Pacific Affordable Housing Corp'</t>
         </is>
       </c>
     </row>
@@ -73095,12 +73115,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>34</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>entity: generated 'OODB2, LP, a Washington Limited Partnership' -&gt; manual 'OODB2, LP'</t>
+          <t>city: generated 'Los Angeles' -&gt; manual 'El Sobrante'</t>
         </is>
       </c>
     </row>
@@ -73112,12 +73132,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>34</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>entity: generated 'Affordable Housing Alliance II, Inc., d/b/a Integrity Housing, a Colorado nonprofit corporation' -&gt; manual 'Affordable Housing Alliance II, Inc. dba Integrity Housing'</t>
+          <t>county: generated 'Los Angeles' -&gt; manual 'Contra Costa'</t>
         </is>
       </c>
     </row>
@@ -73129,12 +73149,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>27</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>investor_1: generated 'AOF / Pacific Affordable Housing Corp.' -&gt; manual 'AOF'</t>
+          <t>total_units: generated '24' -&gt; manual '52'</t>
         </is>
       </c>
     </row>
@@ -73146,12 +73166,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>28</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>nonprofit_partner: generated 'AOF / Pacific Affordable Housing Corp.' -&gt; manual 'Pacific Affordable Housing Corp'</t>
+          <t>total_units: generated '22' -&gt; manual '72'</t>
         </is>
       </c>
     </row>
@@ -73163,12 +73183,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>29</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>city: generated 'Los Angeles' -&gt; manual 'El Sobrante'</t>
+          <t>total_units: generated '24' -&gt; manual '48'</t>
         </is>
       </c>
     </row>
@@ -73180,12 +73200,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>county: generated 'Los Angeles' -&gt; manual 'Contra Costa'</t>
+          <t>total_units: generated '65' -&gt; manual '165'</t>
         </is>
       </c>
     </row>
@@ -73197,12 +73217,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>37</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>total_units: generated '24' -&gt; manual '52'</t>
+          <t>property_name: generated '2330 3rd Street Apartments' -&gt; manual '2330 E. 3rd Street Apartments'</t>
         </is>
       </c>
     </row>
@@ -73214,12 +73234,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>48</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>total_units: generated '22' -&gt; manual '72'</t>
+          <t>investor_1: generated 'Ethos Real Estate' -&gt; manual 'Vistria Group'</t>
         </is>
       </c>
     </row>
@@ -73231,12 +73251,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>51</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>total_units: generated '24' -&gt; manual '48'</t>
+          <t>total_units: generated '144' -&gt; manual '145'</t>
         </is>
       </c>
     </row>
@@ -73248,12 +73268,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>54</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>total_units: generated '65' -&gt; manual '165'</t>
+          <t>total_units: generated '42' -&gt; manual '356'</t>
         </is>
       </c>
     </row>
@@ -73265,12 +73285,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>property_name: generated '2330 3rd Street Apartments' -&gt; manual '2330 E. 3rd Street Apartments'</t>
+          <t>entity: generated 'PREG 5150 ECR Los Altos, LP, a California limited partnership' -&gt; manual 'Prometheus Real Estate Group'</t>
         </is>
       </c>
     </row>
@@ -73282,12 +73302,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Ethos Real Estate' -&gt; manual 'Vistria Group'</t>
+          <t>total_units: generated '29' -&gt; manual '196'</t>
         </is>
       </c>
     </row>
@@ -73299,12 +73319,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>76</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>nonprofit_partner: generated 'Step Forward Communities' -&gt; manual 'Step Forward Comminities'</t>
+          <t>entity: generated '3 SIOF 1451 W MLK BLVD, LP' -&gt; manual '1451 W. MLK Boulevard Apartments'</t>
         </is>
       </c>
     </row>
@@ -73316,12 +73336,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>78</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>total_units: generated '144' -&gt; manual '145'</t>
+          <t>investor_1: generated 'Vintage Housing Holdings, LLC' -&gt; manual 'Kennedy Wilson'</t>
         </is>
       </c>
     </row>
@@ -73333,12 +73353,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>78</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>total_units: generated '42' -&gt; manual '356'</t>
+          <t>nonprofit_partner: generated 'Pacific Housing, Inc.' -&gt; manual 'Hearthstone Housing Foundation'</t>
         </is>
       </c>
     </row>
@@ -73350,12 +73370,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>78</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>investor_1: generated 'BRIDGE Housing Corporation' -&gt; manual 'Bridge Housing'</t>
+          <t>total_units: generated '8' -&gt; manual '1008'</t>
         </is>
       </c>
     </row>
@@ -73367,12 +73387,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>81</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>nonprofit_partner: generated 'BRIDGE Housing Corporation' -&gt; manual 'Bridge Housing'</t>
+          <t>total_units: generated '32' -&gt; manual '31'</t>
         </is>
       </c>
     </row>
@@ -73384,12 +73404,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>81</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>entity: generated 'PREG 5150 ECR Los Altos, LP, a California limited partnership' -&gt; manual 'Prometheus Real Estate Group'</t>
+          <t>city_cut: generated '4650.0' -&gt; manual '4500'</t>
         </is>
       </c>
     </row>
@@ -73401,12 +73421,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>79</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>total_units: generated '29' -&gt; manual '196'</t>
+          <t>entity: generated '2 SIOF 10811 S Compton Ave, LP' -&gt; manual '10811 S. Compton Ave Apartments'</t>
         </is>
       </c>
     </row>
@@ -73418,12 +73438,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>158</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>entity: generated '3 SIOF 1451 W MLK BLVD, LP' -&gt; manual '1451 W. MLK Boulevard Apartments'</t>
+          <t>total_units: generated '30' -&gt; manual '29'</t>
         </is>
       </c>
     </row>
@@ -73435,12 +73455,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>95</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Vintage Housing Holdings, LLC / Kennedy Wilson' -&gt; manual 'Kennedy Wilson'</t>
+          <t>investor_1: generated 'Belveron Partners' -&gt; manual 'Sack Capital Partners'</t>
         </is>
       </c>
     </row>
@@ -73452,12 +73472,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>110</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>nonprofit_partner: generated 'Pacific Housing, Inc.' -&gt; manual 'Hearthstone Housing Foundation'</t>
+          <t>total_units: generated '24' -&gt; manual '42'</t>
         </is>
       </c>
     </row>
@@ -73469,12 +73489,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>120</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>total_units: generated '8' -&gt; manual '1008'</t>
+          <t>city: generated 'Sacramento' -&gt; manual 'Unincorporated'</t>
         </is>
       </c>
     </row>
@@ -73486,12 +73506,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>125</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>total_units: generated '32' -&gt; manual '31'</t>
+          <t>property_name: generated 'Kinglsey Apartments' -&gt; manual 'Kingsley Apartments'</t>
         </is>
       </c>
     </row>
@@ -73503,12 +73523,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>134</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>city_cut: generated '4650.0' -&gt; manual '4500'</t>
+          <t>total_units: generated '69' -&gt; manual '68'</t>
         </is>
       </c>
     </row>
@@ -73520,12 +73540,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>137</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>entity: generated '2 SIOF 10811 S Compton Ave, LP' -&gt; manual '10811 S. Compton Ave Apartments'</t>
+          <t>total_units: generated '42' -&gt; manual '41'</t>
         </is>
       </c>
     </row>
@@ -73537,12 +73557,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>138</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>entity: generated 'SIOF 5 Properties, LP, a California limited partnership' -&gt; manual 'SIOF 5 Properties, LP, California limited partnership'</t>
+          <t>city: generated 'Santa Clara' -&gt; manual 'San Jose'</t>
         </is>
       </c>
     </row>
@@ -73554,12 +73574,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>152</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>entity: generated '2 SIOF 685 W Fourth St, LP, a Delaware limited partnership' -&gt; manual '2 SIOF 685 W Fourth St, LP, Delaware limited partnership'</t>
+          <t>total_units: generated '52' -&gt; manual '152'</t>
         </is>
       </c>
     </row>
@@ -73571,12 +73591,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>155</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Vintage Housing Holdings, LLC / Kennedy Wilson' -&gt; manual 'Vintage Housing Holdings'</t>
+          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
         </is>
       </c>
     </row>
@@ -73588,12 +73608,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>156</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>total_units: generated '30' -&gt; manual '29'</t>
+          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
         </is>
       </c>
     </row>
@@ -73605,12 +73625,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>171</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Belveron Partners' -&gt; manual 'Sack Capital Partners'</t>
+          <t>city_cut: generated '15900.0' -&gt; manual '6300'</t>
         </is>
       </c>
     </row>
@@ -73622,12 +73642,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>181</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>nonprofit_partner: generated 'Las Palmas Housing &amp; Development Corporation' -&gt; manual 'Las Palmas Housing &amp; Development Corp.'</t>
+          <t>city: generated 'Long Beach' -&gt; manual 'Los Angeles'</t>
         </is>
       </c>
     </row>
@@ -73639,12 +73659,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>181</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>investor_1: generated 'BRIDGE Housing Corporation' -&gt; manual 'BRIDGE Housing Corp.'</t>
+          <t>total_units: generated '52' -&gt; manual '152'</t>
         </is>
       </c>
     </row>
@@ -73656,12 +73676,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>144</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>total_units: generated '24' -&gt; manual '42'</t>
+          <t>property_name: generated 'La Vista Apartments' -&gt; manual 'La Vista Apartment Homes'</t>
         </is>
       </c>
     </row>
@@ -73673,12 +73693,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>195</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>city: generated 'Sacramento' -&gt; manual 'Unincorporated'</t>
+          <t>total_units: generated '42' -&gt; manual '41'</t>
         </is>
       </c>
     </row>
@@ -73690,12 +73710,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>196</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>property_name: generated 'Kinglsey Apartments' -&gt; manual 'Kingsley Apartments'</t>
+          <t>address: generated '9750 Airport Blvd, Los Angeles, CA' -&gt; manual '9750 Airport Blvd, Westchester, CA 90045'</t>
         </is>
       </c>
     </row>
@@ -73707,12 +73727,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>199</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>total_units: generated '69' -&gt; manual '68'</t>
+          <t>city_cut: generated '5550.0' -&gt; manual '5500'</t>
         </is>
       </c>
     </row>
@@ -73724,12 +73744,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>208</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>address: generated '5805 Charlotte Drive, San Jose, CA' -&gt; manual '5805 Charlotte Drive, San Jose, CA 95123'</t>
+          <t>address: generated '2481 South Sawtelle Blvd, Los Angeles, CA' -&gt; manual '2481 Sawtelle Blvd, Los Angeles, CA 90064'</t>
         </is>
       </c>
     </row>
@@ -73741,12 +73761,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>49</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>total_units: generated '42' -&gt; manual '41'</t>
+          <t>entity: generated 'Standard Summerwood II LP' -&gt; manual 'Standard Properties'</t>
         </is>
       </c>
     </row>
@@ -73758,12 +73778,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>49</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>property_name: generated 'Coliseum Connections Transit Village Apartments' -&gt; manual 'Coliseum Transit Village'</t>
+          <t>investor_1: generated 'Standard Property Company, Inc.' -&gt; manual 'Standard Properties'</t>
         </is>
       </c>
     </row>
@@ -73775,12 +73795,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>204</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>city: generated 'Santa Clara' -&gt; manual 'San Jose'</t>
+          <t>total_units: generated '50' -&gt; manual '49'</t>
         </is>
       </c>
     </row>
@@ -73792,12 +73812,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>206</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>property_name: generated 'Coliseum Connections Transit Village Apartments' -&gt; manual 'Coliseum Connections'</t>
+          <t>county: generated 'San Diego' -&gt; manual 'Los Angeles'</t>
         </is>
       </c>
     </row>
@@ -73809,12 +73829,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>209</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>property_name: generated 'The Langham Apartments' -&gt; manual 'Langham Apartments'</t>
+          <t>investor_1: generated 'Zenith Property Group LLC' -&gt; manual 'Red Stone Equity Partners'</t>
         </is>
       </c>
     </row>
@@ -73826,12 +73846,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>151</t>
+          <t>209</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>property_name: generated 'The Piccadilly Apartments' -&gt; manual 'Piccadilly Apartments'</t>
+          <t>term_years: generated '35' -&gt; manual '15'</t>
         </is>
       </c>
     </row>
@@ -73843,12 +73863,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>210</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>total_units: generated '52' -&gt; manual '152'</t>
+          <t>term_years: generated '55' -&gt; manual '10'</t>
         </is>
       </c>
     </row>
@@ -73860,12 +73880,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>226</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
+          <t>term_years: generated '15' -&gt; manual '10'</t>
         </is>
       </c>
     </row>
@@ -73877,12 +73897,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>228</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
+          <t>term_years: generated '10' -&gt; manual '15'</t>
         </is>
       </c>
     </row>
@@ -73894,12 +73914,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>171</t>
+          <t>230</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>city_cut: generated '15900.0' -&gt; manual '6300'</t>
+          <t>address: generated '11821 Foothill Blvd, Los Angeles, CA' -&gt; manual '11821 Foothill Blvd, Lake View Terrace, CA 91342'</t>
         </is>
       </c>
     </row>
@@ -73911,12 +73931,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>217</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>city: generated 'Long Beach' -&gt; manual 'Los Angeles'</t>
+          <t>total_units: generated '35' -&gt; manual '34'</t>
         </is>
       </c>
     </row>
@@ -73928,12 +73948,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>211</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>total_units: generated '52' -&gt; manual '152'</t>
+          <t>entity: generated 'Haven, LP' -&gt; manual 'Heven LP'</t>
         </is>
       </c>
     </row>
@@ -73945,12 +73965,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>190</t>
+          <t>211</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>entity: generated 'St. Anton Highlands LP' -&gt; manual 'St. Anton Highland, LP'</t>
+          <t>address: generated '6530 Independence Avenue, Los Angeles' -&gt; manual '6530 Independence Ave, Canoga Park, CA 91303'</t>
         </is>
       </c>
     </row>
@@ -73962,12 +73982,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>212</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>property_name: generated 'La Vista Apartments' -&gt; manual 'La Vista Apartment Homes'</t>
+          <t>address: generated '2075 West Jefferson Blvd., Los Angeles' -&gt; manual '2075 W Jefferson BlvdLos Angeles, CA 90018'</t>
         </is>
       </c>
     </row>
@@ -73979,12 +73999,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>231</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>total_units: generated '42' -&gt; manual '41'</t>
+          <t>nonprofit_partner: generated 'Bedford' -&gt; manual 'Bedford Affordable Housing Foundation'</t>
         </is>
       </c>
     </row>
@@ -73996,12 +74016,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>233</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>address: generated '9750 Airport Blvd, Los Angeles, CA' -&gt; manual '9750 Airport Blvd, Westchester, CA 90045'</t>
+          <t>term_years: generated '55' -&gt; manual '10'</t>
         </is>
       </c>
     </row>
@@ -74013,12 +74033,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>235</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>city_cut: generated '5550.0' -&gt; manual '5500'</t>
+          <t>address: generated '3950 W. Ingraham Street, Los Angeles, CA' -&gt; manual '3950 Ingraham St, San Diego, CA 92109'</t>
         </is>
       </c>
     </row>
@@ -74030,12 +74050,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>236</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>address: generated '2625 Cullen Street, Los Angeles, CA' -&gt; manual '2625 Cullen St, Los Angeles, CA 90034'</t>
+          <t>total_units: generated '136' -&gt; manual '108'</t>
         </is>
       </c>
     </row>
@@ -74047,1302 +74067,673 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>208</t>
+          <t>225</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>address: generated '2481 South Sawtelle Blvd, Los Angeles, CA' -&gt; manual '2481 Sawtelle Blvd, Los Angeles, CA 90064'</t>
+          <t>term_years: generated '30' -&gt; manual '55'</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>property_name: generated 'Summerwood Apartment Homes' -&gt; manual 'Summerwood Apartments Homes Apartments'</t>
+          <t>AIN 6020022027 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>33</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>entity: generated 'Standard Summerwood II LP' -&gt; manual 'Standard Properties'</t>
+          <t>AIN 6020022027 (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>76</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Standard Property Company, Inc.' -&gt; manual 'Standard Properties'</t>
+          <t>AIN 5036031006 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>99</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>total_units: generated '50' -&gt; manual '49'</t>
+          <t>AIN 4262018026 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>132</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>county: generated 'San Diego' -&gt; manual 'Los Angeles'</t>
+          <t>AIN 6020022027 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>224</t>
+          <t>137</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>address: generated '1454 West Florence Avenue, Los Angeles, CA' -&gt; manual '1454 W Florence Ave, Los Angeles, CA 90047'</t>
+          <t>AIN 2125017014 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>143</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Zenith Property Group LLC' -&gt; manual 'Red Stone Equity Partners'</t>
+          <t>AIN 41416654 (Alameda): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>158</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>term_years: generated '35' -&gt; manual '15'</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>182</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>term_years: generated '55' -&gt; manual '10'</t>
+          <t>AIN 5036031006 (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>196</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>address: generated '142 Fig Tree Lane, Martinez, CA' -&gt; manual '142 Fig Tree Lane, Martinez, CA 94553'</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>197</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>term_years: generated '15' -&gt; manual '10'</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>201</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>nonprofit_partner: generated 'The Foundation for Affordable Housing' -&gt; manual 'Foundation for Affordable Housing'</t>
+          <t>AIN (none) (Santa Barbara): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>206</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>term_years: generated '10' -&gt; manual '15'</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>207</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>property_name: generated 'Hansen Village Apartments' -&gt; manual 'Hansen illage Apartments'</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>208</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>nonprofit_partner: generated 'The Foundation for Affordable Housing' -&gt; manual 'Foundation for Affordable Housing'</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>215</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>address: generated '11821 Foothill Blvd, Los Angeles, CA' -&gt; manual '11821 Foothill Blvd, Lake View Terrace, CA 91342'</t>
+          <t>AIN 5539028040 (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>232</t>
+          <t>226</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>address: generated '12091 Bayport Street, Garden Grove, CA' -&gt; manual '12091 Bayport St, Garden Grove, CA 92840'</t>
+          <t>AIN (none) (Contra Costa): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>189</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>address: generated '16077 Ashland Avenue, San Lorenzo' -&gt; manual '16077 Ashland Ave, San Lorenzo, CA 94580'</t>
+          <t>AIN 46745075 (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>217</t>
+          <t>189</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>total_units: generated '35' -&gt; manual '34'</t>
+          <t>AIN 46745074 (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>215</t>
+          <t>189</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>address: generated '511 N. Hoover Street, Los Angeles' -&gt; manual '511 N. Hoover Street, Los Angeles, California'</t>
+          <t>AIN 46745073 (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>198</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>entity: generated 'Haven, LP' -&gt; manual 'Heven LP'</t>
+          <t>AIN (none) (Santa Clara): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>address: generated '6530 Independence Avenue, Los Angeles' -&gt; manual '6530 Independence Ave, Canoga Park, CA 91303'</t>
+          <t>AIN 128101150 (Solano) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>212</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>address: generated '2075 West Jefferson Blvd., Los Angeles' -&gt; manual '2075 W Jefferson BlvdLos Angeles, CA 90018'</t>
+          <t>AIN 128101050 (Solano) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>213</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>address: generated '5416 Jackson Street, North Highlands' -&gt; manual '5416 Jackson St, North Highlands, CA 95660'</t>
+          <t>AIN 128105060 (Solano) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>214</t>
+          <t>182/76</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>address: generated '444 North Amelia Avenue, San Dimas' -&gt; manual '444 N Amelia Ave, San Dimas, CA 91773'</t>
+          <t>AIN 5036031006 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>200/218</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>address: generated '220 47th Street, San Diego' -&gt; manual '220 47th St, San Diego, CA 92102'</t>
+          <t>AIN 5040021006 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>231</t>
+          <t>130/179</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>nonprofit_partner: generated 'Bedford' -&gt; manual 'Bedford Affordable Housing Foundation'</t>
+          <t>AIN 5080006008 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>231</t>
+          <t>126/173</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>address: generated '160 S. Virgil Avenue, Los Angeles' -&gt; manual '160 S Virgil Ave, Los Angeles, CA 90004'</t>
+          <t>AIN 5094005005 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>127/174</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>address: generated '926 S. Kingsley Drive, Los Angeles, CA' -&gt; manual '926 S Kingsley Dr, Los Angeles, CA 90006'</t>
+          <t>AIN 5094006003 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>122/165</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>term_years: generated '55' -&gt; manual '10'</t>
+          <t>AIN 5094017020 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>234</t>
+          <t>124/169</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>address: generated '939 S. Kingsley Drive, Los Angeles, CA' -&gt; manual '939 S Kingsley Dr, Los Angeles, CA 90006'</t>
+          <t>AIN 5094023025 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>235</t>
+          <t>128/175</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>address: generated '3950 W. Ingraham Street, Los Angeles, CA' -&gt; manual '3950 Ingraham St, San Diego, CA 92109'</t>
+          <t>AIN 5502019004 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>125/170</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>total_units: generated '136' -&gt; manual '108'</t>
+          <t>AIN 5503024012 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>129/177</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>address: generated '6985 S. Centinela Avenue, Los Angeles, CA' -&gt; manual '6985 S. Centinela Avenue, Los Angeles, CA 90045'</t>
+          <t>AIN 5517005016 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>237</t>
+          <t>121/162</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>address: generated '1178 N. Edgemont Street, Los Angeles, CA' -&gt; manual '1178 N Edgemont St, Los Angeles, CA 90029'</t>
+          <t>AIN 5518013024 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>123/168</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>entity: generated 'CG Bennington, LP and JSP Bennington, LP' -&gt; manual 'CG Bennington, LP / JSP Bennington, LP'</t>
+          <t>AIN 5518020021 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>135/220</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>term_years: generated '30' -&gt; manual '55'</t>
+          <t>AIN 5518026004 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>fetch-fallback</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>10/132</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>AIN 6020022027 (Los Angeles) has no current roll data; using manual value</t>
+          <t>AIN 6020022027 assigned to multiple projects</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>shared-ain</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>152/181</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
-        <is>
-          <t>AIN 6020022027 (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>76</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>AIN 5036031006 (Los Angeles) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>99</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>AIN 4262018026 (Los Angeles) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>132</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>AIN 6020022027 (Los Angeles) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>137</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>AIN 2125017014 (Los Angeles) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>143</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>AIN 41416654 (Alameda): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>158</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>182</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>AIN 5036031006 (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>196</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>197</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>201</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>AIN (none) (Santa Barbara): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>206</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>207</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>208</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>215</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>AIN 5539028040 (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>226</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>AIN (none) (Contra Costa): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>189</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>AIN 46745075 (Santa Clara): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>189</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>AIN 46745074 (Santa Clara): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>189</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>AIN 46745073 (Santa Clara): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>198</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>AIN (none) (Santa Clara): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>AIN 128101150 (Solano) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>AIN 128101050 (Solano) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>AIN 128105060 (Solano) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>182/76</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>AIN 5036031006 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>200/218</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>AIN 5040021006 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>130/179</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>AIN 5080006008 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>126/173</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>AIN 5094005005 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>127/174</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>AIN 5094006003 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>122/165</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>AIN 5094017020 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>124/169</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>AIN 5094023025 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>128/175</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>AIN 5502019004 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>125/170</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>AIN 5503024012 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>129/177</t>
-        </is>
-      </c>
-      <c r="C163" t="inlineStr">
-        <is>
-          <t>AIN 5517005016 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>121/162</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>AIN 5518013024 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>123/168</t>
-        </is>
-      </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>AIN 5518020021 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>135/220</t>
-        </is>
-      </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>AIN 5518026004 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>10/132</t>
-        </is>
-      </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>AIN 6020022027 assigned to multiple projects</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>shared-ain</t>
-        </is>
-      </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>152/181</t>
-        </is>
-      </c>
-      <c r="C168" t="inlineStr">
         <is>
           <t>AIN 7157012017 assigned to multiple projects</t>
         </is>

</xml_diff>

<commit_message>
Adjudicate override conflicts: documents win 9, manual wins 12
A: dropped overrides where documents/situs are authoritative (Hive is
Long Beach per situs, Montecito is Santa Clara, entity shorthands and
typos, the stale San Diego address on 3950 Ingraham). B: kept manual
values with reviewed notes (neighborhood/zip refinements, agenda
errors the collaborator caught, the Kingsley typo, nonprofit
attribution judgments) — conflicts cleared, provenance retained.
Remaining conflicts are the journalist's adjudication list.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -7522,9 +7522,9 @@
           <t>Summerwood Apartment Homes</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Standard Properties</t>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Standard Summerwood II LP</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -7572,9 +7572,9 @@
           <t>2-CMFA-Minutes-04-17-26.pdf</t>
         </is>
       </c>
-      <c r="T50" t="inlineStr">
-        <is>
-          <t>Standard Properties</t>
+      <c r="T50" s="2" t="inlineStr">
+        <is>
+          <t>Standard Property Company, Inc.</t>
         </is>
       </c>
       <c r="V50" s="2" t="inlineStr">
@@ -7629,7 +7629,7 @@
       </c>
       <c r="AL50" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; entity:collaborator-sheet; investor_1:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -9104,66 +9104,81 @@
           <t>Harken Apartments</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>PREG 5150 ECR Los Altos, LP, a California limited partnership</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Los Altos</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Santa Clara</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>25-065</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>2025-01-31</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>authorize</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>operative</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>15167</t>
+        </is>
+      </c>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-04</t>
+        </is>
+      </c>
+      <c r="Q61" s="3" t="inlineStr">
+        <is>
+          <t>1-CMFA-Agenda-1-31-2025.pdf</t>
+        </is>
+      </c>
+      <c r="R61" s="3" t="inlineStr">
+        <is>
+          <t>CMFA-Staff-Report-01-31-25.pdf</t>
+        </is>
+      </c>
+      <c r="S61" s="3" t="inlineStr">
+        <is>
+          <t>2-CMFA-Minutes-1-31-2025.pdf</t>
+        </is>
+      </c>
+      <c r="T61" s="2" t="inlineStr">
         <is>
           <t>Prometheus Real Estate Group</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>Los Altos</t>
-        </is>
-      </c>
-      <c r="F61" s="2" t="inlineStr">
-        <is>
-          <t>Santa Clara</t>
-        </is>
-      </c>
-      <c r="G61" s="2" t="inlineStr">
-        <is>
-          <t>25-065</t>
-        </is>
-      </c>
-      <c r="H61" s="2" t="inlineStr">
-        <is>
-          <t>2025-01-31</t>
-        </is>
-      </c>
-      <c r="I61" s="2" t="inlineStr">
-        <is>
-          <t>authorize</t>
-        </is>
-      </c>
-      <c r="J61" s="2" t="inlineStr">
-        <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="K61" s="2" t="inlineStr">
-        <is>
-          <t>operative</t>
-        </is>
-      </c>
-      <c r="Q61" s="3" t="inlineStr">
-        <is>
-          <t>1-CMFA-Agenda-1-31-2025.pdf</t>
-        </is>
-      </c>
-      <c r="R61" s="3" t="inlineStr">
-        <is>
-          <t>CMFA-Staff-Report-01-31-25.pdf</t>
-        </is>
-      </c>
-      <c r="S61" s="3" t="inlineStr">
-        <is>
-          <t>2-CMFA-Minutes-1-31-2025.pdf</t>
-        </is>
-      </c>
-      <c r="T61" s="2" t="inlineStr">
-        <is>
-          <t>Prometheus Real Estate Group</t>
-        </is>
-      </c>
       <c r="V61" s="2" t="inlineStr">
         <is>
           <t>Hearthstone Housing Foundation</t>
@@ -9216,7 +9231,7 @@
       </c>
       <c r="AL61" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; entity:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -11717,9 +11732,9 @@
           <t>10811 S. Compton Ave Apartments</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>10811 S. Compton Ave Apartments</t>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>2 SIOF 10811 S Compton Ave, LP</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -11829,7 +11844,7 @@
       </c>
       <c r="AL80" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -19563,9 +19578,9 @@
           <t>Flag VII Montecito, L.P.</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr">
-        <is>
-          <t>San Jose</t>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>Santa Clara</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
@@ -19685,7 +19700,7 @@
       </c>
       <c r="AL138" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; city:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -25154,16 +25169,16 @@
           <t>Ackerfield 2 LP</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr">
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>Long Beach</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr">
         <is>
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="F181" s="2" t="inlineStr">
-        <is>
-          <t>Los Angeles</t>
-        </is>
-      </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
           <t>26-039</t>
@@ -25261,7 +25276,7 @@
       </c>
       <c r="AL181" t="inlineStr">
         <is>
-          <t>manual_status:collaborator-sheet; city:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>manual_status:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -28807,9 +28822,9 @@
           <t>Haven Warner Center</t>
         </is>
       </c>
-      <c r="D210" t="inlineStr">
-        <is>
-          <t>Heven LP</t>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>Haven, LP</t>
         </is>
       </c>
       <c r="E210" s="2" t="inlineStr">
@@ -28909,7 +28924,7 @@
       </c>
       <c r="AL210" t="inlineStr">
         <is>
-          <t>entity:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -29014,9 +29029,9 @@
           <t>Grant of $5,000</t>
         </is>
       </c>
-      <c r="AC211" t="inlineStr">
-        <is>
-          <t>2075 W Jefferson BlvdLos Angeles, CA 90018</t>
+      <c r="AC211" s="2" t="inlineStr">
+        <is>
+          <t>2075 West Jefferson Blvd., Los Angeles</t>
         </is>
       </c>
       <c r="AD211" s="2" t="inlineStr">
@@ -29036,7 +29051,7 @@
       </c>
       <c r="AL211" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -31810,9 +31825,9 @@
           <t>Grant of $5,000</t>
         </is>
       </c>
-      <c r="AC234" t="inlineStr">
-        <is>
-          <t>3950 Ingraham St, San Diego, CA 92109</t>
+      <c r="AC234" s="2" t="inlineStr">
+        <is>
+          <t>3950 W. Ingraham Street, Los Angeles, CA</t>
         </is>
       </c>
       <c r="AD234" s="2" t="inlineStr">
@@ -31827,7 +31842,7 @@
       </c>
       <c r="AL234" t="inlineStr">
         <is>
-          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -73052,7 +73067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -73629,12 +73644,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>27</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>nonprofit_partner: generated 'AOF / Pacific Affordable Housing Corp.' -&gt; manual 'Pacific Affordable Housing Corp'</t>
+          <t>total_units: generated '24' -&gt; manual '52'</t>
         </is>
       </c>
     </row>
@@ -73646,12 +73661,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>28</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>city: generated 'Los Angeles' -&gt; manual 'El Sobrante'</t>
+          <t>total_units: generated '22' -&gt; manual '72'</t>
         </is>
       </c>
     </row>
@@ -73663,12 +73678,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>29</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>county: generated 'Los Angeles' -&gt; manual 'Contra Costa'</t>
+          <t>total_units: generated '24' -&gt; manual '48'</t>
         </is>
       </c>
     </row>
@@ -73680,12 +73695,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>total_units: generated '24' -&gt; manual '52'</t>
+          <t>total_units: generated '65' -&gt; manual '165'</t>
         </is>
       </c>
     </row>
@@ -73697,12 +73712,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>48</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>total_units: generated '22' -&gt; manual '72'</t>
+          <t>investor_1: generated 'Ethos Real Estate' -&gt; manual 'Vistria Group'</t>
         </is>
       </c>
     </row>
@@ -73714,12 +73729,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>51</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>total_units: generated '24' -&gt; manual '48'</t>
+          <t>total_units: generated '144' -&gt; manual '145'</t>
         </is>
       </c>
     </row>
@@ -73731,12 +73746,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>54</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>total_units: generated '65' -&gt; manual '165'</t>
+          <t>total_units: generated '42' -&gt; manual '356'</t>
         </is>
       </c>
     </row>
@@ -73748,12 +73763,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>property_name: generated '2330 3rd Street Apartments' -&gt; manual '2330 E. 3rd Street Apartments'</t>
+          <t>total_units: generated '29' -&gt; manual '196'</t>
         </is>
       </c>
     </row>
@@ -73765,12 +73780,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>78</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Ethos Real Estate' -&gt; manual 'Vistria Group'</t>
+          <t>investor_1: generated 'Vintage Housing Holdings, LLC' -&gt; manual 'Kennedy Wilson'</t>
         </is>
       </c>
     </row>
@@ -73782,12 +73797,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>78</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>total_units: generated '144' -&gt; manual '145'</t>
+          <t>nonprofit_partner: generated 'Pacific Housing, Inc.' -&gt; manual 'Hearthstone Housing Foundation'</t>
         </is>
       </c>
     </row>
@@ -73799,12 +73814,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>78</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>total_units: generated '42' -&gt; manual '356'</t>
+          <t>total_units: generated '8' -&gt; manual '1008'</t>
         </is>
       </c>
     </row>
@@ -73816,12 +73831,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>81</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>entity: generated 'PREG 5150 ECR Los Altos, LP, a California limited partnership' -&gt; manual 'Prometheus Real Estate Group'</t>
+          <t>total_units: generated '32' -&gt; manual '31'</t>
         </is>
       </c>
     </row>
@@ -73833,12 +73848,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>81</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>total_units: generated '29' -&gt; manual '196'</t>
+          <t>city_cut: generated '4650.0' -&gt; manual '4500'</t>
         </is>
       </c>
     </row>
@@ -73850,12 +73865,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>158</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Vintage Housing Holdings, LLC' -&gt; manual 'Kennedy Wilson'</t>
+          <t>total_units: generated '30' -&gt; manual '29'</t>
         </is>
       </c>
     </row>
@@ -73867,12 +73882,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>95</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>nonprofit_partner: generated 'Pacific Housing, Inc.' -&gt; manual 'Hearthstone Housing Foundation'</t>
+          <t>investor_1: generated 'Belveron Partners' -&gt; manual 'Sack Capital Partners'</t>
         </is>
       </c>
     </row>
@@ -73884,12 +73899,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>110</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>total_units: generated '8' -&gt; manual '1008'</t>
+          <t>total_units: generated '24' -&gt; manual '42'</t>
         </is>
       </c>
     </row>
@@ -73901,12 +73916,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>134</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>total_units: generated '32' -&gt; manual '31'</t>
+          <t>total_units: generated '69' -&gt; manual '68'</t>
         </is>
       </c>
     </row>
@@ -73918,12 +73933,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>137</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>city_cut: generated '4650.0' -&gt; manual '4500'</t>
+          <t>total_units: generated '42' -&gt; manual '41'</t>
         </is>
       </c>
     </row>
@@ -73935,12 +73950,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>152</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>entity: generated '2 SIOF 10811 S Compton Ave, LP' -&gt; manual '10811 S. Compton Ave Apartments'</t>
+          <t>total_units: generated '52' -&gt; manual '152'</t>
         </is>
       </c>
     </row>
@@ -73952,12 +73967,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>155</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>total_units: generated '30' -&gt; manual '29'</t>
+          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
         </is>
       </c>
     </row>
@@ -73969,12 +73984,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>156</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Belveron Partners' -&gt; manual 'Sack Capital Partners'</t>
+          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
         </is>
       </c>
     </row>
@@ -73986,12 +74001,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>171</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>total_units: generated '24' -&gt; manual '42'</t>
+          <t>city_cut: generated '15900.0' -&gt; manual '6300'</t>
         </is>
       </c>
     </row>
@@ -74003,12 +74018,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>181</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>city: generated 'Sacramento' -&gt; manual 'Unincorporated'</t>
+          <t>total_units: generated '52' -&gt; manual '152'</t>
         </is>
       </c>
     </row>
@@ -74020,12 +74035,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>195</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>property_name: generated 'Kinglsey Apartments' -&gt; manual 'Kingsley Apartments'</t>
+          <t>total_units: generated '42' -&gt; manual '41'</t>
         </is>
       </c>
     </row>
@@ -74037,12 +74052,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>199</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>total_units: generated '69' -&gt; manual '68'</t>
+          <t>city_cut: generated '5550.0' -&gt; manual '5500'</t>
         </is>
       </c>
     </row>
@@ -74054,12 +74069,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>204</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>total_units: generated '42' -&gt; manual '41'</t>
+          <t>total_units: generated '50' -&gt; manual '49'</t>
         </is>
       </c>
     </row>
@@ -74071,12 +74086,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>206</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>city: generated 'Santa Clara' -&gt; manual 'San Jose'</t>
+          <t>county: generated 'San Diego' -&gt; manual 'Los Angeles'</t>
         </is>
       </c>
     </row>
@@ -74088,12 +74103,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>209</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>total_units: generated '52' -&gt; manual '152'</t>
+          <t>investor_1: generated 'Zenith Property Group LLC' -&gt; manual 'Red Stone Equity Partners'</t>
         </is>
       </c>
     </row>
@@ -74105,12 +74120,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>209</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
+          <t>term_years: generated '35' -&gt; manual '15'</t>
         </is>
       </c>
     </row>
@@ -74122,12 +74137,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>210</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
+          <t>term_years: generated '55' -&gt; manual '10'</t>
         </is>
       </c>
     </row>
@@ -74139,12 +74154,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>171</t>
+          <t>226</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>city_cut: generated '15900.0' -&gt; manual '6300'</t>
+          <t>term_years: generated '15' -&gt; manual '10'</t>
         </is>
       </c>
     </row>
@@ -74156,12 +74171,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>228</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>city: generated 'Long Beach' -&gt; manual 'Los Angeles'</t>
+          <t>term_years: generated '10' -&gt; manual '15'</t>
         </is>
       </c>
     </row>
@@ -74173,12 +74188,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>217</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>total_units: generated '52' -&gt; manual '152'</t>
+          <t>total_units: generated '35' -&gt; manual '34'</t>
         </is>
       </c>
     </row>
@@ -74190,12 +74205,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>233</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>property_name: generated 'La Vista Apartments' -&gt; manual 'La Vista Apartment Homes'</t>
+          <t>term_years: generated '55' -&gt; manual '10'</t>
         </is>
       </c>
     </row>
@@ -74207,12 +74222,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>236</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>total_units: generated '42' -&gt; manual '41'</t>
+          <t>total_units: generated '136' -&gt; manual '108'</t>
         </is>
       </c>
     </row>
@@ -74224,707 +74239,350 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>225</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>address: generated '9750 Airport Blvd, Los Angeles, CA' -&gt; manual '9750 Airport Blvd, Westchester, CA 90045'</t>
+          <t>term_years: generated '30' -&gt; manual '55'</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-possible-match</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>city_cut: generated '5550.0' -&gt; manual '5500'</t>
+          <t>entity '381 Turk Street Associates, a California' ~ SCC LP '421 Turk Street Associates, L.P.' (#3326, San Francisco, score 92)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-possible-match</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>208</t>
+          <t>33</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>address: generated '2481 South Sawtelle Blvd, Los Angeles, CA' -&gt; manual '2481 Sawtelle Blvd, Los Angeles, CA 90064'</t>
+          <t>entity 'BIF NON OZ 7524 S HOOVER ST, LP' ~ SCC LP 'BIF NON OZ 7518 S Hoover St, LP' (#14953, Los Angeles, score 93)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-possible-match</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>entity: generated 'Standard Summerwood II LP' -&gt; manual 'Standard Properties'</t>
+          <t>entity 'BIF NON OZ 4228 WESTERN AVE, LP' ~ SCC LP 'BIF NON OZ 4209 Western Ave, LP' (#14952, Los Angeles, score 93)</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-possible-match</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>122</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Standard Property Company, Inc.' -&gt; manual 'Standard Properties'</t>
+          <t>entity '861 Fedora LLLP' ~ SCC LP '836 Fedora L.P.' (#1594, Los Angeles, score 90)</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-possible-match</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>165</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>total_units: generated '50' -&gt; manual '49'</t>
+          <t>entity '861 Fedora LLLP' ~ SCC LP '836 Fedora L.P.' (#1594, Los Angeles, score 90)</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>76</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>county: generated 'San Diego' -&gt; manual 'Los Angeles'</t>
+          <t>AIN 5036031006 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>99</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Zenith Property Group LLC' -&gt; manual 'Red Stone Equity Partners'</t>
+          <t>AIN 4262018026 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>132</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>term_years: generated '35' -&gt; manual '15'</t>
+          <t>AIN 6020022027 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>137</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>term_years: generated '55' -&gt; manual '10'</t>
+          <t>AIN 2125017014 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>158</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>term_years: generated '15' -&gt; manual '10'</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>196</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>term_years: generated '10' -&gt; manual '15'</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>201</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>address: generated '11821 Foothill Blvd, Los Angeles, CA' -&gt; manual '11821 Foothill Blvd, Lake View Terrace, CA 91342'</t>
+          <t>AIN (none) (Santa Barbara): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>217</t>
+          <t>206</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>total_units: generated '35' -&gt; manual '34'</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>207</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>entity: generated 'Haven, LP' -&gt; manual 'Heven LP'</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>208</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>address: generated '6530 Independence Avenue, Los Angeles' -&gt; manual '6530 Independence Ave, Canoga Park, CA 91303'</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>212</t>
+          <t>215</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>address: generated '2075 West Jefferson Blvd., Los Angeles' -&gt; manual '2075 W Jefferson BlvdLos Angeles, CA 90018'</t>
+          <t>AIN 5539028040 (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>231</t>
+          <t>226</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>nonprofit_partner: generated 'Bedford' -&gt; manual 'Bedford Affordable Housing Foundation'</t>
+          <t>AIN (none) (Contra Costa): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>term_years: generated '55' -&gt; manual '10'</t>
+          <t>AIN 128101150 (Solano) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>235</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>address: generated '3950 W. Ingraham Street, Los Angeles, CA' -&gt; manual '3950 Ingraham St, San Diego, CA 92109'</t>
+          <t>AIN 128101050 (Solano) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
-        <is>
-          <t>total_units: generated '136' -&gt; manual '108'</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>override-conflict</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>225</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>term_years: generated '30' -&gt; manual '55'</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>scc-possible-match</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>entity '381 Turk Street Associates, a California' ~ SCC LP '421 Turk Street Associates, L.P.' (#3326, San Francisco, score 92)</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>scc-possible-match</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>entity 'BIF NON OZ 7524 S HOOVER ST, LP' ~ SCC LP 'BIF NON OZ 7518 S Hoover St, LP' (#14953, Los Angeles, score 93)</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>scc-possible-match</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>entity 'BIF NON OZ 4228 WESTERN AVE, LP' ~ SCC LP 'BIF NON OZ 4209 Western Ave, LP' (#14952, Los Angeles, score 93)</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>scc-possible-match</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>122</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>entity '861 Fedora LLLP' ~ SCC LP '836 Fedora L.P.' (#1594, Los Angeles, score 90)</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>scc-possible-match</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>165</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>entity '861 Fedora LLLP' ~ SCC LP '836 Fedora L.P.' (#1594, Los Angeles, score 90)</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>76</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>AIN 5036031006 (Los Angeles) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>99</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>AIN 4262018026 (Los Angeles) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>132</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>AIN 6020022027 (Los Angeles) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>137</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>AIN 2125017014 (Los Angeles) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>158</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>196</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>201</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>AIN (none) (Santa Barbara): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>206</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>207</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>208</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>215</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>AIN 5539028040 (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>226</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>AIN (none) (Contra Costa): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>AIN 128101150 (Solano) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>AIN 128101050 (Solano) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
         <is>
           <t>AIN 128105060 (Solano) has no current roll data; using manual value</t>
         </is>

</xml_diff>

<commit_message>
Parcel assignment auditing: situs validation, sibling sweep, unit reconciliation
New check_parcel_assignments.py stage audits the one human-asserted
link in the pipeline (address -> AIN), noise-gated per review: street/
city-level mismatches only (near-miss house numbers pass, documented
portal picks skipped), same-situs+ZIP sibling sweep, and county-unit
reconciliation gated to apartment-use parcels (LA Units1-5 agree with
grants within 20% on 86% of apartment properties). Fetchers now carry
unit counts and exact situs fields. First run: 15 findings from 354
assignments — including a $7.0M unassigned sibling parcel at
Alexandria II and $15.3M at Market Street Village.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -73067,10 +73067,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
   </cols>
@@ -74585,6 +74585,261 @@
       <c r="C89" t="inlineStr">
         <is>
           <t>AIN 128105060 (Solano) has no current roll data; using manual value</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>assignment-mismatch</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>148</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Park Wilshire Apartments: grant city 'Los Angeles' appears in no assigned parcel's situs</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>assignment-mismatch</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Seaport Village Apartments: no assigned parcel's situs matches address '5601 North Paramount Boulevard' (e.g. 7157031001: 2697 E 56TH WAY LONG BEACH CA 90805; 7157031002: 2687 E 56TH WAY LONG BEACH CA 90805)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>assignment-mismatch</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>569 W. 6th Street. Apartments: grant city 'Los Angeles' appears in no assigned parcel's situs</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>possible-missing-parcel</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Alvarado Streets Apartments: parcel 5136019023 shares situs '1136 S ALVARADO ST LOS ANGELES CA 90006' (Auto, Recreation EQPT, C, $1,039,983) but is not assigned to any project</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>possible-missing-parcel</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Market Street Village Apartmen: parcel 5351441600 shares situs '699 14TH SD' (31, $15,300,000) but is not assigned to any project</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>possible-missing-parcel</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Alexandria II Apartments: parcel 5518012036 shares situs '130 N ALEXANDRIA AVE APT 0104 LOS ANGELES CA 90004' (Five or more apartments, $7,015,185) but is not assigned to any project</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>possible-missing-parcel</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Kenmore II Apartments: parcel 5518018011 shares situs '200 N KENMORE AVE LOS ANGELES CA 90004' (Five or more apartments, $452,268) but is not assigned to any project</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>units-undercount</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>The Waterloo Apartments: county records 5 units on assigned parcels vs 154 in the grant — parcels may be missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>units-undercount</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Candlewood North Apartments: county records 68 units on assigned parcels vs 189 in the grant — parcels may be missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>units-undercount</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Kenmore I Apartments: county records 24 units on assigned parcels vs 42 in the grant — parcels may be missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>units-undercount</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>181</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>The Hive Apartments: county records 50 units on assigned parcels vs 152 in the grant — parcels may be missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>units-undercount</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>1723 Corinth Apartments: county records 10 units on assigned parcels vs 41 in the grant — parcels may be missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>units-undercount</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>231</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Violet on Virgil: county records 159 units on assigned parcels vs 302 in the grant — parcels may be missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>units-undercount</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>926 S. Kingsley Apartments: county records 1 units on assigned parcels vs 136 in the grant — parcels may be missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>units-undercount</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>237</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Edgemont by Angeleno: county records 8 units on assigned parcels vs 34 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Street comparison uses county situs_street and positional address parsing
City-word overlap no longer masquerades as a street match (it hid two
real mis-assignments), streets named after cities survive tokenizing,
and the sibling sweep requires matching street direction (130 N vs
130 S Alexandria are different buildings). Verdicts: 200 situs-match,
89 no-situs, 78 mismatch, 7 documented; 15 findings stand.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -54549,12 +54549,12 @@
           <t>11630 S. Main Street Apartments</t>
         </is>
       </c>
-      <c r="D148" s="2" t="inlineStr">
+      <c r="D148" t="inlineStr">
         <is>
           <t>6083010040</t>
         </is>
       </c>
-      <c r="E148" s="2" t="inlineStr">
+      <c r="E148" t="inlineStr">
         <is>
           <t>6083-010-040</t>
         </is>
@@ -54631,7 +54631,7 @@
       </c>
       <c r="U148" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -67732,7 +67732,7 @@
           <t>926 S. Kingsley Apartments</t>
         </is>
       </c>
-      <c r="D297" s="2" t="inlineStr">
+      <c r="D297" t="inlineStr">
         <is>
           <t>5093023058</t>
         </is>
@@ -67809,7 +67809,7 @@
       </c>
       <c r="U297" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -68120,7 +68120,7 @@
           <t>Edgemont by Angeleno</t>
         </is>
       </c>
-      <c r="D301" s="2" t="inlineStr">
+      <c r="D301" t="inlineStr">
         <is>
           <t>5540023002</t>
         </is>
@@ -68197,7 +68197,7 @@
       </c>
       <c r="U301" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -69429,7 +69429,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D323" s="2" t="inlineStr">
+      <c r="D323" t="inlineStr">
         <is>
           <t>128101140</t>
         </is>
@@ -69491,7 +69491,7 @@
       </c>
       <c r="U323" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -69511,7 +69511,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D324" s="2" t="inlineStr">
+      <c r="D324" t="inlineStr">
         <is>
           <t>128101130</t>
         </is>
@@ -69573,7 +69573,7 @@
       </c>
       <c r="U324" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -69593,7 +69593,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D325" s="2" t="inlineStr">
+      <c r="D325" t="inlineStr">
         <is>
           <t>128101120</t>
         </is>
@@ -69655,7 +69655,7 @@
       </c>
       <c r="U325" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -69675,7 +69675,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D326" s="2" t="inlineStr">
+      <c r="D326" t="inlineStr">
         <is>
           <t>128101110</t>
         </is>
@@ -69737,7 +69737,7 @@
       </c>
       <c r="U326" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -69834,7 +69834,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D328" s="2" t="inlineStr">
+      <c r="D328" t="inlineStr">
         <is>
           <t>128101090</t>
         </is>
@@ -69896,7 +69896,7 @@
       </c>
       <c r="U328" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -69916,7 +69916,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D329" s="2" t="inlineStr">
+      <c r="D329" t="inlineStr">
         <is>
           <t>128101080</t>
         </is>
@@ -69978,7 +69978,7 @@
       </c>
       <c r="U329" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -69998,7 +69998,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D330" s="2" t="inlineStr">
+      <c r="D330" t="inlineStr">
         <is>
           <t>128101070</t>
         </is>
@@ -70060,7 +70060,7 @@
       </c>
       <c r="U330" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -70080,7 +70080,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D331" s="2" t="inlineStr">
+      <c r="D331" t="inlineStr">
         <is>
           <t>128101060</t>
         </is>
@@ -70142,7 +70142,7 @@
       </c>
       <c r="U331" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -70234,7 +70234,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D333" s="2" t="inlineStr">
+      <c r="D333" t="inlineStr">
         <is>
           <t>128101040</t>
         </is>
@@ -70296,7 +70296,7 @@
       </c>
       <c r="U333" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -70316,7 +70316,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D334" s="2" t="inlineStr">
+      <c r="D334" t="inlineStr">
         <is>
           <t>128101030</t>
         </is>
@@ -70378,7 +70378,7 @@
       </c>
       <c r="U334" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -70398,7 +70398,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D335" s="2" t="inlineStr">
+      <c r="D335" t="inlineStr">
         <is>
           <t>128101020</t>
         </is>
@@ -70460,7 +70460,7 @@
       </c>
       <c r="U335" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -70480,7 +70480,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D336" s="2" t="inlineStr">
+      <c r="D336" t="inlineStr">
         <is>
           <t>128101010</t>
         </is>
@@ -70542,7 +70542,7 @@
       </c>
       <c r="U336" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -70562,7 +70562,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D337" s="2" t="inlineStr">
+      <c r="D337" t="inlineStr">
         <is>
           <t>128102110</t>
         </is>
@@ -70624,7 +70624,7 @@
       </c>
       <c r="U337" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -70644,7 +70644,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D338" s="2" t="inlineStr">
+      <c r="D338" t="inlineStr">
         <is>
           <t>128102100</t>
         </is>
@@ -70706,7 +70706,7 @@
       </c>
       <c r="U338" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -70726,7 +70726,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D339" s="2" t="inlineStr">
+      <c r="D339" t="inlineStr">
         <is>
           <t>128102090</t>
         </is>
@@ -70788,7 +70788,7 @@
       </c>
       <c r="U339" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -70808,7 +70808,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D340" s="2" t="inlineStr">
+      <c r="D340" t="inlineStr">
         <is>
           <t>128102080</t>
         </is>
@@ -70870,7 +70870,7 @@
       </c>
       <c r="U340" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -70890,7 +70890,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D341" s="2" t="inlineStr">
+      <c r="D341" t="inlineStr">
         <is>
           <t>128102070</t>
         </is>
@@ -70952,7 +70952,7 @@
       </c>
       <c r="U341" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -70972,7 +70972,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D342" s="2" t="inlineStr">
+      <c r="D342" t="inlineStr">
         <is>
           <t>128102060</t>
         </is>
@@ -71034,7 +71034,7 @@
       </c>
       <c r="U342" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -71054,7 +71054,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D343" s="2" t="inlineStr">
+      <c r="D343" t="inlineStr">
         <is>
           <t>128102050</t>
         </is>
@@ -71116,7 +71116,7 @@
       </c>
       <c r="U343" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -71136,7 +71136,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D344" s="2" t="inlineStr">
+      <c r="D344" t="inlineStr">
         <is>
           <t>128102040</t>
         </is>
@@ -71198,7 +71198,7 @@
       </c>
       <c r="U344" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -71218,7 +71218,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D345" s="2" t="inlineStr">
+      <c r="D345" t="inlineStr">
         <is>
           <t>128102030</t>
         </is>
@@ -71280,7 +71280,7 @@
       </c>
       <c r="U345" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -71300,7 +71300,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D346" s="2" t="inlineStr">
+      <c r="D346" t="inlineStr">
         <is>
           <t>128102020</t>
         </is>
@@ -71362,7 +71362,7 @@
       </c>
       <c r="U346" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -71382,7 +71382,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D347" s="2" t="inlineStr">
+      <c r="D347" t="inlineStr">
         <is>
           <t>128102010</t>
         </is>
@@ -71444,7 +71444,7 @@
       </c>
       <c r="U347" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -71464,7 +71464,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D348" s="2" t="inlineStr">
+      <c r="D348" t="inlineStr">
         <is>
           <t>128102210</t>
         </is>
@@ -71526,7 +71526,7 @@
       </c>
       <c r="U348" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -71546,7 +71546,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D349" s="2" t="inlineStr">
+      <c r="D349" t="inlineStr">
         <is>
           <t>128102200</t>
         </is>
@@ -71608,7 +71608,7 @@
       </c>
       <c r="U349" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -71628,7 +71628,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D350" s="2" t="inlineStr">
+      <c r="D350" t="inlineStr">
         <is>
           <t>128102190</t>
         </is>
@@ -71690,7 +71690,7 @@
       </c>
       <c r="U350" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -71710,7 +71710,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D351" s="2" t="inlineStr">
+      <c r="D351" t="inlineStr">
         <is>
           <t>128102180</t>
         </is>
@@ -71772,7 +71772,7 @@
       </c>
       <c r="U351" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -71792,7 +71792,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D352" s="2" t="inlineStr">
+      <c r="D352" t="inlineStr">
         <is>
           <t>128102170</t>
         </is>
@@ -71854,7 +71854,7 @@
       </c>
       <c r="U352" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -71874,7 +71874,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D353" s="2" t="inlineStr">
+      <c r="D353" t="inlineStr">
         <is>
           <t>128102160</t>
         </is>
@@ -71936,7 +71936,7 @@
       </c>
       <c r="U353" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -71956,7 +71956,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D354" s="2" t="inlineStr">
+      <c r="D354" t="inlineStr">
         <is>
           <t>128102150</t>
         </is>
@@ -72018,7 +72018,7 @@
       </c>
       <c r="U354" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -72038,7 +72038,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D355" s="2" t="inlineStr">
+      <c r="D355" t="inlineStr">
         <is>
           <t>128102140</t>
         </is>
@@ -72100,7 +72100,7 @@
       </c>
       <c r="U355" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -72120,7 +72120,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D356" s="2" t="inlineStr">
+      <c r="D356" t="inlineStr">
         <is>
           <t>128102130</t>
         </is>
@@ -72182,7 +72182,7 @@
       </c>
       <c r="U356" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -72202,7 +72202,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D357" s="2" t="inlineStr">
+      <c r="D357" t="inlineStr">
         <is>
           <t>128102120</t>
         </is>
@@ -72264,7 +72264,7 @@
       </c>
       <c r="U357" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -72284,7 +72284,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D358" s="2" t="inlineStr">
+      <c r="D358" t="inlineStr">
         <is>
           <t>128103090</t>
         </is>
@@ -72346,7 +72346,7 @@
       </c>
       <c r="U358" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -72366,7 +72366,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D359" s="2" t="inlineStr">
+      <c r="D359" t="inlineStr">
         <is>
           <t>128103080</t>
         </is>
@@ -72428,7 +72428,7 @@
       </c>
       <c r="U359" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -72448,7 +72448,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D360" s="2" t="inlineStr">
+      <c r="D360" t="inlineStr">
         <is>
           <t>128103070</t>
         </is>
@@ -72510,7 +72510,7 @@
       </c>
       <c r="U360" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -72530,7 +72530,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D361" s="2" t="inlineStr">
+      <c r="D361" t="inlineStr">
         <is>
           <t>128103060</t>
         </is>
@@ -72592,7 +72592,7 @@
       </c>
       <c r="U361" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -72612,7 +72612,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D362" s="2" t="inlineStr">
+      <c r="D362" t="inlineStr">
         <is>
           <t>128103050</t>
         </is>
@@ -72674,7 +72674,7 @@
       </c>
       <c r="U362" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -72694,7 +72694,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D363" s="2" t="inlineStr">
+      <c r="D363" t="inlineStr">
         <is>
           <t>128103040</t>
         </is>
@@ -72756,7 +72756,7 @@
       </c>
       <c r="U363" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -72776,7 +72776,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D364" s="2" t="inlineStr">
+      <c r="D364" t="inlineStr">
         <is>
           <t>128103030</t>
         </is>
@@ -72838,7 +72838,7 @@
       </c>
       <c r="U364" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -72858,7 +72858,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D365" s="2" t="inlineStr">
+      <c r="D365" t="inlineStr">
         <is>
           <t>128103020</t>
         </is>
@@ -72920,7 +72920,7 @@
       </c>
       <c r="U365" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -72940,7 +72940,7 @@
           <t>Montessa Apartments</t>
         </is>
       </c>
-      <c r="D366" s="2" t="inlineStr">
+      <c r="D366" t="inlineStr">
         <is>
           <t>128103010</t>
         </is>
@@ -73002,7 +73002,7 @@
       </c>
       <c r="U366" s="2" t="inlineStr">
         <is>
-          <t>situs-match</t>
+          <t>mismatch</t>
         </is>
       </c>
     </row>
@@ -76489,12 +76489,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>233</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Seaport Village Apartments: no assigned parcel's situs matches address '5601 North Paramount Boulevard' (e.g. 7157031001: 2697 E 56TH WAY LONG BEACH CA 90805; 7157031002: 2687 E 56TH WAY LONG BEACH CA 90805)</t>
+          <t>926 S. Kingsley Apartments: no assigned parcel's situs matches address '926 S. Kingsley Drive, Los Angeles, CA' (e.g. 5093023058: 926 S HARVARD BLVD LOS ANGELES CA 90006)</t>
         </is>
       </c>
     </row>
@@ -76506,46 +76506,46 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>237</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>569 W. 6th Street. Apartments: grant city 'Los Angeles' appears in no assigned parcel's situs</t>
+          <t>Edgemont by Angeleno: no assigned parcel's situs matches address '1178 N. Edgemont Street, Los Angeles, CA' (e.g. 5540023002: 1178 N HELIOTROPE DR LOS ANGELES CA 90029)</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>possible-missing-parcel</t>
+          <t>assignment-mismatch</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>54</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Alvarado Streets Apartments: parcel 5136019023 shares situs '1136 S ALVARADO ST LOS ANGELES CA 90006' (Auto, Recreation EQPT, C, $1,039,983) but is not assigned to any project</t>
+          <t>Seaport Village Apartments: no assigned parcel's situs matches address '5601 North Paramount Boulevard' (e.g. 7157031001: 2697 E 56TH WAY LONG BEACH CA 90805; 7157031002: 2687 E 56TH WAY LONG BEACH CA 90805)</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>possible-missing-parcel</t>
+          <t>assignment-mismatch</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>77</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Market Street Village Apartmen: parcel 5351441600 shares situs '699 14TH SD' (31, $15,300,000) but is not assigned to any project</t>
+          <t>11630 S. Main Street Apartments: no assigned parcel's situs matches address '11630 Main St, Los Angeles, CA 90061' (e.g. 6083010040: 110 E 116TH ST LOS ANGELES CA 90061)</t>
         </is>
       </c>
     </row>
@@ -76557,12 +76557,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Alexandria II Apartments: parcel 5518012036 shares situs '130 N ALEXANDRIA AVE APT 0104 LOS ANGELES CA 90004' (Five or more apartments, $7,015,185) but is not assigned to any project</t>
+          <t>Alvarado Streets Apartments: parcel 5136019023 shares situs '1136 S ALVARADO ST LOS ANGELES CA 90006' (Auto, Recreation EQPT, C, $1,039,983) but is not assigned to any project</t>
         </is>
       </c>
     </row>
@@ -76574,12 +76574,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Kenmore II Apartments: parcel 5518018011 shares situs '200 N KENMORE AVE LOS ANGELES CA 90004' (Five or more apartments, $452,268) but is not assigned to any project</t>
+          <t>Market Street Village Apartmen: parcel 5351441600 shares situs '699 14TH SD' (31, $15,300,000) but is not assigned to any project</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply portal research: three corrected AINs, Seaport reviewed, 11630 Main confirmed
926 S Kingsley -> 5093023056 ($4.0M); Edgemont -> 5540025003
($1.25M); Park Wilshire is the LOS ANGELES 2424 Wilshire ->
5141004003 ($19.7M — prior Santa Monica parcel was $3.5M, a
5.6x roll-value correction). Seaport Village confirmed as 33
parcels on E 56th Way (all were already assigned); 11630 Main's
AIN confirmed under county situs 114 E 116th St. All three new
AINs fetch values and verify as situs-match.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -48797,7 +48797,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K86" s="2" t="inlineStr">
@@ -48852,7 +48852,7 @@
       </c>
       <c r="U86" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -48904,7 +48904,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr">
@@ -48959,7 +48959,7 @@
       </c>
       <c r="U87" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -49011,7 +49011,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K88" s="2" t="inlineStr">
@@ -49066,7 +49066,7 @@
       </c>
       <c r="U88" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -49118,7 +49118,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K89" s="2" t="inlineStr">
@@ -49173,7 +49173,7 @@
       </c>
       <c r="U89" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -49225,7 +49225,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K90" s="2" t="inlineStr">
@@ -49280,7 +49280,7 @@
       </c>
       <c r="U90" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -49332,7 +49332,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K91" s="2" t="inlineStr">
@@ -49387,7 +49387,7 @@
       </c>
       <c r="U91" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -49439,7 +49439,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K92" s="2" t="inlineStr">
@@ -49494,7 +49494,7 @@
       </c>
       <c r="U92" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -49546,7 +49546,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K93" s="2" t="inlineStr">
@@ -49601,7 +49601,7 @@
       </c>
       <c r="U93" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -49653,7 +49653,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K94" s="2" t="inlineStr">
@@ -49708,7 +49708,7 @@
       </c>
       <c r="U94" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -49760,7 +49760,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K95" s="2" t="inlineStr">
@@ -49815,7 +49815,7 @@
       </c>
       <c r="U95" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -49867,7 +49867,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K96" s="2" t="inlineStr">
@@ -49922,7 +49922,7 @@
       </c>
       <c r="U96" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -49974,7 +49974,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K97" s="2" t="inlineStr">
@@ -50029,7 +50029,7 @@
       </c>
       <c r="U97" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -50081,7 +50081,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K98" s="2" t="inlineStr">
@@ -50136,7 +50136,7 @@
       </c>
       <c r="U98" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -50188,7 +50188,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K99" s="2" t="inlineStr">
@@ -50243,7 +50243,7 @@
       </c>
       <c r="U99" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -50295,7 +50295,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K100" s="2" t="inlineStr">
@@ -50350,7 +50350,7 @@
       </c>
       <c r="U100" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -50402,7 +50402,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K101" s="2" t="inlineStr">
@@ -50457,7 +50457,7 @@
       </c>
       <c r="U101" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -50509,7 +50509,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K102" s="2" t="inlineStr">
@@ -50564,7 +50564,7 @@
       </c>
       <c r="U102" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -50616,7 +50616,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K103" s="2" t="inlineStr">
@@ -50671,7 +50671,7 @@
       </c>
       <c r="U103" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -50723,7 +50723,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K104" s="2" t="inlineStr">
@@ -50778,7 +50778,7 @@
       </c>
       <c r="U104" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -50830,7 +50830,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K105" s="2" t="inlineStr">
@@ -50885,7 +50885,7 @@
       </c>
       <c r="U105" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -50937,7 +50937,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K106" s="2" t="inlineStr">
@@ -50992,7 +50992,7 @@
       </c>
       <c r="U106" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -51044,7 +51044,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K107" s="2" t="inlineStr">
@@ -51099,7 +51099,7 @@
       </c>
       <c r="U107" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -51151,7 +51151,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K108" s="2" t="inlineStr">
@@ -51206,7 +51206,7 @@
       </c>
       <c r="U108" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -51258,7 +51258,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K109" s="2" t="inlineStr">
@@ -51313,7 +51313,7 @@
       </c>
       <c r="U109" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -51365,7 +51365,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K110" s="2" t="inlineStr">
@@ -51420,7 +51420,7 @@
       </c>
       <c r="U110" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -51472,7 +51472,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K111" s="2" t="inlineStr">
@@ -51527,7 +51527,7 @@
       </c>
       <c r="U111" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -51579,7 +51579,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K112" s="2" t="inlineStr">
@@ -51634,7 +51634,7 @@
       </c>
       <c r="U112" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -51686,7 +51686,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K113" s="2" t="inlineStr">
@@ -51741,7 +51741,7 @@
       </c>
       <c r="U113" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -51793,7 +51793,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -51848,7 +51848,7 @@
       </c>
       <c r="U114" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -51900,7 +51900,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K115" s="2" t="inlineStr">
@@ -51955,7 +51955,7 @@
       </c>
       <c r="U115" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -52007,7 +52007,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K116" s="2" t="inlineStr">
@@ -52062,7 +52062,7 @@
       </c>
       <c r="U116" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -52114,7 +52114,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr">
@@ -52169,7 +52169,7 @@
       </c>
       <c r="U117" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -52221,7 +52221,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>Multi-parcel (33)</t>
+          <t>Multi-parcel (33); situs reviewed 2026-08-22: complex fronts 5601 N Paramount Blvd; buildings carry E 56th Way situs (Drew, portal map)</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr">
@@ -52276,7 +52276,7 @@
       </c>
       <c r="U118" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -54576,7 +54576,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>Legacy AIN 6083010038 consolidated to 6083010040</t>
+          <t>situs reviewed 2026-08-22 (Drew, assessor portal): AIN confirmed; county situs is 114 E 116TH ST, differs from marketing address 11630 S Main St</t>
         </is>
       </c>
       <c r="K148" s="2" t="inlineStr">
@@ -54631,7 +54631,7 @@
       </c>
       <c r="U148" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>documented</t>
         </is>
       </c>
     </row>
@@ -60775,17 +60775,17 @@
       </c>
       <c r="D215" s="2" t="inlineStr">
         <is>
-          <t>4276017047</t>
+          <t>5141004003</t>
         </is>
       </c>
       <c r="E215" s="2" t="inlineStr">
         <is>
-          <t>4276-017-047</t>
+          <t>5141-004-003</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>2424 WILSHIRE BLVD SANTA MONICA CA 90403</t>
+          <t>2424 WILSHIRE BLVD LOS ANGELES CA</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
@@ -60795,7 +60795,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>collaborator-sheet</t>
+          <t>manual-repo-edit</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
@@ -60803,6 +60803,11 @@
           <t>manual_verified</t>
         </is>
       </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>Corrected 2026-08-22 (Drew, assessor portal): prior parcel was 2424 Wilshire SANTA MONICA; Park Wilshire is the LA one</t>
+        </is>
+      </c>
       <c r="K215" s="2" t="inlineStr">
         <is>
           <t>2026</t>
@@ -60810,17 +60815,17 @@
       </c>
       <c r="L215" s="2" t="inlineStr">
         <is>
-          <t>2946701</t>
+          <t>8600000</t>
         </is>
       </c>
       <c r="M215" s="2" t="inlineStr">
         <is>
-          <t>576523</t>
+          <t>11100000</t>
         </is>
       </c>
       <c r="N215" s="2" t="inlineStr">
         <is>
-          <t>3523224</t>
+          <t>19700000</t>
         </is>
       </c>
       <c r="O215" s="2" t="inlineStr">
@@ -60830,12 +60835,12 @@
       </c>
       <c r="P215" s="2" t="inlineStr">
         <is>
-          <t>1948</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="Q215" s="2" t="inlineStr">
         <is>
-          <t>Office Buildings</t>
+          <t>Five or more apartments</t>
         </is>
       </c>
       <c r="R215" s="2" t="inlineStr">
@@ -67732,14 +67737,19 @@
           <t>926 S. Kingsley Apartments</t>
         </is>
       </c>
-      <c r="D297" t="inlineStr">
-        <is>
-          <t>5093023058</t>
+      <c r="D297" s="2" t="inlineStr">
+        <is>
+          <t>5093023056</t>
+        </is>
+      </c>
+      <c r="E297" s="2" t="inlineStr">
+        <is>
+          <t>5093-023-056</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>926 S HARVARD BLVD LOS ANGELES CA 90006</t>
+          <t>926 S KINGSLEY DR LOS ANGELES CA 90006</t>
         </is>
       </c>
       <c r="G297" t="inlineStr">
@@ -67749,12 +67759,12 @@
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>script-finder-auto (2026-08-21)</t>
+          <t>manual-repo-edit</t>
         </is>
       </c>
       <c r="J297" t="inlineStr">
         <is>
-          <t>Resolved by LA county situs/geocode search</t>
+          <t>Corrected 2026-08-22 (Drew, assessor portal): prior geocode pick 5093023058 sits at 926 S Harvard Blvd</t>
         </is>
       </c>
       <c r="K297" s="2" t="inlineStr">
@@ -67764,17 +67774,17 @@
       </c>
       <c r="L297" s="2" t="inlineStr">
         <is>
-          <t>1396325</t>
+          <t>2827070</t>
         </is>
       </c>
       <c r="M297" s="2" t="inlineStr">
         <is>
-          <t>587224</t>
+          <t>1172181</t>
         </is>
       </c>
       <c r="N297" s="2" t="inlineStr">
         <is>
-          <t>1983549</t>
+          <t>3999251</t>
         </is>
       </c>
       <c r="O297" s="2" t="inlineStr">
@@ -67784,12 +67794,12 @@
       </c>
       <c r="P297" s="2" t="inlineStr">
         <is>
-          <t>1914</t>
+          <t>1912</t>
         </is>
       </c>
       <c r="Q297" s="2" t="inlineStr">
         <is>
-          <t>Five or more apartments</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="R297" s="2" t="inlineStr">
@@ -67809,7 +67819,7 @@
       </c>
       <c r="U297" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>situs-match</t>
         </is>
       </c>
     </row>
@@ -68120,14 +68130,19 @@
           <t>Edgemont by Angeleno</t>
         </is>
       </c>
-      <c r="D301" t="inlineStr">
-        <is>
-          <t>5540023002</t>
+      <c r="D301" s="2" t="inlineStr">
+        <is>
+          <t>5540025003</t>
+        </is>
+      </c>
+      <c r="E301" s="2" t="inlineStr">
+        <is>
+          <t>5540-025-003</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>1178 N HELIOTROPE DR LOS ANGELES CA 90029</t>
+          <t>1178 N EDGEMONT ST LOS ANGELES CA 90029</t>
         </is>
       </c>
       <c r="G301" t="inlineStr">
@@ -68137,12 +68152,12 @@
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>script-finder-auto (2026-08-21)</t>
+          <t>manual-repo-edit</t>
         </is>
       </c>
       <c r="J301" t="inlineStr">
         <is>
-          <t>Resolved by LA county situs/geocode search</t>
+          <t>Corrected 2026-08-22 (Drew, assessor portal): prior geocode pick 5540023002 sits at 1178 N Heliotrope Dr</t>
         </is>
       </c>
       <c r="K301" s="2" t="inlineStr">
@@ -68152,17 +68167,17 @@
       </c>
       <c r="L301" s="2" t="inlineStr">
         <is>
-          <t>271221</t>
+          <t>1186056</t>
         </is>
       </c>
       <c r="M301" s="2" t="inlineStr">
         <is>
-          <t>331491</t>
+          <t>62424</t>
         </is>
       </c>
       <c r="N301" s="2" t="inlineStr">
         <is>
-          <t>602712</t>
+          <t>1248480</t>
         </is>
       </c>
       <c r="O301" s="2" t="inlineStr">
@@ -68172,12 +68187,12 @@
       </c>
       <c r="P301" s="2" t="inlineStr">
         <is>
-          <t>1962</t>
+          <t>1919</t>
         </is>
       </c>
       <c r="Q301" s="2" t="inlineStr">
         <is>
-          <t>Five or more apartments</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="R301" s="2" t="inlineStr">
@@ -68197,7 +68212,7 @@
       </c>
       <c r="U301" s="2" t="inlineStr">
         <is>
-          <t>mismatch</t>
+          <t>situs-match</t>
         </is>
       </c>
     </row>
@@ -74943,10 +74958,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
   </cols>
@@ -76467,119 +76482,119 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>assignment-mismatch</t>
+          <t>possible-missing-parcel</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Park Wilshire Apartments: grant city 'Los Angeles' appears in no assigned parcel's situs</t>
+          <t>Alvarado Streets Apartments: parcel 5136019023 shares situs '1136 S ALVARADO ST LOS ANGELES CA 90006' (Auto, Recreation EQPT, C, $1,039,983) but is not assigned to any project</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>assignment-mismatch</t>
+          <t>possible-missing-parcel</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>926 S. Kingsley Apartments: no assigned parcel's situs matches address '926 S. Kingsley Drive, Los Angeles, CA' (e.g. 5093023058: 926 S HARVARD BLVD LOS ANGELES CA 90006)</t>
+          <t>Market Street Village Apartmen: parcel 5351441600 shares situs '699 14TH SD' (31, $15,300,000) but is not assigned to any project</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>assignment-mismatch</t>
+          <t>units-undercount</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>237</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Edgemont by Angeleno: no assigned parcel's situs matches address '1178 N. Edgemont Street, Los Angeles, CA' (e.g. 5540023002: 1178 N HELIOTROPE DR LOS ANGELES CA 90029)</t>
+          <t>The Waterloo Apartments: county records 5 units on assigned parcels vs 154 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>assignment-mismatch</t>
+          <t>units-undercount</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>68</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Seaport Village Apartments: no assigned parcel's situs matches address '5601 North Paramount Boulevard' (e.g. 7157031001: 2697 E 56TH WAY LONG BEACH CA 90805; 7157031002: 2687 E 56TH WAY LONG BEACH CA 90805)</t>
+          <t>Candlewood North Apartments: county records 68 units on assigned parcels vs 189 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>assignment-mismatch</t>
+          <t>units-undercount</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>110</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>11630 S. Main Street Apartments: no assigned parcel's situs matches address '11630 Main St, Los Angeles, CA 90061' (e.g. 6083010040: 110 E 116TH ST LOS ANGELES CA 90061)</t>
+          <t>Kenmore I Apartments: county records 24 units on assigned parcels vs 42 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>possible-missing-parcel</t>
+          <t>units-undercount</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>181</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Alvarado Streets Apartments: parcel 5136019023 shares situs '1136 S ALVARADO ST LOS ANGELES CA 90006' (Auto, Recreation EQPT, C, $1,039,983) but is not assigned to any project</t>
+          <t>The Hive Apartments: county records 50 units on assigned parcels vs 152 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>possible-missing-parcel</t>
+          <t>units-undercount</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>195</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Market Street Village Apartmen: parcel 5351441600 shares situs '699 14TH SD' (31, $15,300,000) but is not assigned to any project</t>
+          <t>1723 Corinth Apartments: county records 10 units on assigned parcels vs 41 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>
@@ -76591,131 +76606,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>231</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>The Waterloo Apartments: county records 5 units on assigned parcels vs 154 in the grant — parcels may be missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>units-undercount</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>68</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>Candlewood North Apartments: county records 68 units on assigned parcels vs 189 in the grant — parcels may be missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>units-undercount</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>110</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Kenmore I Apartments: county records 24 units on assigned parcels vs 42 in the grant — parcels may be missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>units-undercount</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>181</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>The Hive Apartments: county records 50 units on assigned parcels vs 152 in the grant — parcels may be missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>units-undercount</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>195</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>1723 Corinth Apartments: county records 10 units on assigned parcels vs 41 in the grant — parcels may be missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>units-undercount</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>231</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
           <t>Violet on Virgil: county records 159 units on assigned parcels vs 302 in the grant — parcels may be missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>units-undercount</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>233</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>926 S. Kingsley Apartments: county records 1 units on assigned parcels vs 136 in the grant — parcels may be missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>units-undercount</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>237</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>Edgemont by Angeleno: county records 8 units on assigned parcels vs 34 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Alvarado parking parcel added; Market Street Village scoped to PAR 2
Alvarado gains same-situs parcel 5136019023 (likely complex parking,
ownership assumed — noted). Market Street Village is a 4-parcel map
(PAR 1-4); the grant covers PAR 2 exactly (229 units, entity '699
14TH Street CSLC LP') — commercial PAR 3 and the separate 242-unit
PAR 4 phase recorded as reviewed exclusions, and the sweep now
respects AINs noted as excluded so decisions stick.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -40962,7 +40962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U389"/>
+  <dimension ref="A1:U390"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -48497,6 +48497,11 @@
           <t>collaborator-sheet</t>
         </is>
       </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Reviewed 2026-08-22: grant covers PAR 2 only (229 units, per staff report and entity name). Same-situs siblings excluded: 5351441600 (PAR 3, commercial), 5351441400 (PAR 1), 5351441700 (PAR 4, 1450 Market — separate 242-unit phase).</t>
+        </is>
+      </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
           <t>2026</t>
@@ -74944,6 +74949,108 @@
       <c r="U389" s="2" t="inlineStr">
         <is>
           <t>no-situs</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Alvarado Streets Apartments</t>
+        </is>
+      </c>
+      <c r="D390" s="2" t="inlineStr">
+        <is>
+          <t>5136019023</t>
+        </is>
+      </c>
+      <c r="E390" s="2" t="inlineStr">
+        <is>
+          <t>5136-019-023</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>1136 S ALVARADO ST LOS ANGELES CA 90006</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>Added 2026-08-22 (Drew): same-situs Auto/Recreation parcel, likely complex parking; ownership not independently verified — assumed part of property</t>
+        </is>
+      </c>
+      <c r="K390" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L390" s="2" t="inlineStr">
+        <is>
+          <t>1039983</t>
+        </is>
+      </c>
+      <c r="M390" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N390" s="2" t="inlineStr">
+        <is>
+          <t>1039983</t>
+        </is>
+      </c>
+      <c r="O390" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P390" s="2" t="inlineStr">
+        <is>
+          <t>1952</t>
+        </is>
+      </c>
+      <c r="Q390" s="2" t="inlineStr">
+        <is>
+          <t>Auto, Recreation EQPT, Construction EQPT, Sales &amp; Service</t>
+        </is>
+      </c>
+      <c r="R390" s="2" t="inlineStr">
+        <is>
+          <t>la-county-api</t>
+        </is>
+      </c>
+      <c r="S390" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="T390" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U390" s="2" t="inlineStr">
+        <is>
+          <t>situs-match</t>
         </is>
       </c>
     </row>
@@ -74958,7 +75065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -76482,34 +76589,34 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>possible-missing-parcel</t>
+          <t>units-undercount</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Alvarado Streets Apartments: parcel 5136019023 shares situs '1136 S ALVARADO ST LOS ANGELES CA 90006' (Auto, Recreation EQPT, C, $1,039,983) but is not assigned to any project</t>
+          <t>The Waterloo Apartments: county records 5 units on assigned parcels vs 154 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>possible-missing-parcel</t>
+          <t>units-undercount</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>68</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Market Street Village Apartmen: parcel 5351441600 shares situs '699 14TH SD' (31, $15,300,000) but is not assigned to any project</t>
+          <t>Candlewood North Apartments: county records 68 units on assigned parcels vs 189 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>
@@ -76521,12 +76628,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>110</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>The Waterloo Apartments: county records 5 units on assigned parcels vs 154 in the grant — parcels may be missing</t>
+          <t>Kenmore I Apartments: county records 24 units on assigned parcels vs 42 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>
@@ -76538,12 +76645,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>181</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Candlewood North Apartments: county records 68 units on assigned parcels vs 189 in the grant — parcels may be missing</t>
+          <t>The Hive Apartments: county records 50 units on assigned parcels vs 152 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>
@@ -76555,12 +76662,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>195</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Kenmore I Apartments: county records 24 units on assigned parcels vs 42 in the grant — parcels may be missing</t>
+          <t>1723 Corinth Apartments: county records 10 units on assigned parcels vs 41 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>
@@ -76572,44 +76679,10 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>231</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
-        <is>
-          <t>The Hive Apartments: county records 50 units on assigned parcels vs 152 in the grant — parcels may be missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>units-undercount</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>195</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>1723 Corinth Apartments: county records 10 units on assigned parcels vs 41 in the grant — parcels may be missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>units-undercount</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>231</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
         <is>
           <t>Violet on Virgil: county records 159 units on assigned parcels vs 302 in the grant — parcels may be missing</t>
         </is>

</xml_diff>

<commit_message>
Waterloo: map both pre-construction parcels (5402-028-022/023)
Demolition not yet started; county values and unit counts reflect the
existing buildings — noted, and the units-undercount check now
respects 'units reviewed' notes so known pre-construction sites stop
flagging.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -40962,7 +40962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U390"/>
+  <dimension ref="A1:U391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42059,6 +42059,11 @@
           <t>manual_verified</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Pre-construction site (demolition not started): project will occupy 5402-028-023 and 5402-028-022; county values/units reflect existing buildings (units reviewed 2026-08-22, Drew)</t>
+        </is>
+      </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2026</t>
@@ -75049,6 +75054,103 @@
         </is>
       </c>
       <c r="U390" s="2" t="inlineStr">
+        <is>
+          <t>situs-match</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>The Waterloo Apartments</t>
+        </is>
+      </c>
+      <c r="D391" s="2" t="inlineStr">
+        <is>
+          <t>5402028022</t>
+        </is>
+      </c>
+      <c r="E391" s="2" t="inlineStr">
+        <is>
+          <t>5402-028-022</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>Pre-construction site (demolition not started): project will occupy 5402-028-023 and 5402-028-022; county values/units reflect existing buildings (units reviewed 2026-08-22, Drew)</t>
+        </is>
+      </c>
+      <c r="K391" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L391" s="2" t="inlineStr">
+        <is>
+          <t>831300</t>
+        </is>
+      </c>
+      <c r="M391" s="2" t="inlineStr">
+        <is>
+          <t>306000</t>
+        </is>
+      </c>
+      <c r="N391" s="2" t="inlineStr">
+        <is>
+          <t>1137300</t>
+        </is>
+      </c>
+      <c r="O391" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P391" s="2" t="inlineStr">
+        <is>
+          <t>1912</t>
+        </is>
+      </c>
+      <c r="Q391" s="2" t="inlineStr">
+        <is>
+          <t>Two Units</t>
+        </is>
+      </c>
+      <c r="R391" s="2" t="inlineStr">
+        <is>
+          <t>la-county-api</t>
+        </is>
+      </c>
+      <c r="S391" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="T391" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="U391" s="2" t="inlineStr">
         <is>
           <t>situs-match</t>
         </is>
@@ -75065,7 +75167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C95"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -76594,12 +76696,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>68</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>The Waterloo Apartments: county records 5 units on assigned parcels vs 154 in the grant — parcels may be missing</t>
+          <t>Candlewood North Apartments: county records 68 units on assigned parcels vs 189 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>
@@ -76611,12 +76713,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>110</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Candlewood North Apartments: county records 68 units on assigned parcels vs 189 in the grant — parcels may be missing</t>
+          <t>Kenmore I Apartments: county records 24 units on assigned parcels vs 42 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>
@@ -76628,12 +76730,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>181</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Kenmore I Apartments: county records 24 units on assigned parcels vs 42 in the grant — parcels may be missing</t>
+          <t>The Hive Apartments: county records 50 units on assigned parcels vs 152 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>
@@ -76645,12 +76747,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>195</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>The Hive Apartments: county records 50 units on assigned parcels vs 152 in the grant — parcels may be missing</t>
+          <t>1723 Corinth Apartments: county records 10 units on assigned parcels vs 41 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>
@@ -76662,27 +76764,10 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>231</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
-        <is>
-          <t>1723 Corinth Apartments: county records 10 units on assigned parcels vs 41 in the grant — parcels may be missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>units-undercount</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>231</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
         <is>
           <t>Violet on Virgil: county records 159 units on assigned parcels vs 302 in the grant — parcels may be missing</t>
         </is>

</xml_diff>

<commit_message>
Close units-undercount findings (Drew, assessor portal research)
Candlewood North spans 2764-001-012..014 (two parcels added); The
Hive's second address 5700 Ackerfield is 7157-012-023; Violet on
Virgil gains lot 5501-017-045; 1723 Corinth marked units-reviewed
(stale/pre-construction). Kenmore I's manual 42-unit override was a
transposition of 24 (staff report, county, and parcel all say 24) —
dropped, generated value flows.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -16059,14 +16059,14 @@
           <t>Kingdom Development, Inc.</t>
         </is>
       </c>
-      <c r="W111" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="X111" t="inlineStr">
-        <is>
-          <t>42</t>
+      <c r="W111" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="X111" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
         </is>
       </c>
       <c r="Y111" s="2" t="inlineStr">
@@ -16106,7 +16106,7 @@
       </c>
       <c r="AL111" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -40962,7 +40962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U391"/>
+  <dimension ref="A1:U395"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -65253,7 +65253,7 @@
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>Resolved by LA county situs/geocode search</t>
+          <t>Resolved by LA county situs/geocode search; Pre-construction/stale county record; building may not yet be built (units reviewed 2026-08-22, Drew)</t>
         </is>
       </c>
       <c r="K264" s="2" t="inlineStr">
@@ -75151,6 +75151,399 @@
         </is>
       </c>
       <c r="U391" s="2" t="inlineStr">
+        <is>
+          <t>situs-match</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Candlewood North Apartments</t>
+        </is>
+      </c>
+      <c r="D392" s="2" t="inlineStr">
+        <is>
+          <t>2764001012</t>
+        </is>
+      </c>
+      <c r="E392" s="2" t="inlineStr">
+        <is>
+          <t>2764-001-012</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>Added 2026-08-22 (Drew, assessor portal): complex spans 2764-001-012..014</t>
+        </is>
+      </c>
+      <c r="K392" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L392" s="2" t="inlineStr">
+        <is>
+          <t>8339520</t>
+        </is>
+      </c>
+      <c r="M392" s="2" t="inlineStr">
+        <is>
+          <t>7956000</t>
+        </is>
+      </c>
+      <c r="N392" s="2" t="inlineStr">
+        <is>
+          <t>16295520</t>
+        </is>
+      </c>
+      <c r="O392" s="2" t="inlineStr">
+        <is>
+          <t>8364491</t>
+        </is>
+      </c>
+      <c r="P392" s="2" t="inlineStr">
+        <is>
+          <t>1965</t>
+        </is>
+      </c>
+      <c r="Q392" s="2" t="inlineStr">
+        <is>
+          <t>Five or more apartments</t>
+        </is>
+      </c>
+      <c r="R392" s="2" t="inlineStr">
+        <is>
+          <t>la-county-api</t>
+        </is>
+      </c>
+      <c r="S392" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="T392" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="U392" s="2" t="inlineStr">
+        <is>
+          <t>situs-match</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Candlewood North Apartments</t>
+        </is>
+      </c>
+      <c r="D393" s="2" t="inlineStr">
+        <is>
+          <t>2764001014</t>
+        </is>
+      </c>
+      <c r="E393" s="2" t="inlineStr">
+        <is>
+          <t>2764-001-014</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>Added 2026-08-22 (Drew, assessor portal): complex spans 2764-001-012..014</t>
+        </is>
+      </c>
+      <c r="K393" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L393" s="2" t="inlineStr">
+        <is>
+          <t>9016800</t>
+        </is>
+      </c>
+      <c r="M393" s="2" t="inlineStr">
+        <is>
+          <t>8896440</t>
+        </is>
+      </c>
+      <c r="N393" s="2" t="inlineStr">
+        <is>
+          <t>17913240</t>
+        </is>
+      </c>
+      <c r="O393" s="2" t="inlineStr">
+        <is>
+          <t>9194867</t>
+        </is>
+      </c>
+      <c r="P393" s="2" t="inlineStr">
+        <is>
+          <t>1964</t>
+        </is>
+      </c>
+      <c r="Q393" s="2" t="inlineStr">
+        <is>
+          <t>Five or more apartments</t>
+        </is>
+      </c>
+      <c r="R393" s="2" t="inlineStr">
+        <is>
+          <t>la-county-api</t>
+        </is>
+      </c>
+      <c r="S393" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="T393" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="U393" s="2" t="inlineStr">
+        <is>
+          <t>situs-match</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>181</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>The Hive Apartments</t>
+        </is>
+      </c>
+      <c r="D394" s="2" t="inlineStr">
+        <is>
+          <t>7157012023</t>
+        </is>
+      </c>
+      <c r="E394" s="2" t="inlineStr">
+        <is>
+          <t>7157-012-023</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>5700 ACKERFIELD AVE LONG BEACH CA</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>Added 2026-08-22 (Drew): staff report prose gives two addresses, 5700 and 5565 Ackerfield; this is 5700</t>
+        </is>
+      </c>
+      <c r="K394" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L394" s="2" t="inlineStr">
+        <is>
+          <t>4762701</t>
+        </is>
+      </c>
+      <c r="M394" s="2" t="inlineStr">
+        <is>
+          <t>20566211</t>
+        </is>
+      </c>
+      <c r="N394" s="2" t="inlineStr">
+        <is>
+          <t>25328912</t>
+        </is>
+      </c>
+      <c r="O394" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P394" s="2" t="inlineStr">
+        <is>
+          <t>1973</t>
+        </is>
+      </c>
+      <c r="Q394" s="2" t="inlineStr">
+        <is>
+          <t>Five or more apartments</t>
+        </is>
+      </c>
+      <c r="R394" s="2" t="inlineStr">
+        <is>
+          <t>la-county-api</t>
+        </is>
+      </c>
+      <c r="S394" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="T394" t="inlineStr">
+        <is>
+          <t>181</t>
+        </is>
+      </c>
+      <c r="U394" s="2" t="inlineStr">
+        <is>
+          <t>situs-match</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>231</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Violet on Virgil</t>
+        </is>
+      </c>
+      <c r="D395" s="2" t="inlineStr">
+        <is>
+          <t>5501017045</t>
+        </is>
+      </c>
+      <c r="E395" s="2" t="inlineStr">
+        <is>
+          <t>5501-017-045</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>manual-repo-edit</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>Added 2026-08-22 (Drew, assessor portal): additional lot completing the 302-unit site</t>
+        </is>
+      </c>
+      <c r="K395" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L395" s="2" t="inlineStr">
+        <is>
+          <t>20247672</t>
+        </is>
+      </c>
+      <c r="M395" s="2" t="inlineStr">
+        <is>
+          <t>33588722</t>
+        </is>
+      </c>
+      <c r="N395" s="2" t="inlineStr">
+        <is>
+          <t>53836394</t>
+        </is>
+      </c>
+      <c r="O395" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P395" s="2" t="inlineStr">
+        <is>
+          <t>1972</t>
+        </is>
+      </c>
+      <c r="Q395" s="2" t="inlineStr">
+        <is>
+          <t>Five or more apartments</t>
+        </is>
+      </c>
+      <c r="R395" s="2" t="inlineStr">
+        <is>
+          <t>la-county-api</t>
+        </is>
+      </c>
+      <c r="S395" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="T395" t="inlineStr">
+        <is>
+          <t>231</t>
+        </is>
+      </c>
+      <c r="U395" s="2" t="inlineStr">
         <is>
           <t>situs-match</t>
         </is>
@@ -75167,7 +75560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -75999,12 +76392,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>134</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>total_units: generated '24' -&gt; manual '42'</t>
+          <t>total_units: generated '69' -&gt; manual '68'</t>
         </is>
       </c>
     </row>
@@ -76016,12 +76409,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>137</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>total_units: generated '69' -&gt; manual '68'</t>
+          <t>total_units: generated '42' -&gt; manual '41'</t>
         </is>
       </c>
     </row>
@@ -76033,12 +76426,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>152</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>total_units: generated '42' -&gt; manual '41'</t>
+          <t>total_units: generated '52' -&gt; manual '152'</t>
         </is>
       </c>
     </row>
@@ -76050,12 +76443,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>155</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>total_units: generated '52' -&gt; manual '152'</t>
+          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
         </is>
       </c>
     </row>
@@ -76067,7 +76460,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>156</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -76084,12 +76477,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>171</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
+          <t>city_cut: generated '15900.0' -&gt; manual '6300'</t>
         </is>
       </c>
     </row>
@@ -76101,12 +76494,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>171</t>
+          <t>181</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>city_cut: generated '15900.0' -&gt; manual '6300'</t>
+          <t>total_units: generated '52' -&gt; manual '152'</t>
         </is>
       </c>
     </row>
@@ -76118,12 +76511,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>195</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>total_units: generated '52' -&gt; manual '152'</t>
+          <t>total_units: generated '42' -&gt; manual '41'</t>
         </is>
       </c>
     </row>
@@ -76135,12 +76528,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>199</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>total_units: generated '42' -&gt; manual '41'</t>
+          <t>city_cut: generated '5550.0' -&gt; manual '5500'</t>
         </is>
       </c>
     </row>
@@ -76152,12 +76545,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>204</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>city_cut: generated '5550.0' -&gt; manual '5500'</t>
+          <t>total_units: generated '50' -&gt; manual '49'</t>
         </is>
       </c>
     </row>
@@ -76169,12 +76562,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>206</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>total_units: generated '50' -&gt; manual '49'</t>
+          <t>county: generated 'San Diego' -&gt; manual 'Los Angeles'</t>
         </is>
       </c>
     </row>
@@ -76186,12 +76579,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>209</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>county: generated 'San Diego' -&gt; manual 'Los Angeles'</t>
+          <t>investor_1: generated 'Zenith Property Group LLC' -&gt; manual 'Red Stone Equity Partners'</t>
         </is>
       </c>
     </row>
@@ -76208,7 +76601,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Zenith Property Group LLC' -&gt; manual 'Red Stone Equity Partners'</t>
+          <t>term_years: generated '35' -&gt; manual '15'</t>
         </is>
       </c>
     </row>
@@ -76220,12 +76613,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>210</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>term_years: generated '35' -&gt; manual '15'</t>
+          <t>term_years: generated '55' -&gt; manual '10'</t>
         </is>
       </c>
     </row>
@@ -76237,12 +76630,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>226</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>term_years: generated '55' -&gt; manual '10'</t>
+          <t>term_years: generated '15' -&gt; manual '10'</t>
         </is>
       </c>
     </row>
@@ -76254,12 +76647,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>228</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>term_years: generated '15' -&gt; manual '10'</t>
+          <t>term_years: generated '10' -&gt; manual '15'</t>
         </is>
       </c>
     </row>
@@ -76271,12 +76664,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>217</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>term_years: generated '10' -&gt; manual '15'</t>
+          <t>total_units: generated '35' -&gt; manual '34'</t>
         </is>
       </c>
     </row>
@@ -76288,12 +76681,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>217</t>
+          <t>233</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>total_units: generated '35' -&gt; manual '34'</t>
+          <t>term_years: generated '55' -&gt; manual '10'</t>
         </is>
       </c>
     </row>
@@ -76305,12 +76698,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>236</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>term_years: generated '55' -&gt; manual '10'</t>
+          <t>total_units: generated '136' -&gt; manual '108'</t>
         </is>
       </c>
     </row>
@@ -76322,29 +76715,29 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>225</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>total_units: generated '136' -&gt; manual '108'</t>
+          <t>term_years: generated '30' -&gt; manual '55'</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-possible-match</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>term_years: generated '30' -&gt; manual '55'</t>
+          <t>entity '381 Turk Street Associates, a California' ~ SCC LP '421 Turk Street Associates, L.P.' (#3326, San Francisco, score 92)</t>
         </is>
       </c>
     </row>
@@ -76356,12 +76749,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>33</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>entity '381 Turk Street Associates, a California' ~ SCC LP '421 Turk Street Associates, L.P.' (#3326, San Francisco, score 92)</t>
+          <t>entity 'BIF NON OZ 7524 S HOOVER ST, LP' ~ SCC LP 'BIF NON OZ 7518 S Hoover St, LP' (#14953, Los Angeles, score 93)</t>
         </is>
       </c>
     </row>
@@ -76373,12 +76766,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>entity 'BIF NON OZ 7524 S HOOVER ST, LP' ~ SCC LP 'BIF NON OZ 7518 S Hoover St, LP' (#14953, Los Angeles, score 93)</t>
+          <t>entity 'BIF NON OZ 4228 WESTERN AVE, LP' ~ SCC LP 'BIF NON OZ 4209 Western Ave, LP' (#14952, Los Angeles, score 93)</t>
         </is>
       </c>
     </row>
@@ -76390,12 +76783,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>122</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>entity 'BIF NON OZ 4228 WESTERN AVE, LP' ~ SCC LP 'BIF NON OZ 4209 Western Ave, LP' (#14952, Los Angeles, score 93)</t>
+          <t>entity '861 Fedora LLLP' ~ SCC LP '836 Fedora L.P.' (#1594, Los Angeles, score 90)</t>
         </is>
       </c>
     </row>
@@ -76407,7 +76800,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>165</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -76419,17 +76812,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>scc-possible-match</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>165</t>
+          <t>76</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>entity '861 Fedora LLLP' ~ SCC LP '836 Fedora L.P.' (#1594, Los Angeles, score 90)</t>
+          <t>AIN 5036031006 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
@@ -76441,12 +76834,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>99</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>AIN 5036031006 (Los Angeles) has no current roll data; using manual value</t>
+          <t>AIN 4262018026 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
@@ -76458,12 +76851,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>132</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>AIN 4262018026 (Los Angeles) has no current roll data; using manual value</t>
+          <t>AIN 6020022027 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
@@ -76475,29 +76868,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>137</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>AIN 6020022027 (Los Angeles) has no current roll data; using manual value</t>
+          <t>AIN 2125017014 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>fetch-fallback</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>158</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>AIN 2125017014 (Los Angeles) has no current roll data; using manual value</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -76509,7 +76902,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>196</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -76526,12 +76919,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>201</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN (none) (Santa Barbara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -76543,12 +76936,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>201</t>
+          <t>206</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>AIN (none) (Santa Barbara): no roll values from any source</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -76560,7 +76953,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>207</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -76577,7 +76970,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>208</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -76594,12 +76987,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>208</t>
+          <t>215</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN 5539028040 (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -76611,29 +77004,29 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>215</t>
+          <t>226</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>AIN 5539028040 (Los Angeles): no roll values from any source</t>
+          <t>AIN (none) (Contra Costa): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>AIN (none) (Contra Costa): no roll values from any source</t>
+          <t>AIN 128101150 (Solano) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
@@ -76650,7 +77043,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>AIN 128101150 (Solano) has no current roll data; using manual value</t>
+          <t>AIN 128101050 (Solano) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
@@ -76667,109 +77060,24 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>AIN 128101050 (Solano) has no current roll data; using manual value</t>
+          <t>AIN 128105060 (Solano) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>fetch-fallback</t>
+          <t>units-undercount</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>110</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>AIN 128105060 (Solano) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>units-undercount</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>68</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>Candlewood North Apartments: county records 68 units on assigned parcels vs 189 in the grant — parcels may be missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>units-undercount</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>110</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
           <t>Kenmore I Apartments: county records 24 units on assigned parcels vs 42 in the grant — parcels may be missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>units-undercount</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>181</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>The Hive Apartments: county records 50 units on assigned parcels vs 152 in the grant — parcels may be missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>units-undercount</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>195</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>1723 Corinth Apartments: county records 10 units on assigned parcels vs 41 in the grant — parcels may be missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>units-undercount</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>231</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>Violet on Virgil: county records 159 units on assigned parcels vs 302 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-run assignment checks post-rebuild; units-undercount cleared
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -75560,7 +75560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -77061,23 +77061,6 @@
       <c r="C88" t="inlineStr">
         <is>
           <t>AIN 128105060 (Solano) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>units-undercount</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>110</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>Kenmore I Apartments: county records 24 units on assigned parcels vs 42 in the grant — parcels may be missing</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
4228 Western: Healdsburg was an agenda error; one LA property, three events
Res 25-511 (2025-10-24) listed 'PS 4228 Western Ave, LP' under City
of Healdsburg, County of Sonoma — pulled at that meeting, then
re-agendized 2025-11-07 under Los Angeles as 25-531 and approved.
County/city overrides on 348 group all three rows as one property:
40 (BIF era) superseded, 348 pulled, 349 operative. No Sonoma
property ever existed; no parcels needed for pulled items.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -37727,14 +37727,14 @@
           <t>PS 4228 Western Ave, LP, a Delaware limited partnership</t>
         </is>
       </c>
-      <c r="E285" s="2" t="inlineStr">
-        <is>
-          <t>Healdsburg</t>
-        </is>
-      </c>
-      <c r="F285" s="2" t="inlineStr">
-        <is>
-          <t>Sonoma</t>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="G285" s="2" t="inlineStr">
@@ -37785,6 +37785,11 @@
       <c r="AK285" t="inlineStr">
         <is>
           <t>generated</t>
+        </is>
+      </c>
+      <c r="AL285" t="inlineStr">
+        <is>
+          <t>county:manual-repo-edit; city:manual-repo-edit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
QA check: operative grant without SCC when a superseded sibling holds one
An SCC belongs to the LP, not the property, so after a sponsor change the
prior LP's certificate matches only the superseded row and the operative
row correctly reads blank until the new LP files its own. New
scc-superseded-only finding surfaces the two current cases (132 Hoover,
134 Avalon — both BIF -> PS handoffs) so a blank isn't read as
"never filed".

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -75745,7 +75745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -77031,34 +77031,34 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>fetch-fallback</t>
+          <t>scc-superseded-only</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>132</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>AIN 5036031006 (Los Angeles) has no current roll data; using manual value</t>
+          <t>operative entity 'PS 7518 Hoover St, LP' has no SCC, but the property's superseded grant 10 ('BIF NON OZ 7518 S Hoover St, LP, a Delaw') holds SCC 14953 (2024-11-25) — new sponsor's LP must file its own</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>fetch-fallback</t>
+          <t>scc-superseded-only</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>134</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>AIN 4262018026 (Los Angeles) has no current roll data; using manual value</t>
+          <t>operative entity 'PS 10705 Avalon Blvd, LP' has no SCC, but the property's superseded grant 303 ('BIF NON OZ 10705 Avalon Blvd, LP, a Cali') holds SCC 14852 (2024-10-03) — new sponsor's LP must file its own</t>
         </is>
       </c>
     </row>
@@ -77070,12 +77070,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>76</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>AIN 6020022027 (Los Angeles) has no current roll data; using manual value</t>
+          <t>AIN 5036031006 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
@@ -77087,46 +77087,46 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>99</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>AIN 2125017014 (Los Angeles) has no current roll data; using manual value</t>
+          <t>AIN 4262018026 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>132</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN 6020022027 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>137</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN 2125017014 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
@@ -77138,12 +77138,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>201</t>
+          <t>158</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>AIN (none) (Santa Barbara): no roll values from any source</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -77155,7 +77155,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>196</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -77172,12 +77172,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>201</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN (none) (Santa Barbara): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -77189,7 +77189,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>208</t>
+          <t>206</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -77206,12 +77206,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>215</t>
+          <t>207</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>AIN 5539028040 (Los Angeles): no roll values from any source</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -77223,46 +77223,46 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>208</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>AIN (none) (Contra Costa): no roll values from any source</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>fetch-fallback</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>215</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>AIN 128101150 (Solano) has no current roll data; using manual value</t>
+          <t>AIN 5539028040 (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>fetch-fallback</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>226</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>AIN 128101050 (Solano) has no current roll data; using manual value</t>
+          <t>AIN (none) (Contra Costa): no roll values from any source</t>
         </is>
       </c>
     </row>
@@ -77278,6 +77278,40 @@
         </is>
       </c>
       <c r="C90" t="inlineStr">
+        <is>
+          <t>AIN 128101150 (Solano) has no current roll data; using manual value</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>fetch-fallback</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>AIN 128101050 (Solano) has no current roll data; using manual value</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>fetch-fallback</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
         <is>
           <t>AIN 128105060 (Solano) has no current roll data; using manual value</t>
         </is>

</xml_diff>

<commit_message>
Self-healing dedupe: same AIN under two authorizations of one property
When a property's parcels were researched under both an original grant
and its re-authorization, two live rows pointed at the same
operative_project_id and an operative-keyed SUMIF counted the parcel
twice (24 rows / 12 properties, mostly the Kadisha portfolio).
build_dataset now keeps the operative grant's own row and marks the
others legacy_redundant in the OUTPUT only (manual/ untouched), each
with a parcel-dedup QA finding. Future re-authorizations dedupe
automatically. README documents the two-id design and the exclusion
rule for sum formulas.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -58947,7 +58947,7 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
@@ -59049,7 +59049,7 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
@@ -59151,7 +59151,7 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
@@ -59253,7 +59253,7 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
@@ -59355,7 +59355,7 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
@@ -59457,7 +59457,7 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
@@ -59559,7 +59559,7 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
@@ -59661,7 +59661,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
@@ -59763,7 +59763,7 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
@@ -59865,7 +59865,7 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
@@ -60151,7 +60151,7 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
@@ -61398,7 +61398,7 @@
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="H219" t="inlineStr">
@@ -75745,7 +75745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -77314,6 +77314,210 @@
       <c r="C92" t="inlineStr">
         <is>
           <t>AIN 128105060 (Solano) has no current roll data; using manual value</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>parcel-dedup</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>AIN 5518013024 (Alexandria II Apartments) also assigned under operative grant 162; this row marked legacy_redundant so sums count it once</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>parcel-dedup</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>122</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>AIN 5094017020 (Fedora Apartments) also assigned under operative grant 165; this row marked legacy_redundant so sums count it once</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>parcel-dedup</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>AIN 5518020021 (Kenmore II Apartments) also assigned under operative grant 168; this row marked legacy_redundant so sums count it once</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>parcel-dedup</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>AIN 5094023025 (Kenmore III Apartments) also assigned under operative grant 169; this row marked legacy_redundant so sums count it once</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>parcel-dedup</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>AIN 5503024012 (Kingsley Apartments) also assigned under operative grant 170; this row marked legacy_redundant so sums count it once</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>parcel-dedup</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>126</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>AIN 5094005005 (Mariposa I Apartments) also assigned under operative grant 173; this row marked legacy_redundant so sums count it once</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>parcel-dedup</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>127</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>AIN 5094006003 (Mariposa III Apartments) also assigned under operative grant 174; this row marked legacy_redundant so sums count it once</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>parcel-dedup</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>AIN 5502019004 (Mariposa IV Apartments) also assigned under operative grant 175; this row marked legacy_redundant so sums count it once</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>parcel-dedup</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>AIN 5517005016 (Oxford II Apartments) also assigned under operative grant 177; this row marked legacy_redundant so sums count it once</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>parcel-dedup</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>AIN 5080006008 (Western Apartments) also assigned under operative grant 179; this row marked legacy_redundant so sums count it once</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>parcel-dedup</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>152</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>AIN 7157012023 (The Hive at Ackerfield Apartments) also assigned under operative grant 181; this row marked legacy_redundant so sums count it once</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>parcel-dedup</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>135</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>AIN 5518026004 (236 Berendo Apartments) also assigned under operative grant 220; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Unit-count parsing fixes + self-refuting conflict suppression
Parser (extract_total_units): handle thousands separators ("1,008-unit"
parsed as 8), never match "units per acre" (Seaport Village's 42 was a
density; real count 356 rentable units), add "N rentable units" pattern.

Merge: override-conflict findings are now skipped when (a) generated and
manual values agree (stale "differs" notes), or (b) the generated
total_units is below the generated restricted_units — impossible, the
signature of a multi-building property where the parser caught one
building, so the manual total wins without adjudication (Santa Monica
portfolios, The Hive). New units-inconsistent QA finding flags the
impossible signature when no manual override rescues it. Generic
multi-building summing deliberately not attempted (portfolio-context
numbers nearby would poison it).

override-conflict findings: 36 -> 28.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -37472,14 +37472,14 @@
       </c>
       <c r="W250" s="2" t="inlineStr">
         <is>
+          <t>1008</t>
+        </is>
+      </c>
+      <c r="X250" s="2" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="X250" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
       <c r="Y250" s="2" t="inlineStr">
         <is>
           <t>at 80% AMI</t>
@@ -37497,12 +37497,12 @@
       </c>
       <c r="AB250" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>604800</t>
         </is>
       </c>
       <c r="AC250" s="2" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>151200</t>
         </is>
       </c>
       <c r="AE250" s="2" t="inlineStr">
@@ -40124,14 +40124,14 @@
       </c>
       <c r="W271" s="2" t="inlineStr">
         <is>
+          <t>1008</t>
+        </is>
+      </c>
+      <c r="X271" s="2" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="X271" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
       <c r="Y271" s="2" t="inlineStr">
         <is>
           <t>at 80% AMI</t>
@@ -40149,12 +40149,12 @@
       </c>
       <c r="AB271" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>604800</t>
         </is>
       </c>
       <c r="AC271" s="2" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>151200</t>
         </is>
       </c>
       <c r="AE271" s="2" t="inlineStr">
@@ -40545,14 +40545,14 @@
       </c>
       <c r="W274" s="2" t="inlineStr">
         <is>
+          <t>1008</t>
+        </is>
+      </c>
+      <c r="X274" s="2" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="X274" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
       <c r="Y274" s="2" t="inlineStr">
         <is>
           <t>at 80% AMI</t>
@@ -40570,12 +40570,12 @@
       </c>
       <c r="AB274" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>604800</t>
         </is>
       </c>
       <c r="AC274" s="2" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>151200</t>
         </is>
       </c>
       <c r="AD274" s="2" t="inlineStr">
@@ -79943,7 +79943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -80520,12 +80520,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>48</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>total_units: generated '24' -&gt; manual '52'</t>
+          <t>investor_1: generated 'Ethos Real Estate' -&gt; manual 'Vistria Group'</t>
         </is>
       </c>
     </row>
@@ -80537,12 +80537,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>51</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>total_units: generated '22' -&gt; manual '72'</t>
+          <t>total_units: generated '144' -&gt; manual '145'</t>
         </is>
       </c>
     </row>
@@ -80554,12 +80554,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>total_units: generated '24' -&gt; manual '48'</t>
+          <t>total_units: generated '29' -&gt; manual '196'</t>
         </is>
       </c>
     </row>
@@ -80571,12 +80571,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>78</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>total_units: generated '65' -&gt; manual '165'</t>
+          <t>investor_1: generated 'Vintage Housing Holdings, LLC' -&gt; manual 'Kennedy Wilson'</t>
         </is>
       </c>
     </row>
@@ -80588,12 +80588,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>78</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Ethos Real Estate' -&gt; manual 'Vistria Group'</t>
+          <t>nonprofit_partner: generated 'Pacific Housing, Inc.' -&gt; manual 'Hearthstone Housing Foundation'</t>
         </is>
       </c>
     </row>
@@ -80605,12 +80605,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>81</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>total_units: generated '144' -&gt; manual '145'</t>
+          <t>total_units: generated '32' -&gt; manual '31'</t>
         </is>
       </c>
     </row>
@@ -80622,12 +80622,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>81</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>total_units: generated '42' -&gt; manual '356'</t>
+          <t>city_cut: generated '4650.0' -&gt; manual '4500'</t>
         </is>
       </c>
     </row>
@@ -80639,12 +80639,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>158</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>total_units: generated '29' -&gt; manual '196'</t>
+          <t>total_units: generated '30' -&gt; manual '29'</t>
         </is>
       </c>
     </row>
@@ -80656,12 +80656,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>95</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Vintage Housing Holdings, LLC' -&gt; manual 'Kennedy Wilson'</t>
+          <t>investor_1: generated 'Belveron Partners' -&gt; manual 'Sack Capital Partners'</t>
         </is>
       </c>
     </row>
@@ -80673,12 +80673,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>134</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>nonprofit_partner: generated 'Pacific Housing, Inc.' -&gt; manual 'Hearthstone Housing Foundation'</t>
+          <t>total_units: generated '69' -&gt; manual '68'</t>
         </is>
       </c>
     </row>
@@ -80690,12 +80690,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>137</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>total_units: generated '8' -&gt; manual '1008'</t>
+          <t>total_units: generated '42' -&gt; manual '41'</t>
         </is>
       </c>
     </row>
@@ -80707,12 +80707,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>155</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>total_units: generated '32' -&gt; manual '31'</t>
+          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
         </is>
       </c>
     </row>
@@ -80724,12 +80724,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>156</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>city_cut: generated '4650.0' -&gt; manual '4500'</t>
+          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
         </is>
       </c>
     </row>
@@ -80741,12 +80741,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>171</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>total_units: generated '30' -&gt; manual '29'</t>
+          <t>city_cut: generated '15900.0' -&gt; manual '6300'</t>
         </is>
       </c>
     </row>
@@ -80758,12 +80758,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>195</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Belveron Partners' -&gt; manual 'Sack Capital Partners'</t>
+          <t>total_units: generated '42' -&gt; manual '41'</t>
         </is>
       </c>
     </row>
@@ -80775,12 +80775,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>199</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>total_units: generated '69' -&gt; manual '68'</t>
+          <t>city_cut: generated '5550.0' -&gt; manual '5500'</t>
         </is>
       </c>
     </row>
@@ -80792,12 +80792,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>204</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>total_units: generated '42' -&gt; manual '41'</t>
+          <t>total_units: generated '50' -&gt; manual '49'</t>
         </is>
       </c>
     </row>
@@ -80809,12 +80809,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>206</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>total_units: generated '52' -&gt; manual '152'</t>
+          <t>county: generated 'San Diego' -&gt; manual 'Los Angeles'</t>
         </is>
       </c>
     </row>
@@ -80826,12 +80826,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>209</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
+          <t>investor_1: generated 'Zenith Property Group LLC' -&gt; manual 'Red Stone Equity Partners'</t>
         </is>
       </c>
     </row>
@@ -80843,12 +80843,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>209</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
+          <t>term_years: generated '35' -&gt; manual '15'</t>
         </is>
       </c>
     </row>
@@ -80860,12 +80860,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>171</t>
+          <t>210</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>city_cut: generated '15900.0' -&gt; manual '6300'</t>
+          <t>term_years: generated '55' -&gt; manual '10'</t>
         </is>
       </c>
     </row>
@@ -80877,12 +80877,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>226</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>total_units: generated '52' -&gt; manual '152'</t>
+          <t>term_years: generated '15' -&gt; manual '10'</t>
         </is>
       </c>
     </row>
@@ -80894,12 +80894,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>228</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>total_units: generated '42' -&gt; manual '41'</t>
+          <t>term_years: generated '10' -&gt; manual '15'</t>
         </is>
       </c>
     </row>
@@ -80911,12 +80911,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>217</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>city_cut: generated '5550.0' -&gt; manual '5500'</t>
+          <t>total_units: generated '35' -&gt; manual '34'</t>
         </is>
       </c>
     </row>
@@ -80928,12 +80928,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>233</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>total_units: generated '50' -&gt; manual '49'</t>
+          <t>term_years: generated '55' -&gt; manual '10'</t>
         </is>
       </c>
     </row>
@@ -80945,12 +80945,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>236</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>county: generated 'San Diego' -&gt; manual 'Los Angeles'</t>
+          <t>total_units: generated '136' -&gt; manual '108'</t>
         </is>
       </c>
     </row>
@@ -80962,556 +80962,556 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>225</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Zenith Property Group LLC' -&gt; manual 'Red Stone Equity Partners'</t>
+          <t>term_years: generated '30' -&gt; manual '55'</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-possible-match</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>term_years: generated '35' -&gt; manual '15'</t>
+          <t>entity '381 Turk Street Associates, a California' ~ SCC LP '421 Turk Street Associates, L.P.' (#3326, San Francisco, score 92)</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-possible-match</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>33</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>term_years: generated '55' -&gt; manual '10'</t>
+          <t>entity 'BIF NON OZ 7524 S HOOVER ST, LP' ~ SCC LP 'BIF NON OZ 7518 S Hoover St, LP' (#14953, Los Angeles, score 93)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-possible-match</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>term_years: generated '15' -&gt; manual '10'</t>
+          <t>entity 'BIF NON OZ 4228 WESTERN AVE, LP' ~ SCC LP 'BIF NON OZ 4209 Western Ave, LP' (#14952, Los Angeles, score 93)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-manual-unmatched</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>48</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>term_years: generated '10' -&gt; manual '15'</t>
+          <t>manual scc_filed=True but no BOE certificate matches entity 'Hillsdale Property LP'; closest: 'Hillsdale Property San Mateo, LP' (#15018, San Mateo, score 78)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-manual-unmatched</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>217</t>
+          <t>58</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>total_units: generated '35' -&gt; manual '34'</t>
+          <t>manual scc_filed=True but no BOE certificate matches entity 'Post Chaparral, LP, a Delaware limited p'; closest: 'Post Palmdale Chaparral, LP' (#15197, Los Angeles, score 76)</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-possible-match</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>122</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>term_years: generated '55' -&gt; manual '10'</t>
+          <t>entity '861 Fedora LLLP' ~ SCC LP '836 Fedora L.P.' (#1594, Los Angeles, score 90)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-possible-match</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>165</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>total_units: generated '136' -&gt; manual '108'</t>
+          <t>entity '861 Fedora LLLP' ~ SCC LP '836 Fedora L.P.' (#1594, Los Angeles, score 90)</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-superseded-only</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>132</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>term_years: generated '30' -&gt; manual '55'</t>
+          <t>operative entity 'PS 7518 Hoover St, LP' has no SCC, but the property's superseded grant 10 ('BIF NON OZ 7518 S Hoover St, LP, a Delaw') holds SCC 14953 (2024-11-25) — new sponsor's LP must file its own</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>scc-possible-match</t>
+          <t>scc-superseded-only</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>134</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>entity '381 Turk Street Associates, a California' ~ SCC LP '421 Turk Street Associates, L.P.' (#3326, San Francisco, score 92)</t>
+          <t>operative entity 'PS 10705 Avalon Blvd, LP' has no SCC, but the property's superseded grant 303 ('BIF NON OZ 10705 Avalon Blvd, LP, a Cali') holds SCC 14852 (2024-10-03) — new sponsor's LP must file its own</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>scc-possible-match</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>76</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>entity 'BIF NON OZ 7524 S HOOVER ST, LP' ~ SCC LP 'BIF NON OZ 7518 S Hoover St, LP' (#14953, Los Angeles, score 93)</t>
+          <t>AIN 5036031006 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>scc-possible-match</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>99</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>entity 'BIF NON OZ 4228 WESTERN AVE, LP' ~ SCC LP 'BIF NON OZ 4209 Western Ave, LP' (#14952, Los Angeles, score 93)</t>
+          <t>AIN 4262018026 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>scc-manual-unmatched</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>132</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>manual scc_filed=True but no BOE certificate matches entity 'Hillsdale Property LP'; closest: 'Hillsdale Property San Mateo, LP' (#15018, San Mateo, score 78)</t>
+          <t>AIN 6020022027 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>scc-manual-unmatched</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>137</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>manual scc_filed=True but no BOE certificate matches entity 'Post Chaparral, LP, a Delaware limited p'; closest: 'Post Palmdale Chaparral, LP' (#15197, Los Angeles, score 76)</t>
+          <t>AIN 2125017014 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>scc-possible-match</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>158</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>entity '861 Fedora LLLP' ~ SCC LP '836 Fedora L.P.' (#1594, Los Angeles, score 90)</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>scc-possible-match</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>165</t>
+          <t>196</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>entity '861 Fedora LLLP' ~ SCC LP '836 Fedora L.P.' (#1594, Los Angeles, score 90)</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>scc-superseded-only</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>201</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>operative entity 'PS 7518 Hoover St, LP' has no SCC, but the property's superseded grant 10 ('BIF NON OZ 7518 S Hoover St, LP, a Delaw') holds SCC 14953 (2024-11-25) — new sponsor's LP must file its own</t>
+          <t>AIN (none) (Santa Barbara): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>scc-superseded-only</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>206</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>operative entity 'PS 10705 Avalon Blvd, LP' has no SCC, but the property's superseded grant 303 ('BIF NON OZ 10705 Avalon Blvd, LP, a Cali') holds SCC 14852 (2024-10-03) — new sponsor's LP must file its own</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>fetch-fallback</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>207</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>AIN 5036031006 (Los Angeles) has no current roll data; using manual value</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>fetch-fallback</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>208</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>AIN 4262018026 (Los Angeles) has no current roll data; using manual value</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>fetch-fallback</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>215</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>AIN 6020022027 (Los Angeles) has no current roll data; using manual value</t>
+          <t>AIN 5539028040 (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>fetch-fallback</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>226</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>AIN 2125017014 (Los Angeles) has no current roll data; using manual value</t>
+          <t>AIN (none) (Contra Costa): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN 128101150 (Solano) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN 128101050 (Solano) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>201</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>AIN (none) (Santa Barbara): no roll values from any source</t>
+          <t>AIN 128105060 (Solano) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>121</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN 5518013024 (Alexandria II Apartments) also assigned under operative grant 162; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>122</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN 5094017020 (Fedora Apartments) also assigned under operative grant 165; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>208</t>
+          <t>123</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
+          <t>AIN 5518020021 (Kenmore II Apartments) also assigned under operative grant 168; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>215</t>
+          <t>124</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>AIN 5539028040 (Los Angeles): no roll values from any source</t>
+          <t>AIN 5094023025 (Kenmore III Apartments) also assigned under operative grant 169; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>parcel-no-values</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>125</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>AIN (none) (Contra Costa): no roll values from any source</t>
+          <t>AIN 5503024012 (Kingsley Apartments) also assigned under operative grant 170; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>fetch-fallback</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>126</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>AIN 128101150 (Solano) has no current roll data; using manual value</t>
+          <t>AIN 5094005005 (Mariposa I Apartments) also assigned under operative grant 173; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>fetch-fallback</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>127</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>AIN 128101050 (Solano) has no current roll data; using manual value</t>
+          <t>AIN 5094006003 (Mariposa III Apartments) also assigned under operative grant 174; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>fetch-fallback</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>128</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>AIN 128105060 (Solano) has no current roll data; using manual value</t>
+          <t>AIN 5502019004 (Mariposa IV Apartments) also assigned under operative grant 175; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
@@ -81523,12 +81523,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>129</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>AIN 5518013024 (Alexandria II Apartments) also assigned under operative grant 162; this row marked legacy_redundant so sums count it once</t>
+          <t>AIN 5517005016 (Oxford II Apartments) also assigned under operative grant 177; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
@@ -81540,12 +81540,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>130</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>AIN 5094017020 (Fedora Apartments) also assigned under operative grant 165; this row marked legacy_redundant so sums count it once</t>
+          <t>AIN 5080006008 (Western Apartments) also assigned under operative grant 179; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
@@ -81557,12 +81557,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>152</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>AIN 5518020021 (Kenmore II Apartments) also assigned under operative grant 168; this row marked legacy_redundant so sums count it once</t>
+          <t>AIN 7157012023 (The Hive at Ackerfield Apartments) also assigned under operative grant 181; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
@@ -81574,146 +81574,10 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>124</t>
+          <t>135</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
-        <is>
-          <t>AIN 5094023025 (Kenmore III Apartments) also assigned under operative grant 169; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>125</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>AIN 5503024012 (Kingsley Apartments) also assigned under operative grant 170; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>126</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>AIN 5094005005 (Mariposa I Apartments) also assigned under operative grant 173; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>127</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>AIN 5094006003 (Mariposa III Apartments) also assigned under operative grant 174; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>128</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>AIN 5502019004 (Mariposa IV Apartments) also assigned under operative grant 175; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>129</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>AIN 5517005016 (Oxford II Apartments) also assigned under operative grant 177; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>130</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>AIN 5080006008 (Western Apartments) also assigned under operative grant 179; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>152</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>AIN 7157012023 (The Hive at Ackerfield Apartments) also assigned under operative grant 181; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>135</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
         <is>
           <t>AIN 5518026004 (236 Berendo Apartments) also assigned under operative grant 220; this row marked legacy_redundant so sums count it once</t>
         </is>

</xml_diff>

<commit_message>
Incorporate Drew's override adjudications (QA findings review 2026-08)
Drew reviewed every override-conflict against source documents and
portals; rulings incorporated:

- 28 overrides dropped where the generated value proved correct
  (investors, term_years, city_cut, county, entity, and the off-by-one
  manager's-unit totals), including 78's paired investor_2 row and two
  made redundant by the parser fixes (54 Seaport, 78 Bella Vista).
- 7 kept where manual proved correct (Santa Monica portfolio sums,
  Creekside 145, Harken 196, and Eleos-for-consistency on 2), with notes
  rewritten to record the adjudication instead of firing conflicts.
- The Hive (152/181): both prior values wrong — corrected to 153 units
  including the manager's unit (fees recompute to $91,800 / $22,950).

override-conflict findings: 28 -> 0. QA total: 95 -> 67.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -467,7 +467,7 @@
     <col width="38" customWidth="1" min="17" max="17"/>
     <col width="38" customWidth="1" min="18" max="18"/>
     <col width="38" customWidth="1" min="19" max="19"/>
-    <col width="30" customWidth="1" min="20" max="20"/>
+    <col width="31" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="38" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
@@ -8203,9 +8203,9 @@
           <t>2-CMFA-Minutes-10-11-2024-1.pdf</t>
         </is>
       </c>
-      <c r="T49" t="inlineStr">
-        <is>
-          <t>Vistria Group</t>
+      <c r="T49" s="2" t="inlineStr">
+        <is>
+          <t>Ethos Real Estate</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -8280,7 +8280,7 @@
       </c>
       <c r="AO49" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; scc_filed:collaborator-sheet; investor_1:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; scc_filed:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -9160,7 +9160,7 @@
           <t>Pacific Housing, Inc.</t>
         </is>
       </c>
-      <c r="W55" t="inlineStr">
+      <c r="W55" s="2" t="inlineStr">
         <is>
           <t>356</t>
         </is>
@@ -9222,7 +9222,7 @@
       </c>
       <c r="AO55" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; resolution:collaborator-sheet; total_units:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; resolution:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -12913,22 +12913,22 @@
           <t>2-CMFA-Minutes-06-27-2025.pdf</t>
         </is>
       </c>
-      <c r="T79" t="inlineStr">
+      <c r="T79" s="2" t="inlineStr">
+        <is>
+          <t>Vintage Housing Holdings, LLC</t>
+        </is>
+      </c>
+      <c r="U79" s="2" t="inlineStr">
         <is>
           <t>Kennedy Wilson</t>
         </is>
       </c>
-      <c r="U79" t="inlineStr">
-        <is>
-          <t>Vintage Housing Holdings</t>
-        </is>
-      </c>
-      <c r="V79" t="inlineStr">
-        <is>
-          <t>Hearthstone Housing Foundation</t>
-        </is>
-      </c>
-      <c r="W79" t="inlineStr">
+      <c r="V79" s="2" t="inlineStr">
+        <is>
+          <t>Pacific Housing, Inc.</t>
+        </is>
+      </c>
+      <c r="W79" s="2" t="inlineStr">
         <is>
           <t>1008</t>
         </is>
@@ -12995,7 +12995,7 @@
       </c>
       <c r="AO79" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; new_build:collaborator-sheet; link:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; link:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -13374,9 +13374,9 @@
           <t>Housing on Merit</t>
         </is>
       </c>
-      <c r="W82" t="inlineStr">
-        <is>
-          <t>31</t>
+      <c r="W82" s="2" t="inlineStr">
+        <is>
+          <t>32</t>
         </is>
       </c>
       <c r="X82" t="inlineStr">
@@ -13394,14 +13394,14 @@
           <t>30</t>
         </is>
       </c>
-      <c r="AA82" t="inlineStr">
-        <is>
-          <t>4500</t>
+      <c r="AA82" s="2" t="inlineStr">
+        <is>
+          <t>4650.0</t>
         </is>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
-          <t>18600</t>
+          <t>19200</t>
         </is>
       </c>
       <c r="AC82" s="2" t="inlineStr">
@@ -13436,7 +13436,7 @@
       </c>
       <c r="AO82" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; restricted_units:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -15492,9 +15492,9 @@
           <t>2-CMFA-Minutes-08-08-25.pdf</t>
         </is>
       </c>
-      <c r="T96" t="inlineStr">
-        <is>
-          <t>Sack Capital Partners</t>
+      <c r="T96" s="2" t="inlineStr">
+        <is>
+          <t>Belveron Partners</t>
         </is>
       </c>
       <c r="U96" t="inlineStr">
@@ -15574,7 +15574,7 @@
       </c>
       <c r="AO96" t="inlineStr">
         <is>
-          <t>investor_2:collaborator-sheet; acquisition_date:collaborator-sheet; link:collaborator-sheet; resolution:collaborator-sheet; investor_1:collaborator-sheet; address:collaborator-sheet</t>
+          <t>investor_2:collaborator-sheet; acquisition_date:collaborator-sheet; link:collaborator-sheet; resolution:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -21228,16 +21228,16 @@
           <t>Housing On Merit</t>
         </is>
       </c>
-      <c r="W134" t="inlineStr">
+      <c r="W134" s="2" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="X134" s="2" t="inlineStr">
         <is>
           <t>68</t>
         </is>
       </c>
-      <c r="X134" s="2" t="inlineStr">
-        <is>
-          <t>68</t>
-        </is>
-      </c>
       <c r="Y134" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -21255,12 +21255,12 @@
       </c>
       <c r="AB134" s="2" t="inlineStr">
         <is>
-          <t>40800</t>
+          <t>41400</t>
         </is>
       </c>
       <c r="AC134" s="2" t="inlineStr">
         <is>
-          <t>10200</t>
+          <t>10350</t>
         </is>
       </c>
       <c r="AD134" s="2" t="inlineStr">
@@ -21290,7 +21290,7 @@
       </c>
       <c r="AO134" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -21659,16 +21659,16 @@
           <t>Las Palmas Housing &amp; Development Corporation</t>
         </is>
       </c>
-      <c r="W137" t="inlineStr">
+      <c r="W137" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="X137" s="2" t="inlineStr">
         <is>
           <t>41</t>
         </is>
       </c>
-      <c r="X137" s="2" t="inlineStr">
-        <is>
-          <t>41</t>
-        </is>
-      </c>
       <c r="Y137" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -21686,12 +21686,12 @@
       </c>
       <c r="AB137" s="2" t="inlineStr">
         <is>
-          <t>24600</t>
+          <t>25200</t>
         </is>
       </c>
       <c r="AC137" s="2" t="inlineStr">
         <is>
-          <t>6150</t>
+          <t>6300</t>
         </is>
       </c>
       <c r="AD137" s="2" t="inlineStr">
@@ -21721,7 +21721,7 @@
       </c>
       <c r="AO137" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -23936,14 +23936,14 @@
       </c>
       <c r="W152" t="inlineStr">
         <is>
+          <t>153</t>
+        </is>
+      </c>
+      <c r="X152" s="2" t="inlineStr">
+        <is>
           <t>152</t>
         </is>
       </c>
-      <c r="X152" s="2" t="inlineStr">
-        <is>
-          <t>152</t>
-        </is>
-      </c>
       <c r="Y152" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -23961,12 +23961,12 @@
       </c>
       <c r="AB152" s="2" t="inlineStr">
         <is>
-          <t>91200</t>
+          <t>91800</t>
         </is>
       </c>
       <c r="AC152" s="2" t="inlineStr">
         <is>
-          <t>22800</t>
+          <t>22950</t>
         </is>
       </c>
       <c r="AE152" s="2" t="inlineStr">
@@ -23991,7 +23991,7 @@
       </c>
       <c r="AO152" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; total_units:manual-repo-edit; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -24310,9 +24310,9 @@
           <t>Trailview Apartments</t>
         </is>
       </c>
-      <c r="D155" t="inlineStr">
-        <is>
-          <t>TBD LP</t>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>A limited partnership to be formed by Kairos Investment Management and Pacific Housing</t>
         </is>
       </c>
       <c r="E155" s="2" t="inlineStr">
@@ -24442,7 +24442,7 @@
       </c>
       <c r="AO155" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; built:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; built:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -24462,9 +24462,9 @@
           <t>Casa Serena Apartments</t>
         </is>
       </c>
-      <c r="D156" t="inlineStr">
-        <is>
-          <t>TBD LP</t>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>A limited partnership to be formed by Kairos Investment Management and Pacific Housing</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
@@ -24594,7 +24594,7 @@
       </c>
       <c r="AO156" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; built:collaborator-sheet; entity:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; built:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -24796,16 +24796,16 @@
           <t>A Community of Friends</t>
         </is>
       </c>
-      <c r="W158" t="inlineStr">
+      <c r="W158" s="2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="X158" s="2" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="X158" s="2" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
       <c r="Y158" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -24823,7 +24823,7 @@
       </c>
       <c r="AB158" s="2" t="inlineStr">
         <is>
-          <t>17400</t>
+          <t>18000</t>
         </is>
       </c>
       <c r="AC158" s="2" t="inlineStr">
@@ -24853,7 +24853,7 @@
       </c>
       <c r="AO158" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet; total_units:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; manual_status:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -26662,21 +26662,21 @@
           <t>55</t>
         </is>
       </c>
-      <c r="AA171" t="inlineStr">
+      <c r="AA171" s="2" t="inlineStr">
+        <is>
+          <t>15900.0</t>
+        </is>
+      </c>
+      <c r="AB171" s="2" t="inlineStr">
+        <is>
+          <t>25200</t>
+        </is>
+      </c>
+      <c r="AC171" s="2" t="inlineStr">
         <is>
           <t>6300</t>
         </is>
       </c>
-      <c r="AB171" s="2" t="inlineStr">
-        <is>
-          <t>25200</t>
-        </is>
-      </c>
-      <c r="AC171" s="2" t="inlineStr">
-        <is>
-          <t>6300</t>
-        </is>
-      </c>
       <c r="AD171" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -26699,7 +26699,7 @@
       </c>
       <c r="AO171" t="inlineStr">
         <is>
-          <t>address:collaborator-sheet; city_cut:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -28049,14 +28049,14 @@
       </c>
       <c r="W181" t="inlineStr">
         <is>
+          <t>153</t>
+        </is>
+      </c>
+      <c r="X181" s="2" t="inlineStr">
+        <is>
           <t>152</t>
         </is>
       </c>
-      <c r="X181" s="2" t="inlineStr">
-        <is>
-          <t>152</t>
-        </is>
-      </c>
       <c r="Y181" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -28074,12 +28074,12 @@
       </c>
       <c r="AB181" s="2" t="inlineStr">
         <is>
-          <t>91200</t>
+          <t>91800</t>
         </is>
       </c>
       <c r="AC181" s="2" t="inlineStr">
         <is>
-          <t>22800</t>
+          <t>22950</t>
         </is>
       </c>
       <c r="AD181" s="2" t="inlineStr">
@@ -28104,7 +28104,7 @@
       </c>
       <c r="AO181" t="inlineStr">
         <is>
-          <t>manual_status:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>manual_status:collaborator-sheet; total_units:manual-repo-edit; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -29863,16 +29863,16 @@
           <t>Foundation for Affordable Housing</t>
         </is>
       </c>
-      <c r="W194" t="inlineStr">
+      <c r="W194" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="X194" s="2" t="inlineStr">
         <is>
           <t>41</t>
         </is>
       </c>
-      <c r="X194" s="2" t="inlineStr">
-        <is>
-          <t>41</t>
-        </is>
-      </c>
       <c r="Y194" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -29890,12 +29890,12 @@
       </c>
       <c r="AB194" s="2" t="inlineStr">
         <is>
-          <t>24600</t>
+          <t>25200</t>
         </is>
       </c>
       <c r="AC194" s="2" t="inlineStr">
         <is>
-          <t>6150</t>
+          <t>6300</t>
         </is>
       </c>
       <c r="AD194" s="2" t="inlineStr">
@@ -29925,7 +29925,7 @@
       </c>
       <c r="AO194" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; address:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -30446,9 +30446,9 @@
           <t>30</t>
         </is>
       </c>
-      <c r="AA198" t="inlineStr">
-        <is>
-          <t>5500</t>
+      <c r="AA198" s="2" t="inlineStr">
+        <is>
+          <t>5550.0</t>
         </is>
       </c>
       <c r="AB198" s="2" t="inlineStr">
@@ -30483,7 +30483,7 @@
       </c>
       <c r="AO198" t="inlineStr">
         <is>
-          <t>city_cut:collaborator-sheet; address:manual-repo-edit</t>
+          <t>address:manual-repo-edit</t>
         </is>
       </c>
     </row>
@@ -31141,16 +31141,16 @@
           <t>Las Palmas Housing &amp; Development Corporation</t>
         </is>
       </c>
-      <c r="W203" t="inlineStr">
+      <c r="W203" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="X203" s="2" t="inlineStr">
         <is>
           <t>49</t>
         </is>
       </c>
-      <c r="X203" s="2" t="inlineStr">
-        <is>
-          <t>49</t>
-        </is>
-      </c>
       <c r="Y203" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -31168,12 +31168,12 @@
       </c>
       <c r="AB203" s="2" t="inlineStr">
         <is>
-          <t>29400</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="AC203" s="2" t="inlineStr">
         <is>
-          <t>7350</t>
+          <t>7500</t>
         </is>
       </c>
       <c r="AD203" s="2" t="inlineStr">
@@ -31203,7 +31203,7 @@
       </c>
       <c r="AO203" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; address:manual-repo-edit</t>
+          <t>new_build:collaborator-sheet; address:manual-repo-edit</t>
         </is>
       </c>
     </row>
@@ -31370,9 +31370,9 @@
           <t>Escondido</t>
         </is>
       </c>
-      <c r="F205" t="inlineStr">
-        <is>
-          <t>Los Angeles</t>
+      <c r="F205" s="2" t="inlineStr">
+        <is>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -31487,7 +31487,7 @@
       </c>
       <c r="AO205" t="inlineStr">
         <is>
-          <t>manual_status:collaborator-sheet; county:collaborator-sheet; address:collaborator-sheet</t>
+          <t>manual_status:collaborator-sheet; address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -31831,9 +31831,9 @@
           <t>2-CMFA-Minutes-05-29-26.pdf</t>
         </is>
       </c>
-      <c r="T208" t="inlineStr">
-        <is>
-          <t>Red Stone Equity Partners</t>
+      <c r="T208" s="2" t="inlineStr">
+        <is>
+          <t>Zenith Property Group LLC</t>
         </is>
       </c>
       <c r="V208" s="2" t="inlineStr">
@@ -31856,9 +31856,9 @@
           <t>100% at 80% AMI</t>
         </is>
       </c>
-      <c r="Z208" t="inlineStr">
-        <is>
-          <t>15</t>
+      <c r="Z208" s="2" t="inlineStr">
+        <is>
+          <t>35</t>
         </is>
       </c>
       <c r="AA208" s="2" t="inlineStr">
@@ -31898,7 +31898,7 @@
       </c>
       <c r="AO208" t="inlineStr">
         <is>
-          <t>investor_1:collaborator-sheet; address:collaborator-sheet; term_years:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -31998,9 +31998,9 @@
           <t>100% at 80% AMI</t>
         </is>
       </c>
-      <c r="Z209" t="inlineStr">
-        <is>
-          <t>10</t>
+      <c r="Z209" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
         </is>
       </c>
       <c r="AB209" s="2" t="inlineStr">
@@ -32031,11 +32031,6 @@
       <c r="AN209" t="inlineStr">
         <is>
           <t>generated</t>
-        </is>
-      </c>
-      <c r="AO209" t="inlineStr">
-        <is>
-          <t>term_years:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -32977,16 +32972,16 @@
           <t>Las Palmas Housing &amp; Development Corporation</t>
         </is>
       </c>
-      <c r="W216" t="inlineStr">
+      <c r="W216" s="2" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="X216" s="2" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="X216" s="2" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
       <c r="Y216" s="2" t="inlineStr">
         <is>
           <t>100% at 80% AMI</t>
@@ -33004,12 +32999,12 @@
       </c>
       <c r="AB216" s="2" t="inlineStr">
         <is>
-          <t>20400</t>
+          <t>21000</t>
         </is>
       </c>
       <c r="AC216" s="2" t="inlineStr">
         <is>
-          <t>5100</t>
+          <t>5250</t>
         </is>
       </c>
       <c r="AD216" s="2" t="inlineStr">
@@ -33039,7 +33034,7 @@
       </c>
       <c r="AO216" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; total_units:collaborator-sheet; address:manual-repo-edit</t>
+          <t>new_build:collaborator-sheet; address:manual-repo-edit</t>
         </is>
       </c>
     </row>
@@ -34033,9 +34028,9 @@
           <t>100% at 80% AMI</t>
         </is>
       </c>
-      <c r="Z224" t="inlineStr">
-        <is>
-          <t>55</t>
+      <c r="Z224" s="2" t="inlineStr">
+        <is>
+          <t>30</t>
         </is>
       </c>
       <c r="AA224" s="2" t="inlineStr">
@@ -34075,7 +34070,7 @@
       </c>
       <c r="AO224" t="inlineStr">
         <is>
-          <t>address:collaborator-sheet; term_years:collaborator-sheet</t>
+          <t>address:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -34170,9 +34165,9 @@
           <t>80% at 80% AMI</t>
         </is>
       </c>
-      <c r="Z225" t="inlineStr">
-        <is>
-          <t>10</t>
+      <c r="Z225" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
         </is>
       </c>
       <c r="AB225" s="2" t="inlineStr">
@@ -34212,7 +34207,7 @@
       </c>
       <c r="AO225" t="inlineStr">
         <is>
-          <t>manual_status:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet; term_years:collaborator-sheet</t>
+          <t>manual_status:collaborator-sheet; investor_1:collaborator-sheet; nonprofit_partner:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -34434,9 +34429,9 @@
           <t>50% at 80% AMI</t>
         </is>
       </c>
-      <c r="Z227" t="inlineStr">
-        <is>
-          <t>15</t>
+      <c r="Z227" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="AB227" s="2" t="inlineStr">
@@ -34476,7 +34471,7 @@
       </c>
       <c r="AO227" t="inlineStr">
         <is>
-          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet; term_years:collaborator-sheet</t>
+          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -35124,9 +35119,9 @@
           <t>100% at 80% AMI</t>
         </is>
       </c>
-      <c r="Z232" t="inlineStr">
-        <is>
-          <t>10</t>
+      <c r="Z232" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
         </is>
       </c>
       <c r="AB232" s="2" t="inlineStr">
@@ -35166,7 +35161,7 @@
       </c>
       <c r="AO232" t="inlineStr">
         <is>
-          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet; term_years:collaborator-sheet</t>
+          <t>investor_1:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -35520,16 +35515,16 @@
           <t>Integrity Housing</t>
         </is>
       </c>
-      <c r="W235" t="inlineStr">
+      <c r="W235" s="2" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="X235" t="inlineStr">
         <is>
           <t>108</t>
         </is>
       </c>
-      <c r="X235" t="inlineStr">
-        <is>
-          <t>108</t>
-        </is>
-      </c>
       <c r="Y235" s="2" t="inlineStr">
         <is>
           <t>80%</t>
@@ -35542,12 +35537,12 @@
       </c>
       <c r="AB235" s="2" t="inlineStr">
         <is>
-          <t>64800</t>
+          <t>81600</t>
         </is>
       </c>
       <c r="AC235" s="2" t="inlineStr">
         <is>
-          <t>16200</t>
+          <t>20400</t>
         </is>
       </c>
       <c r="AD235" s="2" t="inlineStr">
@@ -35582,7 +35577,7 @@
       </c>
       <c r="AO235" t="inlineStr">
         <is>
-          <t>new_build:collaborator-sheet; investor_1:collaborator-sheet; total_units:collaborator-sheet; restricted_units:collaborator-sheet</t>
+          <t>new_build:collaborator-sheet; investor_1:collaborator-sheet; restricted_units:collaborator-sheet</t>
         </is>
       </c>
     </row>
@@ -79943,10 +79938,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
   </cols>
@@ -80498,1086 +80493,610 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-possible-match</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Oak Road' -&gt; manual 'Eleos Ventures, LLC'</t>
+          <t>entity '381 Turk Street Associates, a California' ~ SCC LP '421 Turk Street Associates, L.P.' (#3326, San Francisco, score 92)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-possible-match</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>33</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Ethos Real Estate' -&gt; manual 'Vistria Group'</t>
+          <t>entity 'BIF NON OZ 7524 S HOOVER ST, LP' ~ SCC LP 'BIF NON OZ 7518 S Hoover St, LP' (#14953, Los Angeles, score 93)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-possible-match</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>total_units: generated '144' -&gt; manual '145'</t>
+          <t>entity 'BIF NON OZ 4228 WESTERN AVE, LP' ~ SCC LP 'BIF NON OZ 4209 Western Ave, LP' (#14952, Los Angeles, score 93)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-manual-unmatched</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>48</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>total_units: generated '29' -&gt; manual '196'</t>
+          <t>manual scc_filed=True but no BOE certificate matches entity 'Hillsdale Property LP'; closest: 'Hillsdale Property San Mateo, LP' (#15018, San Mateo, score 78)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-manual-unmatched</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>58</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Vintage Housing Holdings, LLC' -&gt; manual 'Kennedy Wilson'</t>
+          <t>manual scc_filed=True but no BOE certificate matches entity 'Post Chaparral, LP, a Delaware limited p'; closest: 'Post Palmdale Chaparral, LP' (#15197, Los Angeles, score 76)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-possible-match</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>122</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>nonprofit_partner: generated 'Pacific Housing, Inc.' -&gt; manual 'Hearthstone Housing Foundation'</t>
+          <t>entity '861 Fedora LLLP' ~ SCC LP '836 Fedora L.P.' (#1594, Los Angeles, score 90)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-possible-match</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>165</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>total_units: generated '32' -&gt; manual '31'</t>
+          <t>entity '861 Fedora LLLP' ~ SCC LP '836 Fedora L.P.' (#1594, Los Angeles, score 90)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-superseded-only</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>132</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>city_cut: generated '4650.0' -&gt; manual '4500'</t>
+          <t>operative entity 'PS 7518 Hoover St, LP' has no SCC, but the property's superseded grant 10 ('BIF NON OZ 7518 S Hoover St, LP, a Delaw') holds SCC 14953 (2024-11-25) — new sponsor's LP must file its own</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>scc-superseded-only</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>134</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>total_units: generated '30' -&gt; manual '29'</t>
+          <t>operative entity 'PS 10705 Avalon Blvd, LP' has no SCC, but the property's superseded grant 303 ('BIF NON OZ 10705 Avalon Blvd, LP, a Cali') holds SCC 14852 (2024-10-03) — new sponsor's LP must file its own</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>76</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Belveron Partners' -&gt; manual 'Sack Capital Partners'</t>
+          <t>AIN 5036031006 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>99</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>total_units: generated '69' -&gt; manual '68'</t>
+          <t>AIN 4262018026 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>132</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>total_units: generated '42' -&gt; manual '41'</t>
+          <t>AIN 6020022027 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>137</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
+          <t>AIN 2125017014 (Los Angeles) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>158</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>entity: generated 'A limited partnership to be formed by Kairos Investment Management and Pacific Housing' -&gt; manual 'TBD LP'</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>171</t>
+          <t>196</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>city_cut: generated '15900.0' -&gt; manual '6300'</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>201</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>total_units: generated '42' -&gt; manual '41'</t>
+          <t>AIN (none) (Santa Barbara): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>206</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>city_cut: generated '5550.0' -&gt; manual '5500'</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>207</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>total_units: generated '50' -&gt; manual '49'</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>208</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>county: generated 'San Diego' -&gt; manual 'Los Angeles'</t>
+          <t>AIN (none) (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>215</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>investor_1: generated 'Zenith Property Group LLC' -&gt; manual 'Red Stone Equity Partners'</t>
+          <t>AIN 5539028040 (Los Angeles): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-no-values</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>226</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>term_years: generated '35' -&gt; manual '15'</t>
+          <t>AIN (none) (Contra Costa): no roll values from any source</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>term_years: generated '55' -&gt; manual '10'</t>
+          <t>AIN 128101150 (Solano) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>term_years: generated '15' -&gt; manual '10'</t>
+          <t>AIN 128101050 (Solano) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>fetch-fallback</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>term_years: generated '10' -&gt; manual '15'</t>
+          <t>AIN 128105060 (Solano) has no current roll data; using manual value</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>217</t>
+          <t>121</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>total_units: generated '35' -&gt; manual '34'</t>
+          <t>AIN 5518013024 (Alexandria II Apartments) also assigned under operative grant 162; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>122</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>term_years: generated '55' -&gt; manual '10'</t>
+          <t>AIN 5094017020 (Fedora Apartments) also assigned under operative grant 165; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>123</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>total_units: generated '136' -&gt; manual '108'</t>
+          <t>AIN 5518020021 (Kenmore II Apartments) also assigned under operative grant 168; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>override-conflict</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>124</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>term_years: generated '30' -&gt; manual '55'</t>
+          <t>AIN 5094023025 (Kenmore III Apartments) also assigned under operative grant 169; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>scc-possible-match</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>125</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>entity '381 Turk Street Associates, a California' ~ SCC LP '421 Turk Street Associates, L.P.' (#3326, San Francisco, score 92)</t>
+          <t>AIN 5503024012 (Kingsley Apartments) also assigned under operative grant 170; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>scc-possible-match</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>126</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>entity 'BIF NON OZ 7524 S HOOVER ST, LP' ~ SCC LP 'BIF NON OZ 7518 S Hoover St, LP' (#14953, Los Angeles, score 93)</t>
+          <t>AIN 5094005005 (Mariposa I Apartments) also assigned under operative grant 173; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>scc-possible-match</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>127</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>entity 'BIF NON OZ 4228 WESTERN AVE, LP' ~ SCC LP 'BIF NON OZ 4209 Western Ave, LP' (#14952, Los Angeles, score 93)</t>
+          <t>AIN 5094006003 (Mariposa III Apartments) also assigned under operative grant 174; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>scc-manual-unmatched</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>128</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>manual scc_filed=True but no BOE certificate matches entity 'Hillsdale Property LP'; closest: 'Hillsdale Property San Mateo, LP' (#15018, San Mateo, score 78)</t>
+          <t>AIN 5502019004 (Mariposa IV Apartments) also assigned under operative grant 175; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>scc-manual-unmatched</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>129</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>manual scc_filed=True but no BOE certificate matches entity 'Post Chaparral, LP, a Delaware limited p'; closest: 'Post Palmdale Chaparral, LP' (#15197, Los Angeles, score 76)</t>
+          <t>AIN 5517005016 (Oxford II Apartments) also assigned under operative grant 177; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>scc-possible-match</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>130</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>entity '861 Fedora LLLP' ~ SCC LP '836 Fedora L.P.' (#1594, Los Angeles, score 90)</t>
+          <t>AIN 5080006008 (Western Apartments) also assigned under operative grant 179; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>scc-possible-match</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>165</t>
+          <t>152</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>entity '861 Fedora LLLP' ~ SCC LP '836 Fedora L.P.' (#1594, Los Angeles, score 90)</t>
+          <t>AIN 7157012023 (The Hive at Ackerfield Apartments) also assigned under operative grant 181; this row marked legacy_redundant so sums count it once</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>scc-superseded-only</t>
+          <t>parcel-dedup</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>135</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
-        <is>
-          <t>operative entity 'PS 7518 Hoover St, LP' has no SCC, but the property's superseded grant 10 ('BIF NON OZ 7518 S Hoover St, LP, a Delaw') holds SCC 14953 (2024-11-25) — new sponsor's LP must file its own</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>scc-superseded-only</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>134</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>operative entity 'PS 10705 Avalon Blvd, LP' has no SCC, but the property's superseded grant 303 ('BIF NON OZ 10705 Avalon Blvd, LP, a Cali') holds SCC 14852 (2024-10-03) — new sponsor's LP must file its own</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>76</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>AIN 5036031006 (Los Angeles) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>99</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>AIN 4262018026 (Los Angeles) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>132</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>AIN 6020022027 (Los Angeles) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>137</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>AIN 2125017014 (Los Angeles) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>158</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>196</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>201</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>AIN (none) (Santa Barbara): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>206</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>207</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>208</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>AIN (none) (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>215</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>AIN 5539028040 (Los Angeles): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>parcel-no-values</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>226</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>AIN (none) (Contra Costa): no roll values from any source</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>AIN 128101150 (Solano) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>AIN 128101050 (Solano) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>fetch-fallback</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>AIN 128105060 (Solano) has no current roll data; using manual value</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>121</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>AIN 5518013024 (Alexandria II Apartments) also assigned under operative grant 162; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>122</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>AIN 5094017020 (Fedora Apartments) also assigned under operative grant 165; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>123</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>AIN 5518020021 (Kenmore II Apartments) also assigned under operative grant 168; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>124</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>AIN 5094023025 (Kenmore III Apartments) also assigned under operative grant 169; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>125</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>AIN 5503024012 (Kingsley Apartments) also assigned under operative grant 170; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>126</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>AIN 5094005005 (Mariposa I Apartments) also assigned under operative grant 173; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>127</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>AIN 5094006003 (Mariposa III Apartments) also assigned under operative grant 174; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>128</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>AIN 5502019004 (Mariposa IV Apartments) also assigned under operative grant 175; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>129</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>AIN 5517005016 (Oxford II Apartments) also assigned under operative grant 177; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>130</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>AIN 5080006008 (Western Apartments) also assigned under operative grant 179; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>152</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>AIN 7157012023 (The Hive at Ackerfield Apartments) also assigned under operative grant 181; this row marked legacy_redundant so sums count it once</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>parcel-dedup</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>135</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
         <is>
           <t>AIN 5518026004 (236 Berendo Apartments) also assigned under operative grant 220; this row marked legacy_redundant so sums count it once</t>
         </is>

</xml_diff>

<commit_message>
Add reproducible county summary (pivot table) to dataset and workbook
New output/dataset/county_summary.csv + "County summary" workbook tab,
rebuilt on every run: one row per county over live operative grants
(excluding dead/stale) with project count, SCC-confirmed count, JPA
closing/annual fee sums, confirmed exemption from county rolls (live
parcels keyed by operative_project_id) and its 1% tax reduction, plus
total/restricted unit and city-cut sums; TOTAL row last. All cells
tinted as automated. Current totals: 184 live operative projects, 64
SCC-confirmed, $801.6M confirmed exemptions -> $8.02M/yr tax reduction.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grants" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parcels" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA findings" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="County summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA findings" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -81349,6 +81350,1020 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>county</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>operative_projects</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>with_scc_filed</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>jpa_closing_fees</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>jpa_annual_fees</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>confirmed_exemption</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>confirmed_tax_reduction</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>total_units</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>restricted_units</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>city_cut</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Alameda</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>626400</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>156600</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>83017361</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>830174</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>1044</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>979</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>102000</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Contra Costa</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>896400</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>224300</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>46831134</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>468311</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>1494</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>1303</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>142350</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Fresno</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>166800</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>41700</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>278</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>278</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>41700</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>6121000</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>1562450</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>348365149</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>3483651</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>10198</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>8629</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>1111775</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Marin</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>59400</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>14850</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Napa</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>88800</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>22200</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>148</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>148</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>22200</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>1071600</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>267900</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>204152723</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2041527</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>1837</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>1413</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>187250</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sacramento</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>676800</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>169200</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>23179668</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>231797</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>1128</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>1017</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>109800</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>San Bernardino</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>42600</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>10650</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>4156500</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>41565</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>10650</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>1519300</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>382325</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>49157189</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>491572</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>2653</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>2202</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>240716</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>197400</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>49350</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>329</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>236</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>35400</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>San Mateo</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>847800</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>211950</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>28000</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>280</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>1413</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>1147</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>142275</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Santa Barbara</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>276000</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>69000</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>460</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>460</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>57000</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Santa Clara</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>1538400</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>384600</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>35568556</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>355686</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>2739</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>2065</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>210600</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Santa Cruz</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>90000</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>22500</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>22500</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Solano</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>180600</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>45150</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>7127607</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>71276</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>301</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>28500</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Sonoma</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>22200</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>5550</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>5550</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>14421500</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>3640275</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>801583887</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>8015839</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>24379</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>20423</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>2470266</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -82552,7 +83567,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
County summary: estimated_exemption / estimated_tax_reduction columns
Projection for properties not yet on the roll: assessed value x
restricted ratio x k, where k is the median of that ratio over
properties WITH confirmed exemptions, re-fitted each build (currently
0.980 over 36 confirmed). Median, not OLS — the tails are first-year
partial filings (Hillsdale's $28K on $252M) and renumbered-parcel value
gaps (820 MacArthur's exemption exceeds its assessed value). Estimates
are capped at assessed value; restricted ratio falls back to
restricted_pct when unit counts are missing; confirmed exemptions pass
through unchanged. Headline: $3.88B estimated exemptions -> $38.8M/yr
projected tax reduction vs $801.6M/$8.0M confirmed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -81350,7 +81350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -81363,6 +81363,8 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -81403,15 +81405,25 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>estimated_exemption</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>estimated_tax_reduction</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>total_units</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>restricted_units</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>city_cut</t>
         </is>
@@ -81455,15 +81467,25 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
+          <t>260499619</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>2604996</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>1044</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>979</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>102000</t>
         </is>
@@ -81507,15 +81529,25 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
+          <t>318881999</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>3188820</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
           <t>1494</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>1303</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>142350</t>
         </is>
@@ -81559,15 +81591,25 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
+          <t>29735832</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>297358</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
           <t>278</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>278</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>41700</t>
         </is>
@@ -81611,15 +81653,25 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
+          <t>1264768719</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>12647687</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
           <t>10198</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>8629</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>1111775</t>
         </is>
@@ -81663,15 +81715,25 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
+          <t>33215308</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>332153</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
           <t>99</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>99</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -81715,15 +81777,25 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
+          <t>45778059</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>457781</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
           <t>148</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>148</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>22200</t>
         </is>
@@ -81767,15 +81839,25 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
+          <t>420796578</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>4207966</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
           <t>1837</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>1413</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>187250</t>
         </is>
@@ -81819,15 +81901,25 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
+          <t>143948867</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>1439489</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
           <t>1128</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>1017</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>109800</t>
         </is>
@@ -81871,15 +81963,25 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
+          <t>4156500</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>41565</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
           <t>71</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>70</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>10650</t>
         </is>
@@ -81923,15 +82025,25 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
+          <t>403625076</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>4036251</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
           <t>2653</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2202</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>240716</t>
         </is>
@@ -81975,15 +82087,25 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
+          <t>113957436</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>1139574</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
           <t>329</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>236</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>35400</t>
         </is>
@@ -82027,15 +82149,25 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
+          <t>138012042</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>1380120</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
           <t>1413</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>1147</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>142275</t>
         </is>
@@ -82079,15 +82211,25 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
+          <t>22282532</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>222825</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
           <t>460</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>460</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>57000</t>
         </is>
@@ -82131,15 +82273,25 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
+          <t>624773704</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>6247737</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
           <t>2739</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>2065</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>210600</t>
         </is>
@@ -82183,15 +82335,25 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
+          <t>9584501</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>95845</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
           <t>150</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>150</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>22500</t>
         </is>
@@ -82235,15 +82397,25 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
+          <t>35835370</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>358354</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
           <t>301</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>190</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>28500</t>
         </is>
@@ -82287,15 +82459,25 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
+          <t>9941350</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>99413</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
           <t>37</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>5550</t>
         </is>
@@ -82339,15 +82521,25 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
+          <t>3879793492</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>38797935</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
           <t>24379</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>20423</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>2470266</t>
         </is>

</xml_diff>

<commit_message>
Estimator: stated 100% restriction beats the unit ratio (manager's unit is exempt)
Research finding: under RTC 214(g) the exemption prorates by units serving
lower-income households over total residential units, BUT the manager's
unit is itself exempt — 214(g)(3)(C) classes "any manager's units" as
exempt related facilities, and BOE Assessors' Handbook 267 states "A
manager's unit is exempt as incidental to and reasonably necessary for
the accomplishment of the exempt purposes, even if the manager's income
exceeds the prescribed low-income limits" (p.91, the 214(g) section;
p.93 shows the sibling 214(f) formula explicitly counting the manager's
unit in the numerator). So a 41-restricted/42-unit property is 100%
exempt, and the staff reports' "Percent of Restricted Rental Units in
the Project: 100%" header is the correct expectation. _ratio now returns
1.0 whenever restricted_pct is 100, before consulting unit counts.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/dataset/review.xlsx
+++ b/output/dataset/review.xlsx
@@ -81653,12 +81653,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>1264768719</t>
+          <t>1266439164</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>12647687</t>
+          <t>12664392</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -82025,12 +82025,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>403625076</t>
+          <t>404140279</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>4036251</t>
+          <t>4041403</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -82521,12 +82521,12 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>3879793492</t>
+          <t>3881979140</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>38797935</t>
+          <t>38819791</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">

</xml_diff>